<commit_message>
data: update tax decisions 2026-07-26
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="AJ27" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -9394,7 +9394,7 @@
       </c>
       <c r="AJ11" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -10429,7 +10429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10796,8 +10796,53 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-26T16:17:41+08:00</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23 至 2026-07-26</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M7"/>
+  <autoFilter ref="A1:M8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-07-27
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日运行日志" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ27"/>
+  <dimension ref="A1:AJ29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -785,7 +785,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1293,7 +1293,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2653,7 +2653,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2771,7 +2771,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2913,7 +2913,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3171,7 +3171,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3441,7 +3441,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3713,7 +3713,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3965,7 +3965,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4005,20 +4005,288 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>DOC-bed9330343ed06af</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>税务处理决定书</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
+      <c r="S28" s="3" t="n"/>
+      <c r="T28" s="3" t="n"/>
+      <c r="U28" s="3" t="n"/>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W28" s="4" t="n"/>
+      <c r="X28" s="4" t="n"/>
+      <c r="Y28" s="4" t="n"/>
+      <c r="Z28" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA28" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD28" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE28" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF28" s="2" t="inlineStr"/>
+      <c r="AG28" s="2" t="inlineStr"/>
+      <c r="AH28" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI28" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ28" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="n"/>
+      <c r="S29" s="3" t="n"/>
+      <c r="T29" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U29" s="3" t="n"/>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W29" s="4" t="n"/>
+      <c r="X29" s="4" t="n"/>
+      <c r="Y29" s="4" t="n"/>
+      <c r="Z29" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA29" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD29" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE29" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF29" s="2" t="inlineStr"/>
+      <c r="AG29" s="2" t="inlineStr"/>
+      <c r="AH29" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI29" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ29" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ27"/>
-  <conditionalFormatting sqref="AD2:AD27">
+  <autoFilter ref="A1:AJ29"/>
+  <conditionalFormatting sqref="AD2:AD29">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI27">
+  <conditionalFormatting sqref="AI2:AI29">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4059,6 +4327,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF25" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE27" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE28" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -4071,7 +4341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ13"/>
+  <dimension ref="A1:AJ15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4386,7 +4656,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -4520,7 +4790,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -4652,7 +4922,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -4780,7 +5050,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -4918,7 +5188,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -5054,7 +5324,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -5186,7 +5456,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -5324,7 +5594,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -5466,7 +5736,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -5596,7 +5866,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -5724,7 +5994,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -5848,7 +6118,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -5888,20 +6158,288 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>DOC-bed9330343ed06af</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>税务处理决定书</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
+      <c r="S14" s="3" t="n"/>
+      <c r="T14" s="3" t="n"/>
+      <c r="U14" s="3" t="n"/>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W14" s="4" t="n"/>
+      <c r="X14" s="4" t="n"/>
+      <c r="Y14" s="4" t="n"/>
+      <c r="Z14" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA14" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD14" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE14" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr"/>
+      <c r="AH14" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI14" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ14" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="n"/>
+      <c r="S15" s="3" t="n"/>
+      <c r="T15" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U15" s="3" t="n"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W15" s="4" t="n"/>
+      <c r="X15" s="4" t="n"/>
+      <c r="Y15" s="4" t="n"/>
+      <c r="Z15" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA15" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE15" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AH15" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI15" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ13"/>
-  <conditionalFormatting sqref="AD2:AD13">
+  <autoFilter ref="A1:AJ15"/>
+  <conditionalFormatting sqref="AD2:AD15">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI13">
+  <conditionalFormatting sqref="AI2:AI15">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5922,6 +6460,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF11" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE13" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE15" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -6239,7 +6779,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -6357,7 +6897,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -6479,7 +7019,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -6605,7 +7145,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -6731,7 +7271,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -6849,7 +7389,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -6971,7 +7511,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -7093,7 +7633,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -7215,7 +7755,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -7337,7 +7877,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -7459,7 +7999,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -7581,7 +8121,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -7699,7 +8239,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -7821,7 +8361,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -7915,7 +8455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ11"/>
+  <dimension ref="A1:AJ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8216,7 +8756,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -8342,7 +8882,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -8460,7 +9000,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -8582,7 +9122,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -8704,7 +9244,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -8822,7 +9362,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8964,7 +9504,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -9106,7 +9646,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -9234,7 +9774,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -9358,7 +9898,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -9398,20 +9938,288 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>DOC-bed9330343ed06af</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>税务处理决定书</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
+      <c r="S12" s="3" t="n"/>
+      <c r="T12" s="3" t="n"/>
+      <c r="U12" s="3" t="n"/>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W12" s="4" t="n"/>
+      <c r="X12" s="4" t="n"/>
+      <c r="Y12" s="4" t="n"/>
+      <c r="Z12" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA12" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD12" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE12" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="inlineStr"/>
+      <c r="AH12" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI12" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ12" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="n"/>
+      <c r="T13" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U13" s="3" t="n"/>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W13" s="4" t="n"/>
+      <c r="X13" s="4" t="n"/>
+      <c r="Y13" s="4" t="n"/>
+      <c r="Z13" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA13" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD13" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE13" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF13" s="2" t="inlineStr"/>
+      <c r="AG13" s="2" t="inlineStr"/>
+      <c r="AH13" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI13" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ13" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ11"/>
-  <conditionalFormatting sqref="AD2:AD11">
+  <autoFilter ref="A1:AJ13"/>
+  <conditionalFormatting sqref="AD2:AD13">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI11">
+  <conditionalFormatting sqref="AI2:AI13">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9429,6 +10237,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF9" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE10" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE13" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -9742,7 +10552,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9868,7 +10678,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -9986,7 +10796,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10108,7 +10918,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10230,7 +11040,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10348,7 +11158,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10429,7 +11239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10886,8 +11696,57 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27T15:38:15+08:00</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 至 2026-07-27</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>已完成候选发现、逐条访问核验、去重、关联和历史数据增量写入。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M9"/>
+  <autoFilter ref="A1:M10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-07-28
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1293,7 +1293,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2653,7 +2653,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2771,7 +2771,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2913,7 +2913,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3171,7 +3171,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3441,7 +3441,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3713,7 +3713,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3965,7 +3965,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4099,7 +4099,7 @@
         <v>46230</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="AJ28" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4233,7 @@
         <v>46230</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="AJ29" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -4790,7 +4790,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -4922,7 +4922,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -5050,7 +5050,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -5324,7 +5324,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -5594,7 +5594,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -5736,7 +5736,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -6118,7 +6118,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -6252,7 +6252,7 @@
         <v>46230</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
         <v>46230</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -6422,7 +6422,7 @@
       </c>
       <c r="AJ15" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6779,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -6897,7 +6897,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7145,7 +7145,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7389,7 +7389,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -7511,7 +7511,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -7633,7 +7633,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -7755,7 +7755,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -7877,7 +7877,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8239,7 +8239,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -8361,7 +8361,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -8756,7 +8756,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -8882,7 +8882,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -9000,7 +9000,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -9122,7 +9122,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -9244,7 +9244,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -9362,7 +9362,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -9504,7 +9504,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -9646,7 +9646,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -9774,7 +9774,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -10032,7 +10032,7 @@
         <v>46230</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -10068,7 +10068,7 @@
       </c>
       <c r="AJ12" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -10166,7 +10166,7 @@
         <v>46230</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10552,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -10678,7 +10678,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10796,7 +10796,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10918,7 +10918,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11040,7 +11040,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11158,7 +11158,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11239,7 +11239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11745,8 +11745,53 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28T14:31:21+08:00</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25 至 2026-07-28</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M10"/>
+  <autoFilter ref="A1:M11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-07-29
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1293,7 +1293,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2653,7 +2653,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2771,7 +2771,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2913,7 +2913,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3171,7 +3171,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3441,7 +3441,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3713,7 +3713,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3965,7 +3965,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4099,7 +4099,7 @@
         <v>46230</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4233,7 +4233,7 @@
         <v>46230</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4656,7 +4656,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -4790,7 +4790,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -4922,7 +4922,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -5050,7 +5050,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -5324,7 +5324,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -5594,7 +5594,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -5736,7 +5736,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -6118,7 +6118,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -6252,7 +6252,7 @@
         <v>46230</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -6386,7 +6386,7 @@
         <v>46230</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -6779,7 +6779,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -6897,7 +6897,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7145,7 +7145,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7271,7 +7271,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7389,7 +7389,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -7511,7 +7511,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -7633,7 +7633,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -7755,7 +7755,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -7877,7 +7877,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8239,7 +8239,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -8361,7 +8361,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -8756,7 +8756,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -8882,7 +8882,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -9000,7 +9000,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -9122,7 +9122,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -9244,7 +9244,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -9362,7 +9362,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -9504,7 +9504,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -9646,7 +9646,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -9774,7 +9774,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -10032,7 +10032,7 @@
         <v>46230</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -10166,7 +10166,7 @@
         <v>46230</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -10552,7 +10552,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -10678,7 +10678,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10796,7 +10796,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10918,7 +10918,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11040,7 +11040,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11158,7 +11158,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11239,7 +11239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11790,8 +11790,53 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29T14:36:32+08:00</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-26 至 2026-07-29</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M11"/>
+  <autoFilter ref="A1:M12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-01
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -791,7 +791,7 @@
         <v>46233</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
         <v>46234</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“北市税稽处〔2026〕6号”,新值“北市税稽处〔2026〕13号”未静默覆盖。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“北市税稽处〔2026〕6号”,新值“北市税稽处〔2026〕13号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2185,7 +2185,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2429,7 +2429,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2795,7 +2795,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2917,7 +2917,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3177,7 +3177,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3299,7 +3299,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3435,7 +3435,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3567,7 +3567,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3705,7 +3705,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3847,7 +3847,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3977,7 +3977,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4229,7 +4229,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4363,7 +4363,7 @@
         <v>46230</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4497,7 +4497,7 @@
         <v>46230</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4918,7 +4918,7 @@
         <v>46233</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -5054,7 +5054,7 @@
         <v>46234</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“北市税稽处〔2026〕6号”,新值“北市税稽处〔2026〕13号”未静默覆盖。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“北市税稽处〔2026〕6号”,新值“北市税稽处〔2026〕13号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -5320,7 +5320,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -5452,7 +5452,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -5580,7 +5580,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -5718,7 +5718,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -5854,7 +5854,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -5986,7 +5986,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -6124,7 +6124,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -6266,7 +6266,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -6396,7 +6396,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -6524,7 +6524,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -6782,7 +6782,7 @@
         <v>46230</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -6916,7 +6916,7 @@
         <v>46230</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -7311,7 +7311,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7429,7 +7429,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7677,7 +7677,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7803,7 +7803,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7921,7 +7921,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8043,7 +8043,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8165,7 +8165,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8287,7 +8287,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8409,7 +8409,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8531,7 +8531,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8653,7 +8653,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8771,7 +8771,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -8893,7 +8893,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9288,7 +9288,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9414,7 +9414,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -9532,7 +9532,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -9654,7 +9654,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -9776,7 +9776,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -9894,7 +9894,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10036,7 +10036,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10178,7 +10178,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10306,7 +10306,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -10430,7 +10430,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -10564,7 +10564,7 @@
         <v>46230</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -10698,7 +10698,7 @@
         <v>46230</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11084,7 +11084,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11210,7 +11210,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11328,7 +11328,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11450,7 +11450,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11572,7 +11572,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11690,7 +11690,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11771,7 +11771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12465,8 +12465,53 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01T14:34:47+08:00</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 至 2026-08-01</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M14"/>
+  <autoFilter ref="A1:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-03
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46236</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -823,7 +823,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -907,7 +911,7 @@
         <v>46236</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -945,7 +949,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1035,7 +1043,7 @@
         <v>46233</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1171,7 +1179,7 @@
         <v>46234</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1293,7 +1301,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1411,7 +1419,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1543,7 +1551,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1685,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1801,7 +1809,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1927,7 +1935,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2061,7 +2069,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2185,7 +2193,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2311,7 +2319,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2429,7 +2437,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2559,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2673,7 +2681,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2795,7 +2803,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2917,7 +2925,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3039,7 +3047,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3161,7 +3169,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3279,7 +3287,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3421,7 +3429,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3543,7 +3551,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3679,7 +3687,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3811,7 +3819,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3949,7 +3957,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4091,7 +4099,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4221,7 +4229,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4349,7 +4357,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4473,7 +4481,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4607,7 +4615,7 @@
         <v>46230</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4741,7 +4749,7 @@
         <v>46230</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -5166,7 +5174,7 @@
         <v>46233</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -5302,7 +5310,7 @@
         <v>46234</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -5434,7 +5442,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -5568,7 +5576,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -5700,7 +5708,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -5828,7 +5836,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -5966,7 +5974,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -6102,7 +6110,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -6234,7 +6242,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -6372,7 +6380,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -6514,7 +6522,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -6644,7 +6652,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -6772,7 +6780,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -6896,7 +6904,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -7030,7 +7038,7 @@
         <v>46230</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -7164,7 +7172,7 @@
         <v>46230</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -7559,7 +7567,7 @@
         <v>46236</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7597,7 +7605,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -7681,7 +7693,7 @@
         <v>46236</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7719,7 +7731,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -7803,7 +7819,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7921,7 +7937,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -8043,7 +8059,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -8169,7 +8185,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8295,7 +8311,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8413,7 +8429,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8535,7 +8551,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8657,7 +8673,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8779,7 +8795,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8901,7 +8917,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -9023,7 +9039,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9145,7 +9161,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9263,7 +9279,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9385,7 +9401,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9784,7 +9800,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9910,7 +9926,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10028,7 +10044,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10150,7 +10166,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10272,7 +10288,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10390,7 +10406,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10532,7 +10548,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10674,7 +10690,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10802,7 +10818,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -10926,7 +10942,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11060,7 +11076,7 @@
         <v>46230</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11194,7 +11210,7 @@
         <v>46230</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11580,7 +11596,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11706,7 +11722,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11824,7 +11840,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11946,7 +11962,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -12068,7 +12084,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -12186,7 +12202,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -12267,7 +12283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13055,8 +13071,53 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03T15:33:31+08:00</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 至 2026-08-03</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M16"/>
+  <autoFilter ref="A1:M17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-04
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46236</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46236</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         <v>46233</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         <v>46234</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1685,7 +1685,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1809,7 +1809,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2193,7 +2193,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2803,7 +2803,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3047,7 +3047,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3287,7 +3287,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3429,7 +3429,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3551,7 +3551,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3819,7 +3819,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3957,7 +3957,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4099,7 +4099,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4229,7 +4229,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4357,7 +4357,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4481,7 +4481,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4615,7 +4615,7 @@
         <v>46230</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4749,7 +4749,7 @@
         <v>46230</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -5174,7 +5174,7 @@
         <v>46233</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -5310,7 +5310,7 @@
         <v>46234</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -5442,7 +5442,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -5576,7 +5576,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -5708,7 +5708,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -5974,7 +5974,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -6110,7 +6110,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -6242,7 +6242,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -6380,7 +6380,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -6522,7 +6522,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -6652,7 +6652,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -6904,7 +6904,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -7038,7 +7038,7 @@
         <v>46230</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -7172,7 +7172,7 @@
         <v>46230</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -7567,7 +7567,7 @@
         <v>46236</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7693,7 +7693,7 @@
         <v>46236</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7819,7 +7819,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7937,7 +7937,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -8059,7 +8059,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -8185,7 +8185,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8311,7 +8311,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8429,7 +8429,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8551,7 +8551,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8795,7 +8795,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8917,7 +8917,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -9039,7 +9039,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9161,7 +9161,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9279,7 +9279,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9401,7 +9401,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9800,7 +9800,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9926,7 +9926,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10044,7 +10044,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10166,7 +10166,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10288,7 +10288,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10406,7 +10406,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10548,7 +10548,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10690,7 +10690,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10818,7 +10818,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -10942,7 +10942,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11076,7 +11076,7 @@
         <v>46230</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11210,7 +11210,7 @@
         <v>46230</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         <v>46229</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11722,7 +11722,7 @@
         <v>46229</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11840,7 +11840,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11962,7 +11962,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -12084,7 +12084,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -12202,7 +12202,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -12283,7 +12283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13116,8 +13116,53 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T14:32:07+08:00</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01 至 2026-08-04</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M17"/>
+  <autoFilter ref="A1:M18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add resilient official document links
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE14" s="5" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="AI14" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ14" s="2" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE21" s="5" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="AI21" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ21" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE24" s="5" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AI24" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ24" s="2" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE25" s="5" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="AI25" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ25" s="2" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE26" s="5" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="AI26" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ26" s="2" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="AJ34" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。 字段“主要违法事实”存在冲突:保留原值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”,新值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="AJ35" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="AJ37" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -5403,7 +5403,7 @@
       </c>
       <c r="AJ38" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE10" s="5" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="AI10" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ10" s="2" t="inlineStr">
@@ -7643,7 +7643,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -7713,7 +7713,7 @@
       </c>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。 字段“主要违法事实”存在冲突:保留原值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”,新值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -7855,7 +7855,7 @@
       </c>
       <c r="AJ15" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -8109,7 +8109,7 @@
       </c>
       <c r="AJ17" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="AJ18" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE9" s="5" t="inlineStr">
@@ -9752,7 +9752,7 @@
       </c>
       <c r="AI9" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ9" s="2" t="inlineStr">
@@ -10471,7 +10471,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE15" s="5" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="AI15" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ15" s="2" t="inlineStr">
@@ -10593,7 +10593,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE16" s="5" t="inlineStr">
@@ -10610,7 +10610,7 @@
       </c>
       <c r="AI16" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ16" s="2" t="inlineStr">
@@ -10715,7 +10715,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE17" s="5" t="inlineStr">
@@ -10732,7 +10732,7 @@
       </c>
       <c r="AI17" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ17" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ15"/>
+  <dimension ref="A1:AJ10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11750,66 +11750,66 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CASE-365e8a924cf64611</t>
+          <t>CASE-393a878d93a22709</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>DOC-4d14eba16f9aa8a0</t>
+          <t>DOC-cda8cba853896b18</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>广东省</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>贵阳市</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+          <t>广州市</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>番禺区</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
+          <t>国家税务总局广州市番禺区税务局</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>贵州博泰工贸有限公司</t>
+          <t>广州赞荣服装有限公司</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>91520115587255589F</t>
+          <t>91440113MA59AJFJ1J</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>筑税三稽处〔2026〕38号</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽处〔2026〕38号</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="3" t="n"/>
@@ -11819,7 +11819,7 @@
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="4" t="n"/>
       <c r="X4" s="4" t="n">
-        <v>46224</v>
+        <v>46091</v>
       </c>
       <c r="Y4" s="4" t="n"/>
       <c r="Z4" s="4" t="n">
@@ -11848,36 +11848,40 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AF4" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局关于送达税务处理决定书、税务行政处罚决定书的公告</t>
+          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
         </is>
       </c>
       <c r="AI4" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>内容不匹配</t>
         </is>
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CASE-a62e569c195adc3c</t>
+          <t>CASE-f78ec1a594442165</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>DOC-b1dda915d4e6117d</t>
+          <t>DOC-fbbe4a664b14f54b</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -11887,28 +11891,28 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>遵义市</t>
+          <t>安顺市</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局遵义市税务局第一稽查局</t>
+          <t>国家税务总局安顺市税务局</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局遵义市税务局第一稽查局</t>
+          <t>国家税务总局安顺市税务局稽查局</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>贵州服格定商贸有限公司</t>
+          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>91520302MABUEHN034</t>
+          <t>91520423MA6DLH799Q</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -11919,33 +11923,45 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>遵税一稽处〔2026〕30号</t>
+          <t>安市税稽处〔2026〕1号</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>遵税一稽处〔2026〕30号</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr"/>
+          <t>安市税稽处〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>安市税稽罚〔2026〕1号</t>
+        </is>
+      </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>情况进行了检查,违法事实及处理决定如下: 2023年度开具增值税电子普通发票合计金额36,788.18元,税额905.82元,价税37,694.00元,未申报纳税,并且你公司从2023年起所有税种没有进行纳税申报。</t>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>增值税</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="n"/>
+          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>64884.41</v>
+      </c>
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="3" t="n"/>
-      <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="4" t="n"/>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>45898</v>
+      </c>
       <c r="X5" s="4" t="n">
-        <v>46185</v>
+        <v>46043</v>
       </c>
       <c r="Y5" s="4" t="n"/>
       <c r="Z5" s="4" t="n">
@@ -11974,36 +11990,40 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AF5" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局遵义市税务局第一稽查局税务处理决定书(遵税一稽处〔2026〕30 号)</t>
+          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI5" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ5" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。 字段“主要违法事实”存在冲突:保留原值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”,新值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CASE-f8625e66b291a216</t>
+          <t>CASE-f78ec1a594442165</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>DOC-7970511393924720</t>
+          <t>DOC-9a828a6048b54b6c</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -12013,57 +12033,77 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>贵阳市</t>
+          <t>安顺市</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第二稽查局</t>
+          <t>国家税务总局安顺市税务局</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第二稽查局</t>
+          <t>国家税务总局安顺市税务局稽查局</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>贵州翰缤商贸有限公司</t>
+          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>91520114MAAK1C546F</t>
+          <t>91520423MA6DLH799Q</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>筑税二稽处〔2026〕27号</t>
+          <t>安市税稽罚〔2026〕1号</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>筑税二稽处〔2026〕27号</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
+          <t>安市税稽处〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>安市税稽罚〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
       <c r="R6" s="3" t="n"/>
       <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n"/>
+      <c r="T6" s="3" t="n">
+        <v>200000</v>
+      </c>
       <c r="U6" s="3" t="n"/>
-      <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="4" t="n"/>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>45898</v>
+      </c>
       <c r="X6" s="4" t="n">
-        <v>46156</v>
+        <v>46043</v>
       </c>
       <c r="Y6" s="4" t="n"/>
       <c r="Z6" s="4" t="n">
@@ -12074,7 +12114,7 @@
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>仅公告送达/仅文号线索</t>
+          <t>完整文书</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
@@ -12092,69 +12132,69 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AF6" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第二稽查局关于送达《税务处理决定书》的公告</t>
+          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI6" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CASE-0f4867f7b70d12f3</t>
+          <t>CASE-1983d97878508732</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>DOC-6f25d6b79e123d03</t>
+          <t>DOC-f9760895b4f08cc2</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>内蒙古自治区</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>贵阳市</t>
+          <t>二连浩特市</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
+          <t>国家税务总局二连浩特市税务局</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
+          <t>国家税务总局二连浩特市税务局稽查局</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>贵州铂朗物流有限公司</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>91520115MAAK0DB335</t>
-        </is>
-      </c>
+          <t>二连市坤益腾金属有限公司</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -12163,30 +12203,36 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>筑税三稽处〔2026〕17号</t>
+          <t>二税稽处〔2025〕1号</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>筑税三稽处〔2026〕17号</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽罚〔2026〕22号</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
+          <t>二税稽处〔2025〕1号</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>公司院内)涉嫌虚开增值税专用发票的情况进行检查,违法事实 你公司在无真实货物交易的情况下,“让他人为自己”虚开 得有下列虚开发票行为:(一)为他人、为自己开具与实际经营 国人民代表大会常务委员会关于惩治虚开、伪造和非法出售增值 〔1996〕210号)文件:“虚开增值税专用发票的,构成虚开增 值税专用发票罪,具有下列行为之一的,属于虚开增值税专用发 定,你公司上述违法事实中,“让他人为自己”虚开增值税专用 “为他人”虚开增值税专用发票97 份,金额 87,923,181.86 元, 二条第二款的规定虚开发票的,由税务机关没收违法所得; 虚开增值税专用发票行为暂不进行行政处罚,在司法部门作出决 十二条第二款的规定虚开发票的,由税务机关没收违法所得; 依法查处违法行为过程中,发现违法事实涉及的金额、违法事实 的情节、违法事实造成的后果等,根据刑法关于破坏社会主义市 定(二)》(公通字〔2022〕12 号)第五十六条:“〔虚开增值 税专用发票、用于骗取出口退税、抵扣税款发票案(刑法第二百 零五条)〕虚开增值税专用发票或者虚开用于骗取出口退税、抵 扣税款的其他发票,虚开的税款数额在十万元以上或者致使国家 公司虚开增值税专用发票的行为移送公安机关。</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>增值税</t>
+        </is>
+      </c>
       <c r="R7" s="3" t="n"/>
       <c r="S7" s="3" t="n"/>
       <c r="T7" s="3" t="n"/>
       <c r="U7" s="3" t="n"/>
-      <c r="V7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>二条第二款的规定虚开发票的,由税务机关没收违法所得; 十二条第二款的规定虚开发票的,由税务机关没收违法所得;</t>
+        </is>
+      </c>
       <c r="W7" s="4" t="n"/>
-      <c r="X7" s="4" t="n">
-        <v>46122</v>
-      </c>
+      <c r="X7" s="4" t="n"/>
       <c r="Y7" s="4" t="n"/>
       <c r="Z7" s="4" t="n">
         <v>46229</v>
@@ -12196,7 +12242,7 @@
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>仅公告送达/仅文号线索</t>
+          <t>完整文书</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
@@ -12218,97 +12264,99 @@
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局关于送达税务处理决定书税务行政处罚决定书的公告</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="AI7" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CASE-0f4867f7b70d12f3</t>
+          <t>CASE-d4b6986f3f97cd28</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DOC-e8233eb0e06b6e3e</t>
+          <t>DOC-442cf3d9a5280c12</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>内蒙古自治区</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>贵阳市</t>
+          <t>鄂尔多斯市</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
+          <t>第二稽查局</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>贵州铂朗物流有限公司</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>91520115MAAK0DB335</t>
-        </is>
-      </c>
+          <t>廖礼平</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>筑税三稽罚〔2026〕22号</t>
+          <t>鄂税二稽处〔2023〕29号</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>筑税三稽处〔2026〕17号</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽罚〔2026〕22号</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
+          <t>鄂税二稽处〔2023〕29号</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>利煤炭有限责任公司股权涉税问题开展了检查,违法事实及处理</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>个人所得税、印花税</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>15072487.5</v>
+      </c>
+      <c r="S8" s="3" t="n">
+        <v>1046925</v>
+      </c>
       <c r="T8" s="3" t="n"/>
       <c r="U8" s="3" t="n"/>
-      <c r="V8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>以上共计应补缴个人所得税14,997,500.00元。 以上共计应补缴印花税74,987.50元。 规定,对应补缴个人所得税14,997,500.00元加收从2011年4月1</t>
+        </is>
+      </c>
       <c r="W8" s="4" t="n"/>
-      <c r="X8" s="4" t="n">
-        <v>46122</v>
-      </c>
+      <c r="X8" s="4" t="n"/>
       <c r="Y8" s="4" t="n"/>
       <c r="Z8" s="4" t="n">
         <v>46229</v>
@@ -12318,7 +12366,7 @@
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>仅公告送达/仅文号线索</t>
+          <t>完整文书</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
@@ -12340,103 +12388,119 @@
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局关于送达税务处理决定书税务行政处罚决定书的公告</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="AI8" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ8" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>CASE-393a878d93a22709</t>
+          <t>CASE-7e3d4a321440d6a7</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>DOC-cda8cba853896b18</t>
+          <t>DOC-bed9330343ed06af</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>广东省</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>广州市</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>番禺区</t>
-        </is>
-      </c>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局广州市番禺区税务局</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>广州赞荣服装有限公司</t>
+          <t>天津展达科技有限公司</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>91440113MA59AJFJ1J</t>
+          <t>91120116300738701X</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr"/>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="3" t="n"/>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
       <c r="S9" s="3" t="n"/>
       <c r="T9" s="3" t="n"/>
       <c r="U9" s="3" t="n"/>
-      <c r="V9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
       <c r="W9" s="4" t="n"/>
-      <c r="X9" s="4" t="n">
-        <v>46091</v>
-      </c>
+      <c r="X9" s="4" t="n"/>
       <c r="Y9" s="4" t="n"/>
       <c r="Z9" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
         <v>46238</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>仅公告送达/仅文号线索</t>
+          <t>完整文书</t>
         </is>
       </c>
       <c r="AC9" s="2" t="inlineStr">
@@ -12454,124 +12518,116 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF9" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI9" s="2" t="inlineStr">
         <is>
-          <t>内容不匹配</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CASE-f78ec1a594442165</t>
+          <t>CASE-7e3d4a321440d6a7</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>DOC-fbbe4a664b14f54b</t>
+          <t>DOC-388bd01c01bbb789</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>安顺市</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局</t>
+          <t>国家税务总局天津市税务局第一稽查局</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局</t>
+          <t>国家税务总局天津市税务局第一稽查局</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
+          <t>天津展达科技有限公司</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>91520423MA6DLH799Q</t>
+          <t>91120116300738701X</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
+          <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
+          <t>津税一稽处〔2023〕59号</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>安市税稽罚〔2026〕1号</t>
+          <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R10" s="3" t="n">
-        <v>64884.41</v>
-      </c>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="n"/>
       <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3" t="n"/>
+      <c r="T10" s="3" t="n">
+        <v>131368.5</v>
+      </c>
       <c r="U10" s="3" t="n"/>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
-        </is>
-      </c>
-      <c r="W10" s="4" t="n">
-        <v>45898</v>
-      </c>
-      <c r="X10" s="4" t="n">
-        <v>46043</v>
-      </c>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="n"/>
+      <c r="X10" s="4" t="n"/>
       <c r="Y10" s="4" t="n"/>
       <c r="Z10" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AA10" s="4" t="n">
         <v>46238</v>
@@ -12596,15 +12652,11 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF10" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI10" s="2" t="inlineStr">
@@ -12613,683 +12665,25 @@
         </is>
       </c>
       <c r="AJ10" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CASE-f78ec1a594442165</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>DOC-9a828a6048b54b6c</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>贵州省</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>安顺市</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局安顺市税务局</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局安顺市税务局稽查局</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>91520423MA6DLH799Q</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>税务行政处罚决定书</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽罚〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽处〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽罚〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr">
-        <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3" t="n"/>
-      <c r="T11" s="3" t="n">
-        <v>200000</v>
-      </c>
-      <c r="U11" s="3" t="n"/>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
-        </is>
-      </c>
-      <c r="W11" s="4" t="n">
-        <v>45898</v>
-      </c>
-      <c r="X11" s="4" t="n">
-        <v>46043</v>
-      </c>
-      <c r="Y11" s="4" t="n"/>
-      <c r="Z11" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA11" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB11" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC11" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD11" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE11" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF11" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
-      <c r="AG11" s="2" t="inlineStr"/>
-      <c r="AH11" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
-        </is>
-      </c>
-      <c r="AI11" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ11" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CASE-1983d97878508732</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>DOC-f9760895b4f08cc2</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>内蒙古自治区</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>二连浩特市</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局二连浩特市税务局</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局二连浩特市税务局稽查局</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>二连市坤益腾金属有限公司</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>二税稽处〔2025〕1号</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>二税稽处〔2025〕1号</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>公司院内)涉嫌虚开增值税专用发票的情况进行检查,违法事实 你公司在无真实货物交易的情况下,“让他人为自己”虚开 得有下列虚开发票行为:(一)为他人、为自己开具与实际经营 国人民代表大会常务委员会关于惩治虚开、伪造和非法出售增值 〔1996〕210号)文件:“虚开增值税专用发票的,构成虚开增 值税专用发票罪,具有下列行为之一的,属于虚开增值税专用发 定,你公司上述违法事实中,“让他人为自己”虚开增值税专用 “为他人”虚开增值税专用发票97 份,金额 87,923,181.86 元, 二条第二款的规定虚开发票的,由税务机关没收违法所得; 虚开增值税专用发票行为暂不进行行政处罚,在司法部门作出决 十二条第二款的规定虚开发票的,由税务机关没收违法所得; 依法查处违法行为过程中,发现违法事实涉及的金额、违法事实 的情节、违法事实造成的后果等,根据刑法关于破坏社会主义市 定(二)》(公通字〔2022〕12 号)第五十六条:“〔虚开增值 税专用发票、用于骗取出口退税、抵扣税款发票案(刑法第二百 零五条)〕虚开增值税专用发票或者虚开用于骗取出口退税、抵 扣税款的其他发票,虚开的税款数额在十万元以上或者致使国家 公司虚开增值税专用发票的行为移送公安机关。</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>增值税</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3" t="n"/>
-      <c r="T12" s="3" t="n"/>
-      <c r="U12" s="3" t="n"/>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>二条第二款的规定虚开发票的,由税务机关没收违法所得; 十二条第二款的规定虚开发票的,由税务机关没收违法所得;</t>
-        </is>
-      </c>
-      <c r="W12" s="4" t="n"/>
-      <c r="X12" s="4" t="n"/>
-      <c r="Y12" s="4" t="n"/>
-      <c r="Z12" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA12" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB12" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC12" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD12" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE12" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="inlineStr"/>
-      <c r="AH12" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="AI12" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ12" s="2" t="inlineStr">
-        <is>
-          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CASE-d4b6986f3f97cd28</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>DOC-442cf3d9a5280c12</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>内蒙古自治区</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>鄂尔多斯市</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>第二稽查局</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>廖礼平</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>鄂税二稽处〔2023〕29号</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>鄂税二稽处〔2023〕29号</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>利煤炭有限责任公司股权涉税问题开展了检查,违法事实及处理</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>个人所得税、印花税</t>
-        </is>
-      </c>
-      <c r="R13" s="3" t="n">
-        <v>15072487.5</v>
-      </c>
-      <c r="S13" s="3" t="n">
-        <v>1046925</v>
-      </c>
-      <c r="T13" s="3" t="n"/>
-      <c r="U13" s="3" t="n"/>
-      <c r="V13" s="2" t="inlineStr">
-        <is>
-          <t>以上共计应补缴个人所得税14,997,500.00元。 以上共计应补缴印花税74,987.50元。 规定,对应补缴个人所得税14,997,500.00元加收从2011年4月1</t>
-        </is>
-      </c>
-      <c r="W13" s="4" t="n"/>
-      <c r="X13" s="4" t="n"/>
-      <c r="Y13" s="4" t="n"/>
-      <c r="Z13" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA13" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB13" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC13" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD13" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE13" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF13" s="2" t="inlineStr"/>
-      <c r="AG13" s="2" t="inlineStr"/>
-      <c r="AH13" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="AI13" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ13" s="2" t="inlineStr">
-        <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>CASE-7e3d4a321440d6a7</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>DOC-bed9330343ed06af</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>天津展达科技有限公司</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>91120116300738701X</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
-        </is>
-      </c>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="n">
-        <v>920146.9399999999</v>
-      </c>
-      <c r="S14" s="3" t="n"/>
-      <c r="T14" s="3" t="n"/>
-      <c r="U14" s="3" t="n"/>
-      <c r="V14" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
-      <c r="W14" s="4" t="n"/>
-      <c r="X14" s="4" t="n"/>
-      <c r="Y14" s="4" t="n"/>
-      <c r="Z14" s="4" t="n">
-        <v>46230</v>
-      </c>
-      <c r="AA14" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB14" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC14" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD14" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE14" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF14" s="2" t="inlineStr"/>
-      <c r="AG14" s="2" t="inlineStr"/>
-      <c r="AH14" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
-        </is>
-      </c>
-      <c r="AI14" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ14" s="2" t="inlineStr">
-        <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>CASE-7e3d4a321440d6a7</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>DOC-388bd01c01bbb789</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>天津展达科技有限公司</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>91120116300738701X</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>税务行政处罚决定书</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
-        </is>
-      </c>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R15" s="3" t="n"/>
-      <c r="S15" s="3" t="n"/>
-      <c r="T15" s="3" t="n">
-        <v>131368.5</v>
-      </c>
-      <c r="U15" s="3" t="n"/>
-      <c r="V15" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
-      <c r="W15" s="4" t="n"/>
-      <c r="X15" s="4" t="n"/>
-      <c r="Y15" s="4" t="n"/>
-      <c r="Z15" s="4" t="n">
-        <v>46230</v>
-      </c>
-      <c r="AA15" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB15" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC15" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD15" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE15" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr"/>
-      <c r="AH15" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
-        </is>
-      </c>
-      <c r="AI15" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ15" s="2" t="inlineStr">
         <is>
           <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ15"/>
-  <conditionalFormatting sqref="AD2:AD15">
+  <autoFilter ref="A1:AJ10"/>
+  <conditionalFormatting sqref="AD2:AD10">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI15">
+  <conditionalFormatting sqref="AI2:AI10">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13297,20 +12691,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF9" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF10" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE11" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF11" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE13" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE14" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE15" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE8" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE10" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -13323,7 +12712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ9"/>
+  <dimension ref="A1:AJ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13784,66 +13173,66 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CASE-365e8a924cf64611</t>
+          <t>CASE-393a878d93a22709</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>DOC-4d14eba16f9aa8a0</t>
+          <t>DOC-cda8cba853896b18</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>广东省</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>贵阳市</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+          <t>广州市</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>番禺区</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
+          <t>国家税务总局广州市番禺区税务局</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>贵州博泰工贸有限公司</t>
+          <t>广州赞荣服装有限公司</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>91520115587255589F</t>
+          <t>91440113MA59AJFJ1J</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>筑税三稽处〔2026〕38号</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽处〔2026〕38号</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="3" t="n"/>
@@ -13853,7 +13242,7 @@
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="4" t="n"/>
       <c r="X4" s="4" t="n">
-        <v>46224</v>
+        <v>46091</v>
       </c>
       <c r="Y4" s="4" t="n"/>
       <c r="Z4" s="4" t="n">
@@ -13882,648 +13271,42 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AF4" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
       <c r="AG4" s="2" t="inlineStr"/>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局贵阳市税务局第三稽查局关于送达税务处理决定书、税务行政处罚决定书的公告</t>
+          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
         </is>
       </c>
       <c r="AI4" s="2" t="inlineStr">
         <is>
-          <t>页面已删除</t>
+          <t>内容不匹配</t>
         </is>
       </c>
       <c r="AJ4" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>CASE-a62e569c195adc3c</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>DOC-b1dda915d4e6117d</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>贵州省</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>遵义市</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局遵义市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局遵义市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>贵州服格定商贸有限公司</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>91520302MABUEHN034</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>遵税一稽处〔2026〕30号</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>遵税一稽处〔2026〕30号</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>情况进行了检查,违法事实及处理决定如下: 2023年度开具增值税电子普通发票合计金额36,788.18元,税额905.82元,价税37,694.00元,未申报纳税,并且你公司从2023年起所有税种没有进行纳税申报。</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>增值税</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3" t="n"/>
-      <c r="T5" s="3" t="n"/>
-      <c r="U5" s="3" t="n"/>
-      <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="4" t="n"/>
-      <c r="X5" s="4" t="n">
-        <v>46185</v>
-      </c>
-      <c r="Y5" s="4" t="n"/>
-      <c r="Z5" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA5" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB5" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC5" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD5" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE5" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr"/>
-      <c r="AH5" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局遵义市税务局第一稽查局税务处理决定书(遵税一稽处〔2026〕30 号)</t>
-        </is>
-      </c>
-      <c r="AI5" s="2" t="inlineStr">
-        <is>
-          <t>页面已删除</t>
-        </is>
-      </c>
-      <c r="AJ5" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>CASE-f8625e66b291a216</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>DOC-7970511393924720</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>贵州省</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>贵阳市</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第二稽查局</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第二稽查局</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>贵州翰缤商贸有限公司</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>91520114MAAK1C546F</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>筑税二稽处〔2026〕27号</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>筑税二稽处〔2026〕27号</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n"/>
-      <c r="U6" s="3" t="n"/>
-      <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="4" t="n"/>
-      <c r="X6" s="4" t="n">
-        <v>46156</v>
-      </c>
-      <c r="Y6" s="4" t="n"/>
-      <c r="Z6" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA6" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB6" s="2" t="inlineStr">
-        <is>
-          <t>仅公告送达/仅文号线索</t>
-        </is>
-      </c>
-      <c r="AC6" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD6" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE6" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr"/>
-      <c r="AH6" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第二稽查局关于送达《税务处理决定书》的公告</t>
-        </is>
-      </c>
-      <c r="AI6" s="2" t="inlineStr">
-        <is>
-          <t>页面已删除</t>
-        </is>
-      </c>
-      <c r="AJ6" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>CASE-0f4867f7b70d12f3</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>DOC-6f25d6b79e123d03</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>贵州省</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>贵阳市</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>贵州铂朗物流有限公司</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>91520115MAAK0DB335</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽处〔2026〕17号</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽处〔2026〕17号</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽罚〔2026〕22号</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="3" t="n"/>
-      <c r="S7" s="3" t="n"/>
-      <c r="T7" s="3" t="n"/>
-      <c r="U7" s="3" t="n"/>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="4" t="n"/>
-      <c r="X7" s="4" t="n">
-        <v>46122</v>
-      </c>
-      <c r="Y7" s="4" t="n"/>
-      <c r="Z7" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA7" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB7" s="2" t="inlineStr">
-        <is>
-          <t>仅公告送达/仅文号线索</t>
-        </is>
-      </c>
-      <c r="AC7" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD7" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE7" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr"/>
-      <c r="AH7" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局关于送达税务处理决定书税务行政处罚决定书的公告</t>
-        </is>
-      </c>
-      <c r="AI7" s="2" t="inlineStr">
-        <is>
-          <t>页面已删除</t>
-        </is>
-      </c>
-      <c r="AJ7" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>CASE-0f4867f7b70d12f3</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>DOC-e8233eb0e06b6e3e</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>贵州省</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>贵阳市</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>贵州铂朗物流有限公司</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>91520115MAAK0DB335</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>税务行政处罚决定书</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽罚〔2026〕22号</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽处〔2026〕17号</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>筑税三稽罚〔2026〕22号</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
-      <c r="T8" s="3" t="n"/>
-      <c r="U8" s="3" t="n"/>
-      <c r="V8" s="2" t="inlineStr"/>
-      <c r="W8" s="4" t="n"/>
-      <c r="X8" s="4" t="n">
-        <v>46122</v>
-      </c>
-      <c r="Y8" s="4" t="n"/>
-      <c r="Z8" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA8" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB8" s="2" t="inlineStr">
-        <is>
-          <t>仅公告送达/仅文号线索</t>
-        </is>
-      </c>
-      <c r="AC8" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD8" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE8" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF8" s="2" t="inlineStr"/>
-      <c r="AG8" s="2" t="inlineStr"/>
-      <c r="AH8" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局贵阳市税务局第三稽查局关于送达税务处理决定书税务行政处罚决定书的公告</t>
-        </is>
-      </c>
-      <c r="AI8" s="2" t="inlineStr">
-        <is>
-          <t>页面已删除</t>
-        </is>
-      </c>
-      <c r="AJ8" s="2" t="inlineStr">
-        <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CASE-393a878d93a22709</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>DOC-cda8cba853896b18</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>广东省</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>广州市</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>番禺区</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局广州市番禺区税务局</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>广州赞荣服装有限公司</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>91440113MA59AJFJ1J</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>税务行政处罚决定书</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="n"/>
-      <c r="V9" s="2" t="inlineStr"/>
-      <c r="W9" s="4" t="n"/>
-      <c r="X9" s="4" t="n">
-        <v>46091</v>
-      </c>
-      <c r="Y9" s="4" t="n"/>
-      <c r="Z9" s="4" t="n">
-        <v>46229</v>
-      </c>
-      <c r="AA9" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="AB9" s="2" t="inlineStr">
-        <is>
-          <t>仅公告送达/仅文号线索</t>
-        </is>
-      </c>
-      <c r="AC9" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD9" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE9" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF9" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
-      <c r="AG9" s="2" t="inlineStr"/>
-      <c r="AH9" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
-        </is>
-      </c>
-      <c r="AI9" s="2" t="inlineStr">
-        <is>
-          <t>内容不匹配</t>
-        </is>
-      </c>
-      <c r="AJ9" s="2" t="inlineStr">
         <is>
           <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ9"/>
-  <conditionalFormatting sqref="AD2:AD9">
+  <autoFilter ref="A1:AJ4"/>
+  <conditionalFormatting sqref="AD2:AD4">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI9">
+  <conditionalFormatting sqref="AI2:AI4">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14531,12 +13314,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF4" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -14549,7 +13327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15578,8 +14356,204 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T22:34:42+08:00</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 至 2026-08-04</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ProxyError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by ProxyError('Unable to connect to proxy', OSError('Tunnel connection failed: 502...</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T22:37:15+08:00</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 至 2026-08-04</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ProxyError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by ProxyError('Unable to connect to proxy', OSError('Tunnel connection failed: 502...</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T22:40:35+08:00</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 至 2026-08-04</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ProxyError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by ProxyError('Unable to connect to proxy', OSError('Tunnel connection failed: 502...</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T22:42:34+08:00</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28 至 2026-08-04</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ProxyError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by ProxyError('Unable to connect to proxy', OSError('Tunnel connection failed: 502...</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M21"/>
+  <autoFilter ref="A1:M25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-05
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -793,7 +793,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -917,7 +917,7 @@
         <v>46236</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         <v>46236</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1555,7 +1555,7 @@
         <v>46233</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1691,7 +1691,7 @@
         <v>46234</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1809,7 +1809,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2571,7 +2571,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2695,7 +2695,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2955,7 +2955,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3079,7 +3079,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3205,7 +3205,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3445,7 +3445,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3567,7 +3567,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3689,7 +3689,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3811,7 +3811,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4055,7 +4055,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4315,7 +4315,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4437,7 +4437,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4843,7 +4843,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4985,7 +4985,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5115,7 +5115,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5243,7 +5243,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5367,7 +5367,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5501,7 +5501,7 @@
         <v>46230</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5635,7 +5635,7 @@
         <v>46230</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -6199,7 +6199,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -6329,7 +6329,7 @@
         <v>46233</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -6465,7 +6465,7 @@
         <v>46234</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -6601,7 +6601,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -6869,7 +6869,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -7001,7 +7001,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -7129,7 +7129,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -7267,7 +7267,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -7403,7 +7403,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -7535,7 +7535,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -7815,7 +7815,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -7945,7 +7945,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -8073,7 +8073,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -8197,7 +8197,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -8331,7 +8331,7 @@
         <v>46230</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -8465,7 +8465,7 @@
         <v>46230</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -8863,7 +8863,7 @@
         <v>46236</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -8989,7 +8989,7 @@
         <v>46236</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -9115,7 +9115,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -9241,7 +9241,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -9363,7 +9363,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -9481,7 +9481,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -9603,7 +9603,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -9721,7 +9721,7 @@
         <v>46229</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -9843,7 +9843,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -9969,7 +9969,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -10095,7 +10095,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -10213,7 +10213,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -10335,7 +10335,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -10457,7 +10457,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -10579,7 +10579,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -10701,7 +10701,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -10823,7 +10823,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -10945,7 +10945,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -11063,7 +11063,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -11185,7 +11185,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -11590,7 +11590,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11708,7 +11708,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11826,7 +11826,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11968,7 +11968,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -12110,7 +12110,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -12238,7 +12238,7 @@
         <v>46229</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -12362,7 +12362,7 @@
         <v>46229</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -12496,7 +12496,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -12630,7 +12630,7 @@
         <v>46230</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -13013,7 +13013,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -13131,7 +13131,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -13249,7 +13249,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -13327,7 +13327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14552,8 +14552,57 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T14:38:52+08:00</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 至 2026-08-05</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M25"/>
+  <autoFilter ref="A1:M26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix continuous tax decision updates
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE34" s="5" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="AI34" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>附件正常</t>
         </is>
       </c>
       <c r="AJ34" s="2" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE35" s="5" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="AI35" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>附件正常</t>
         </is>
       </c>
       <c r="AJ35" s="2" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE14" s="5" t="inlineStr">
@@ -7708,7 +7708,7 @@
       </c>
       <c r="AI14" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>附件正常</t>
         </is>
       </c>
       <c r="AJ14" s="2" t="inlineStr">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE15" s="5" t="inlineStr">
@@ -7850,7 +7850,7 @@
       </c>
       <c r="AI15" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>附件正常</t>
         </is>
       </c>
       <c r="AJ15" s="2" t="inlineStr">
@@ -11289,7 +11289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ10"/>
+  <dimension ref="A1:AJ8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11872,49 +11872,45 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CASE-f78ec1a594442165</t>
+          <t>CASE-1983d97878508732</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>DOC-fbbe4a664b14f54b</t>
+          <t>DOC-f9760895b4f08cc2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>内蒙古自治区</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>安顺市</t>
+          <t>二连浩特市</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局</t>
+          <t>国家税务总局二连浩特市税务局</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局</t>
+          <t>国家税务总局二连浩特市税务局稽查局</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>91520423MA6DLH799Q</t>
-        </is>
-      </c>
+          <t>二连市坤益腾金属有限公司</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
@@ -11923,46 +11919,36 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
+          <t>二税稽处〔2025〕1号</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽罚〔2026〕1号</t>
-        </is>
-      </c>
+          <t>二税稽处〔2025〕1号</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>公司院内)涉嫌虚开增值税专用发票的情况进行检查,违法事实 你公司在无真实货物交易的情况下,“让他人为自己”虚开 得有下列虚开发票行为:(一)为他人、为自己开具与实际经营 国人民代表大会常务委员会关于惩治虚开、伪造和非法出售增值 〔1996〕210号)文件:“虚开增值税专用发票的,构成虚开增 值税专用发票罪,具有下列行为之一的,属于虚开增值税专用发 定,你公司上述违法事实中,“让他人为自己”虚开增值税专用 “为他人”虚开增值税专用发票97 份,金额 87,923,181.86 元, 二条第二款的规定虚开发票的,由税务机关没收违法所得; 虚开增值税专用发票行为暂不进行行政处罚,在司法部门作出决 十二条第二款的规定虚开发票的,由税务机关没收违法所得; 依法查处违法行为过程中,发现违法事实涉及的金额、违法事实 的情节、违法事实造成的后果等,根据刑法关于破坏社会主义市 定(二)》(公通字〔2022〕12 号)第五十六条:“〔虚开增值 税专用发票、用于骗取出口退税、抵扣税款发票案(刑法第二百 零五条)〕虚开增值税专用发票或者虚开用于骗取出口退税、抵 扣税款的其他发票,虚开的税款数额在十万元以上或者致使国家 公司虚开增值税专用发票的行为移送公安机关。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="n">
-        <v>64884.41</v>
-      </c>
+          <t>增值税</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="n"/>
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="3" t="n"/>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
-        </is>
-      </c>
-      <c r="W5" s="4" t="n">
-        <v>45898</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>46043</v>
-      </c>
+          <t>二条第二款的规定虚开发票的,由税务机关没收违法所得; 十二条第二款的规定虚开发票的,由税务机关没收违法所得;</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n"/>
+      <c r="X5" s="4" t="n"/>
       <c r="Y5" s="4" t="n"/>
       <c r="Z5" s="4" t="n">
         <v>46229</v>
@@ -11990,15 +11976,11 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF5" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="inlineStr"/>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="AI5" s="2" t="inlineStr">
@@ -12008,103 +11990,89 @@
       </c>
       <c r="AJ5" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。 字段“主要违法事实”存在冲突:保留原值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”,新值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CASE-f78ec1a594442165</t>
+          <t>CASE-d4b6986f3f97cd28</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>DOC-9a828a6048b54b6c</t>
+          <t>DOC-442cf3d9a5280c12</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>内蒙古自治区</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>安顺市</t>
+          <t>鄂尔多斯市</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局安顺市税务局</t>
-        </is>
-      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局</t>
+          <t>第二稽查局</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>91520423MA6DLH799Q</t>
-        </is>
-      </c>
+          <t>廖礼平</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>安市税稽罚〔2026〕1号</t>
+          <t>鄂税二稽处〔2023〕29号</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽罚〔2026〕1号</t>
-        </is>
-      </c>
+          <t>鄂税二稽处〔2023〕29号</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>利煤炭有限责任公司股权涉税问题开展了检查,违法事实及处理</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n">
-        <v>200000</v>
-      </c>
+          <t>个人所得税、印花税</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>15072487.5</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>1046925</v>
+      </c>
+      <c r="T6" s="3" t="n"/>
       <c r="U6" s="3" t="n"/>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>45898</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>46043</v>
-      </c>
+          <t>以上共计应补缴个人所得税14,997,500.00元。 以上共计应补缴印花税74,987.50元。 规定,对应补缴个人所得税14,997,500.00元加收从2011年4月1</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="n"/>
+      <c r="X6" s="4" t="n"/>
       <c r="Y6" s="4" t="n"/>
       <c r="Z6" s="4" t="n">
         <v>46229</v>
@@ -12132,15 +12100,11 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF6" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="AI6" s="2" t="inlineStr">
@@ -12150,51 +12114,55 @@
       </c>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CASE-1983d97878508732</t>
+          <t>CASE-7e3d4a321440d6a7</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>DOC-f9760895b4f08cc2</t>
+          <t>DOC-bed9330343ed06af</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>内蒙古自治区</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>二连浩特市</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局二连浩特市税务局</t>
+          <t>国家税务总局天津市税务局第一稽查局</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局二连浩特市税务局稽查局</t>
+          <t>国家税务总局天津市税务局第一稽查局</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>二连市坤益腾金属有限公司</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -12203,39 +12171,45 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>二税稽处〔2025〕1号</t>
+          <t>津税一稽处〔2023〕59号</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>二税稽处〔2025〕1号</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr"/>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>公司院内)涉嫌虚开增值税专用发票的情况进行检查,违法事实 你公司在无真实货物交易的情况下,“让他人为自己”虚开 得有下列虚开发票行为:(一)为他人、为自己开具与实际经营 国人民代表大会常务委员会关于惩治虚开、伪造和非法出售增值 〔1996〕210号)文件:“虚开增值税专用发票的,构成虚开增 值税专用发票罪,具有下列行为之一的,属于虚开增值税专用发 定,你公司上述违法事实中,“让他人为自己”虚开增值税专用 “为他人”虚开增值税专用发票97 份,金额 87,923,181.86 元, 二条第二款的规定虚开发票的,由税务机关没收违法所得; 虚开增值税专用发票行为暂不进行行政处罚,在司法部门作出决 十二条第二款的规定虚开发票的,由税务机关没收违法所得; 依法查处违法行为过程中,发现违法事实涉及的金额、违法事实 的情节、违法事实造成的后果等,根据刑法关于破坏社会主义市 定(二)》(公通字〔2022〕12 号)第五十六条:“〔虚开增值 税专用发票、用于骗取出口退税、抵扣税款发票案(刑法第二百 零五条)〕虚开增值税专用发票或者虚开用于骗取出口退税、抵 扣税款的其他发票,虚开的税款数额在十万元以上或者致使国家 公司虚开增值税专用发票的行为移送公安机关。</t>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>增值税</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="n"/>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
       <c r="S7" s="3" t="n"/>
       <c r="T7" s="3" t="n"/>
       <c r="U7" s="3" t="n"/>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>二条第二款的规定虚开发票的,由税务机关没收违法所得; 十二条第二款的规定虚开发票的,由税务机关没收违法所得;</t>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W7" s="4" t="n"/>
       <c r="X7" s="4" t="n"/>
       <c r="Y7" s="4" t="n"/>
       <c r="Z7" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AA7" s="4" t="n">
         <v>46239</v>
@@ -12264,7 +12238,7 @@
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI7" s="2" t="inlineStr">
@@ -12274,92 +12248,102 @@
       </c>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CASE-d4b6986f3f97cd28</t>
+          <t>CASE-7e3d4a321440d6a7</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DOC-442cf3d9a5280c12</t>
+          <t>DOC-388bd01c01bbb789</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>内蒙古自治区</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯市</t>
+          <t>天津市</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>第二稽查局</t>
+          <t>国家税务总局天津市税务局第一稽查局</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>廖礼平</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>鄂税二稽处〔2023〕29号</t>
+          <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>鄂税二稽处〔2023〕29号</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr"/>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>利煤炭有限责任公司股权涉税问题开展了检查,违法事实及处理</t>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>个人所得税、印花税</t>
-        </is>
-      </c>
-      <c r="R8" s="3" t="n">
-        <v>15072487.5</v>
-      </c>
-      <c r="S8" s="3" t="n">
-        <v>1046925</v>
-      </c>
-      <c r="T8" s="3" t="n"/>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="n"/>
+      <c r="S8" s="3" t="n"/>
+      <c r="T8" s="3" t="n">
+        <v>131368.5</v>
+      </c>
       <c r="U8" s="3" t="n"/>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>以上共计应补缴个人所得税14,997,500.00元。 以上共计应补缴印花税74,987.50元。 规定,对应补缴个人所得税14,997,500.00元加收从2011年4月1</t>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W8" s="4" t="n"/>
       <c r="X8" s="4" t="n"/>
       <c r="Y8" s="4" t="n"/>
       <c r="Z8" s="4" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
         <v>46239</v>
@@ -12388,7 +12372,7 @@
       <c r="AG8" s="2" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI8" s="2" t="inlineStr">
@@ -12397,293 +12381,25 @@
         </is>
       </c>
       <c r="AJ8" s="2" t="inlineStr">
-        <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CASE-7e3d4a321440d6a7</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>DOC-bed9330343ed06af</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>天津展达科技有限公司</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>91120116300738701X</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>税务处理决定书</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
-        </is>
-      </c>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R9" s="3" t="n">
-        <v>920146.9399999999</v>
-      </c>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="n"/>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="n"/>
-      <c r="X9" s="4" t="n"/>
-      <c r="Y9" s="4" t="n"/>
-      <c r="Z9" s="4" t="n">
-        <v>46230</v>
-      </c>
-      <c r="AA9" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="AB9" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC9" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD9" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE9" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF9" s="2" t="inlineStr"/>
-      <c r="AG9" s="2" t="inlineStr"/>
-      <c r="AH9" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
-        </is>
-      </c>
-      <c r="AI9" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ9" s="2" t="inlineStr">
-        <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>CASE-7e3d4a321440d6a7</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>DOC-388bd01c01bbb789</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>天津市</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>天津展达科技有限公司</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>91120116300738701X</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>税务行政处罚决定书</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3" t="n">
-        <v>131368.5</v>
-      </c>
-      <c r="U10" s="3" t="n"/>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
-      <c r="W10" s="4" t="n"/>
-      <c r="X10" s="4" t="n"/>
-      <c r="Y10" s="4" t="n"/>
-      <c r="Z10" s="4" t="n">
-        <v>46230</v>
-      </c>
-      <c r="AA10" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="AB10" s="2" t="inlineStr">
-        <is>
-          <t>完整文书</t>
-        </is>
-      </c>
-      <c r="AC10" s="2" t="inlineStr">
-        <is>
-          <t>税务机关官网</t>
-        </is>
-      </c>
-      <c r="AD10" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="AE10" s="5" t="inlineStr">
-        <is>
-          <t>打开原文</t>
-        </is>
-      </c>
-      <c r="AF10" s="2" t="inlineStr"/>
-      <c r="AG10" s="2" t="inlineStr"/>
-      <c r="AH10" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
-        </is>
-      </c>
-      <c r="AI10" s="2" t="inlineStr">
-        <is>
-          <t>正常</t>
-        </is>
-      </c>
-      <c r="AJ10" s="2" t="inlineStr">
         <is>
           <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ10"/>
-  <conditionalFormatting sqref="AD2:AD10">
+  <autoFilter ref="A1:AJ8"/>
+  <conditionalFormatting sqref="AD2:AD8">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI10">
+  <conditionalFormatting sqref="AI2:AI8">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12693,13 +12409,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF4" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE8" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -13327,7 +13039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14601,8 +14313,204 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:11:39+08:00</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 至 2026-08-05</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/nanning/xxgk/swjcgg: RetryError: HTTPConnectionPool(host='127.0.0.1', port=7897): Max retries exceeded with url: http://guangxi.chinatax.gov.cn:8000/nanning/xxgk/swjcgg/ (Caused by ResponseError('too many 502 error responses'))</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="54" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:13:04+08:00</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 至 2026-08-05</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/nanning/xxgk/swjcgg: RetryError: HTTPConnectionPool(host='127.0.0.1', port=7897): Max retries exceeded with url: http://guangxi.chinatax.gov.cn:8000/nanning/xxgk/swjcgg/ (Caused by ResponseError('too many 502 error responses'))</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="54" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:18:21+08:00</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 至 2026-08-05</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://guangxi.chinatax.gov.cn/nanning/xxgk/swjcgg: RetryErro...</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:32:30+08:00</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 至 2026-08-05</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://guangxi.chinatax.gov.cn/nanning/xxgk/swjcgg: RetryErro...</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M26"/>
+  <autoFilter ref="A1:M30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-07
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -819,7 +819,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -937,7 +941,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -9991,7 +9999,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -10109,7 +10121,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -14371,7 +14387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16147,8 +16163,57 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T14:05:45+08:00</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 至 2026-08-07</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M36"/>
+  <autoFilter ref="A1:M37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-08
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46241</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         <v>46240</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>46236</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1937,7 +1937,7 @@
         <v>46233</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
         <v>46234</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2191,7 +2191,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2309,7 +2309,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2445,7 +2445,7 @@
         <v>46238</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2707,7 +2707,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3103,7 +3103,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3361,7 +3361,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3487,7 +3487,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3621,7 +3621,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3745,7 +3745,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3871,7 +3871,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3989,7 +3989,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4111,7 +4111,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4233,7 +4233,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4355,7 +4355,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4477,7 +4477,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4599,7 +4599,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4721,7 +4721,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4839,7 +4839,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4981,7 +4981,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5103,7 +5103,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5371,7 +5371,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5509,7 +5509,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5651,7 +5651,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5781,7 +5781,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5909,7 +5909,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6033,7 +6033,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
         <v>46230</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6301,7 +6301,7 @@
         <v>46230</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6749,7 +6749,7 @@
         <v>46240</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -6883,7 +6883,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7011,7 +7011,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7141,7 +7141,7 @@
         <v>46233</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7277,7 +7277,7 @@
         <v>46234</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7413,7 +7413,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -7553,7 +7553,7 @@
         <v>46240</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -7695,7 +7695,7 @@
         <v>46240</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -7831,7 +7831,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -7965,7 +7965,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8097,7 +8097,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8225,7 +8225,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8363,7 +8363,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -8499,7 +8499,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -8769,7 +8769,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -8911,7 +8911,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9041,7 +9041,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -9169,7 +9169,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -9293,7 +9293,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -9427,7 +9427,7 @@
         <v>46230</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -9561,7 +9561,7 @@
         <v>46230</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -9965,7 +9965,7 @@
         <v>46241</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -10087,7 +10087,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10209,7 +10209,7 @@
         <v>46236</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10335,7 +10335,7 @@
         <v>46236</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10461,7 +10461,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10587,7 +10587,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10709,7 +10709,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10827,7 +10827,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10949,7 +10949,7 @@
         <v>46229</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11067,7 +11067,7 @@
         <v>46229</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11189,7 +11189,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11315,7 +11315,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11441,7 +11441,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -11559,7 +11559,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -11681,7 +11681,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -11925,7 +11925,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12047,7 +12047,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -12169,7 +12169,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -12291,7 +12291,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -12409,7 +12409,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -12531,7 +12531,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -12938,7 +12938,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -13056,7 +13056,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -13174,7 +13174,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -13302,7 +13302,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -13426,7 +13426,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -13560,7 +13560,7 @@
         <v>46230</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -13694,7 +13694,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14191,7 +14191,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14309,7 +14309,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14387,7 +14387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16212,8 +16212,57 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08T13:07:28+08:00</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01 至 2026-08-08</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M37"/>
+  <autoFilter ref="A1:M38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-09
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1489,7 +1489,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1615,7 +1619,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -11075,7 +11083,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -11201,7 +11213,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -15467,7 +15483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17447,8 +17463,57 @@
         </is>
       </c>
     </row>
+    <row r="41" ht="54" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09T13:36:08+08:00</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02 至 2026-08-09</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /qzsswj/xxgk/sjxxgk/qtgg_23603/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinata...</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M40"/>
+  <autoFilter ref="A1:M41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-10
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -799,7 +799,7 @@
         <v>46242</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>46241</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
         <v>46241</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         <v>46240</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         <v>46243</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1581,7 +1581,7 @@
         <v>46243</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         <v>46236</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1965,7 +1965,7 @@
         <v>46236</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2091,7 +2091,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2477,7 +2477,7 @@
         <v>46233</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2613,7 +2613,7 @@
         <v>46234</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
         <v>46238</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         <v>46238</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         <v>46238</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3109,7 +3109,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>46240</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         <v>46240</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3777,7 +3777,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4027,7 +4027,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4161,7 +4161,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4411,7 +4411,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4529,7 +4529,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4651,7 +4651,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4895,7 +4895,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5139,7 +5139,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5261,7 +5261,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5379,7 +5379,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5521,7 +5521,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5779,7 +5779,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5911,7 +5911,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6049,7 +6049,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6321,7 +6321,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6449,7 +6449,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6707,7 +6707,7 @@
         <v>46230</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6841,7 +6841,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -7299,7 +7299,7 @@
         <v>46242</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7577,7 +7577,7 @@
         <v>46240</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7711,7 +7711,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7839,7 +7839,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7969,7 +7969,7 @@
         <v>46233</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8105,7 +8105,7 @@
         <v>46234</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8241,7 +8241,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8381,7 +8381,7 @@
         <v>46240</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8659,7 +8659,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8793,7 +8793,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8925,7 +8925,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9053,7 +9053,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9191,7 +9191,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9327,7 +9327,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9459,7 +9459,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9597,7 +9597,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -9739,7 +9739,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -9997,7 +9997,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -10121,7 +10121,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -10255,7 +10255,7 @@
         <v>46230</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -10389,7 +10389,7 @@
         <v>46230</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -10797,7 +10797,7 @@
         <v>46241</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -10919,7 +10919,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11045,7 +11045,7 @@
         <v>46243</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11175,7 +11175,7 @@
         <v>46243</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11301,7 +11301,7 @@
         <v>46236</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11427,7 +11427,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11553,7 +11553,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -11679,7 +11679,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -11801,7 +11801,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11919,7 +11919,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -12041,7 +12041,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -12159,7 +12159,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -12407,7 +12407,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -12651,7 +12651,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -12773,7 +12773,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12895,7 +12895,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -13261,7 +13261,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -13383,7 +13383,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -13501,7 +13501,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -13623,7 +13623,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -14034,7 +14034,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14152,7 +14152,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14270,7 +14270,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14398,7 +14398,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14522,7 +14522,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14656,7 +14656,7 @@
         <v>46230</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14790,7 +14790,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15169,7 +15169,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15287,7 +15287,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15405,7 +15405,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17512,8 +17512,57 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10T13:41:25+08:00</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03 至 2026-08-10</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/nanning/xxgk/swjcgg: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /nanning/xxgk/swjcgg (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('Remote end closed c...</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M41"/>
+  <autoFilter ref="A1:M42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-11
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -799,7 +799,7 @@
         <v>46242</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>46241</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
         <v>46241</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         <v>46240</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         <v>46243</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1581,7 +1581,7 @@
         <v>46243</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         <v>46236</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1965,7 +1965,7 @@
         <v>46236</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2091,7 +2091,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2477,7 +2477,7 @@
         <v>46233</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2613,7 +2613,7 @@
         <v>46234</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
         <v>46238</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         <v>46238</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         <v>46238</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3109,7 +3109,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>46240</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         <v>46240</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3777,7 +3777,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4027,7 +4027,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4161,7 +4161,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4411,7 +4411,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4529,7 +4529,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4651,7 +4651,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4895,7 +4895,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5139,7 +5139,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5261,7 +5261,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5379,7 +5379,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5521,7 +5521,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5779,7 +5779,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5911,7 +5911,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6049,7 +6049,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6321,7 +6321,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6449,7 +6449,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6707,7 +6707,7 @@
         <v>46230</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6841,7 +6841,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -7299,7 +7299,7 @@
         <v>46242</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7577,7 +7577,7 @@
         <v>46240</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7711,7 +7711,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7839,7 +7839,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7969,7 +7969,7 @@
         <v>46233</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8105,7 +8105,7 @@
         <v>46234</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8241,7 +8241,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8381,7 +8381,7 @@
         <v>46240</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8659,7 +8659,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8793,7 +8793,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8925,7 +8925,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9053,7 +9053,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9191,7 +9191,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9327,7 +9327,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9459,7 +9459,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9597,7 +9597,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -9739,7 +9739,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -9997,7 +9997,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -10121,7 +10121,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -10255,7 +10255,7 @@
         <v>46230</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -10389,7 +10389,7 @@
         <v>46230</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -10797,7 +10797,7 @@
         <v>46241</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -10919,7 +10919,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11045,7 +11045,7 @@
         <v>46243</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11175,7 +11175,7 @@
         <v>46243</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11301,7 +11301,7 @@
         <v>46236</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11427,7 +11427,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11553,7 +11553,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -11679,7 +11679,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -11801,7 +11801,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11919,7 +11919,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -12041,7 +12041,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -12159,7 +12159,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -12407,7 +12407,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -12651,7 +12651,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -12773,7 +12773,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12895,7 +12895,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -13261,7 +13261,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -13383,7 +13383,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -13501,7 +13501,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -13623,7 +13623,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -14034,7 +14034,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14152,7 +14152,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14270,7 +14270,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14398,7 +14398,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14522,7 +14522,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14656,7 +14656,7 @@
         <v>46230</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14790,7 +14790,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15169,7 +15169,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15287,7 +15287,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15405,7 +15405,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17610,8 +17610,57 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11T13:18:46+08:00</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04 至 2026-08-11</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/hechi/tzgg_15562/tzgg_15563/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /hechi/tzgg_15562/tzgg_15563/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('R...</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M43"/>
+  <autoFilter ref="A1:M44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-12
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -799,7 +799,7 @@
         <v>46242</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>46241</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
         <v>46241</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         <v>46240</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         <v>46243</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1581,7 +1581,7 @@
         <v>46243</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         <v>46236</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1965,7 +1965,7 @@
         <v>46236</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2091,7 +2091,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2477,7 +2477,7 @@
         <v>46233</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2613,7 +2613,7 @@
         <v>46234</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
         <v>46238</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         <v>46238</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         <v>46238</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3109,7 +3109,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>46240</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         <v>46240</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3777,7 +3777,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4027,7 +4027,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4161,7 +4161,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4411,7 +4411,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4529,7 +4529,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4651,7 +4651,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4895,7 +4895,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5139,7 +5139,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5261,7 +5261,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5379,7 +5379,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5521,7 +5521,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5779,7 +5779,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5911,7 +5911,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6049,7 +6049,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6321,7 +6321,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6449,7 +6449,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6707,7 +6707,7 @@
         <v>46230</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6841,7 +6841,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -7299,7 +7299,7 @@
         <v>46242</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7577,7 +7577,7 @@
         <v>46240</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7711,7 +7711,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -7839,7 +7839,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -7969,7 +7969,7 @@
         <v>46233</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8105,7 +8105,7 @@
         <v>46234</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8241,7 +8241,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8381,7 +8381,7 @@
         <v>46240</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8659,7 +8659,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -8793,7 +8793,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -8925,7 +8925,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9053,7 +9053,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9191,7 +9191,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9327,7 +9327,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9459,7 +9459,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9597,7 +9597,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -9739,7 +9739,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -9997,7 +9997,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -10121,7 +10121,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -10255,7 +10255,7 @@
         <v>46230</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -10389,7 +10389,7 @@
         <v>46230</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -10797,7 +10797,7 @@
         <v>46241</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -10919,7 +10919,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11045,7 +11045,7 @@
         <v>46243</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11175,7 +11175,7 @@
         <v>46243</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11301,7 +11301,7 @@
         <v>46236</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11427,7 +11427,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11553,7 +11553,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -11679,7 +11679,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -11801,7 +11801,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11919,7 +11919,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -12041,7 +12041,7 @@
         <v>46229</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -12159,7 +12159,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -12407,7 +12407,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -12651,7 +12651,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -12773,7 +12773,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12895,7 +12895,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -13261,7 +13261,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -13383,7 +13383,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -13501,7 +13501,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -13623,7 +13623,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -14034,7 +14034,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14152,7 +14152,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14270,7 +14270,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14398,7 +14398,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14522,7 +14522,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14656,7 +14656,7 @@
         <v>46230</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14790,7 +14790,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15169,7 +15169,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15287,7 +15287,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15405,7 +15405,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17708,8 +17708,57 @@
         </is>
       </c>
     </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12T13:43:38+08:00</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05 至 2026-08-12</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M45"/>
+  <autoFilter ref="A1:M46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-13
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -819,7 +819,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -909,7 +913,7 @@
         <v>46246</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -947,7 +951,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1045,7 +1053,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1185,7 +1193,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1311,7 +1319,7 @@
         <v>46241</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1433,7 +1441,7 @@
         <v>46241</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1567,7 +1575,7 @@
         <v>46240</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1697,7 +1705,7 @@
         <v>46243</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1827,7 +1835,7 @@
         <v>46243</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1961,7 +1969,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2085,7 +2093,7 @@
         <v>46236</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2211,7 +2219,7 @@
         <v>46236</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2337,7 +2345,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2463,7 +2471,7 @@
         <v>46238</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2593,7 +2601,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2723,7 +2731,7 @@
         <v>46233</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2859,7 +2867,7 @@
         <v>46234</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2977,7 +2985,7 @@
         <v>46238</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3095,7 +3103,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3231,7 +3239,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3355,7 +3363,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3493,7 +3501,7 @@
         <v>46240</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3635,7 +3643,7 @@
         <v>46240</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3757,7 +3765,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3889,7 +3897,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4023,7 +4031,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4147,7 +4155,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4273,7 +4281,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4415,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4531,7 +4539,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4657,7 +4665,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4775,7 +4783,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4897,7 +4905,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5019,7 +5027,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5141,7 +5149,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5263,7 +5271,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5385,7 +5393,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5507,7 +5515,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5625,7 +5633,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5767,7 +5775,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5889,7 +5897,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6025,7 +6033,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6157,7 +6165,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6295,7 +6303,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6437,7 +6445,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6567,7 +6575,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6695,7 +6703,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6819,7 +6827,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6953,7 +6961,7 @@
         <v>46230</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -7087,7 +7095,7 @@
         <v>46230</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7541,7 +7549,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7579,7 +7587,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -7677,7 +7689,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7817,7 +7829,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7955,7 +7967,7 @@
         <v>46240</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -8089,7 +8101,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -8217,7 +8229,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8347,7 +8359,7 @@
         <v>46233</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8483,7 +8495,7 @@
         <v>46234</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8619,7 +8631,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8759,7 +8771,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8901,7 +8913,7 @@
         <v>46240</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -9037,7 +9049,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -9171,7 +9183,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9303,7 +9315,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9431,7 +9443,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9569,7 +9581,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9705,7 +9717,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9837,7 +9849,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -9975,7 +9987,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -10117,7 +10129,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -10247,7 +10259,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -10375,7 +10387,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -10499,7 +10511,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -10633,7 +10645,7 @@
         <v>46230</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -10767,7 +10779,7 @@
         <v>46230</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -11173,7 +11185,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11211,7 +11223,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -11295,7 +11311,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11417,7 +11433,7 @@
         <v>46241</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11543,7 +11559,7 @@
         <v>46243</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11673,7 +11689,7 @@
         <v>46243</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11799,7 +11815,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11925,7 +11941,7 @@
         <v>46236</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -12051,7 +12067,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -12177,7 +12193,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -12299,7 +12315,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -12417,7 +12433,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -12539,7 +12555,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -12657,7 +12673,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -12779,7 +12795,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -12905,7 +12921,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -13031,7 +13047,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -13149,7 +13165,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -13271,7 +13287,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -13393,7 +13409,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -13515,7 +13531,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -13637,7 +13653,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -13759,7 +13775,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -13881,7 +13897,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -13999,7 +14015,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -14121,7 +14137,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -14534,7 +14550,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14652,7 +14668,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14770,7 +14786,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14898,7 +14914,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -15022,7 +15038,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -15156,7 +15172,7 @@
         <v>46230</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -15290,7 +15306,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15669,7 +15685,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15787,7 +15803,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15905,7 +15921,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15983,7 +15999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18310,8 +18326,57 @@
         </is>
       </c>
     </row>
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13T13:46:02+08:00</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06 至 2026-08-13</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/hechi/tzgg_15562/tzgg_15563/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /hechi/tzgg_15562/tzgg_15563/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('R...</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M47"/>
+  <autoFilter ref="A1:M48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-14
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日运行日志" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ51"/>
+  <dimension ref="A1:AJ52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -781,7 +781,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         <v>46246</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
         <v>46241</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         <v>46241</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         <v>46240</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1705,7 +1705,7 @@
         <v>46243</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1835,7 +1835,7 @@
         <v>46243</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2093,7 +2093,7 @@
         <v>46236</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
         <v>46236</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         <v>46238</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
         <v>46233</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46234</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         <v>46238</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3103,7 +3103,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3363,7 +3363,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
         <v>46240</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         <v>46240</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3765,7 +3765,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3897,7 +3897,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4031,7 +4031,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4281,7 +4281,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4415,7 +4415,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4539,7 +4539,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4665,7 +4665,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4783,7 +4783,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4905,7 +4905,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5027,7 +5027,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5271,7 +5271,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5393,7 +5393,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5775,7 +5775,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6033,7 +6033,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6165,7 +6165,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6303,7 +6303,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6445,7 +6445,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6575,7 +6575,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6703,7 +6703,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6827,7 +6827,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6869,16 +6869,16 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>CASE-7e3d4a321440d6a7</t>
+          <t>CASE-3996d04fd944424e</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>DOC-bed9330343ed06af</t>
+          <t>DOC-af179599b7f27421</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -6904,12 +6904,12 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>天津展达科技有限公司</t>
+          <t>信硕(天津)国际货运代理有限公司</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>91120116300738701X</t>
+          <t>91120105MA06WEYU7C</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
@@ -6920,48 +6920,38 @@
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
+          <t>津税一稽处〔2022〕270号</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
+          <t>津税一稽处〔2022〕270号</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+          <t>我局(所)于2022年6月24日至2022年8月18日对你(单位)(地址:天津市河北区建昌道街道铁工东里增57-1号)2019年12月2日至2022年5月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位无生产经营地点,虚假注册,无社保信息,与上下游企业无银行交易记录,收取上游企业虚开的增值税发票后脱离税务机关监管,经核实,你单位不符合正常企业构成要件,认定为假企业。 你单位在2019年12月02日-2022年5月31日期间,未发生真实货物、劳务交易,对下游13户企业开具增值税普通发票990份,发票代码012001900105,发票号码04884187-04884216,04893407-04893421,04898548,06548576-06548620,06671887-06671896,06807185-06807194,06909763-06909797,07353556-07353600,07359910-07359954,07369273-07369317,07374190-07374214,07379166-07379235,09307219-09307288,09319483-09319552,09327879-09327948,11915880-11915949,11925651-11925720,11937167-11937236,11941265-11941334,11945987-11946000,11948001-11948056,发票代码012001900104,发票号码24048210-24048219,虚开增值税普通发票不含税金额73000214.83元,税额0元,价税合计73000214.83元。</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R50" s="3" t="n">
-        <v>920146.9399999999</v>
-      </c>
+          <t>增值税、消费税</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="n"/>
       <c r="S50" s="3" t="n"/>
       <c r="T50" s="3" t="n"/>
       <c r="U50" s="3" t="n"/>
-      <c r="V50" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V50" s="2" t="inlineStr"/>
       <c r="W50" s="4" t="n"/>
       <c r="X50" s="4" t="n"/>
       <c r="Y50" s="4" t="n"/>
       <c r="Z50" s="4" t="n">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6987,7 +6977,7 @@
       <c r="AG50" s="2" t="inlineStr"/>
       <c r="AH50" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达信硕(天津)国际货运代理有限公司《税务处理决定书》的公告</t>
         </is>
       </c>
       <c r="AI50" s="2" t="inlineStr">
@@ -6997,13 +6987,13 @@
       </c>
       <c r="AJ50" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -7012,7 +7002,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>DOC-388bd01c01bbb789</t>
+          <t>DOC-bed9330343ed06af</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -7049,24 +7039,24 @@
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
           <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
-      <c r="N51" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O51" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
           <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
@@ -7077,11 +7067,11 @@
           <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
         </is>
       </c>
-      <c r="R51" s="3" t="n"/>
+      <c r="R51" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
       <c r="S51" s="3" t="n"/>
-      <c r="T51" s="3" t="n">
-        <v>131368.5</v>
-      </c>
+      <c r="T51" s="3" t="n"/>
       <c r="U51" s="3" t="n"/>
       <c r="V51" s="2" t="inlineStr">
         <is>
@@ -7095,7 +7085,7 @@
         <v>46230</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7135,20 +7125,154 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="n"/>
+      <c r="S52" s="3" t="n"/>
+      <c r="T52" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U52" s="3" t="n"/>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W52" s="4" t="n"/>
+      <c r="X52" s="4" t="n"/>
+      <c r="Y52" s="4" t="n"/>
+      <c r="Z52" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA52" s="4" t="n">
+        <v>46248</v>
+      </c>
+      <c r="AB52" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC52" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD52" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE52" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF52" s="2" t="inlineStr"/>
+      <c r="AG52" s="2" t="inlineStr"/>
+      <c r="AH52" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI52" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ52" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ51"/>
-  <conditionalFormatting sqref="AD2:AD51">
+  <autoFilter ref="A1:AJ52"/>
+  <conditionalFormatting sqref="AD2:AD52">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI51">
+  <conditionalFormatting sqref="AI2:AI52">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7226,6 +7350,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE49" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE50" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE51" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE52" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -7238,7 +7363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ26"/>
+  <dimension ref="A1:AJ27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7549,7 +7674,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7689,7 +7814,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7829,7 +7954,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -7967,7 +8092,7 @@
         <v>46240</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -8101,7 +8226,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -8229,7 +8354,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8484,7 @@
         <v>46233</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8495,7 +8620,7 @@
         <v>46234</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8631,7 +8756,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8771,7 +8896,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -8913,7 +9038,7 @@
         <v>46240</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -9049,7 +9174,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -9183,7 +9308,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9315,7 +9440,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9443,7 +9568,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9581,7 +9706,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9717,7 +9842,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9849,7 +9974,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -9987,7 +10112,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -10129,7 +10254,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -10259,7 +10384,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -10387,7 +10512,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -10511,7 +10636,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -10553,16 +10678,16 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>CASE-7e3d4a321440d6a7</t>
+          <t>CASE-3996d04fd944424e</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>DOC-bed9330343ed06af</t>
+          <t>DOC-af179599b7f27421</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -10588,12 +10713,12 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>天津展达科技有限公司</t>
+          <t>信硕(天津)国际货运代理有限公司</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>91120116300738701X</t>
+          <t>91120105MA06WEYU7C</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
@@ -10604,48 +10729,38 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
+          <t>津税一稽处〔2022〕270号</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
+          <t>津税一稽处〔2022〕270号</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+          <t>我局(所)于2022年6月24日至2022年8月18日对你(单位)(地址:天津市河北区建昌道街道铁工东里增57-1号)2019年12月2日至2022年5月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位无生产经营地点,虚假注册,无社保信息,与上下游企业无银行交易记录,收取上游企业虚开的增值税发票后脱离税务机关监管,经核实,你单位不符合正常企业构成要件,认定为假企业。 你单位在2019年12月02日-2022年5月31日期间,未发生真实货物、劳务交易,对下游13户企业开具增值税普通发票990份,发票代码012001900105,发票号码04884187-04884216,04893407-04893421,04898548,06548576-06548620,06671887-06671896,06807185-06807194,06909763-06909797,07353556-07353600,07359910-07359954,07369273-07369317,07374190-07374214,07379166-07379235,09307219-09307288,09319483-09319552,09327879-09327948,11915880-11915949,11925651-11925720,11937167-11937236,11941265-11941334,11945987-11946000,11948001-11948056,发票代码012001900104,发票号码24048210-24048219,虚开增值税普通发票不含税金额73000214.83元,税额0元,价税合计73000214.83元。</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R25" s="3" t="n">
-        <v>920146.9399999999</v>
-      </c>
+          <t>增值税、消费税</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="n"/>
       <c r="S25" s="3" t="n"/>
       <c r="T25" s="3" t="n"/>
       <c r="U25" s="3" t="n"/>
-      <c r="V25" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V25" s="2" t="inlineStr"/>
       <c r="W25" s="4" t="n"/>
       <c r="X25" s="4" t="n"/>
       <c r="Y25" s="4" t="n"/>
       <c r="Z25" s="4" t="n">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -10671,7 +10786,7 @@
       <c r="AG25" s="2" t="inlineStr"/>
       <c r="AH25" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达信硕(天津)国际货运代理有限公司《税务处理决定书》的公告</t>
         </is>
       </c>
       <c r="AI25" s="2" t="inlineStr">
@@ -10681,13 +10796,13 @@
       </c>
       <c r="AJ25" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -10696,7 +10811,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>DOC-388bd01c01bbb789</t>
+          <t>DOC-bed9330343ed06af</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -10733,24 +10848,24 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
           <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
           <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
@@ -10761,11 +10876,11 @@
           <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
         </is>
       </c>
-      <c r="R26" s="3" t="n"/>
+      <c r="R26" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
       <c r="S26" s="3" t="n"/>
-      <c r="T26" s="3" t="n">
-        <v>131368.5</v>
-      </c>
+      <c r="T26" s="3" t="n"/>
       <c r="U26" s="3" t="n"/>
       <c r="V26" s="2" t="inlineStr">
         <is>
@@ -10779,7 +10894,7 @@
         <v>46230</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -10819,20 +10934,154 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="n"/>
+      <c r="S27" s="3" t="n"/>
+      <c r="T27" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U27" s="3" t="n"/>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W27" s="4" t="n"/>
+      <c r="X27" s="4" t="n"/>
+      <c r="Y27" s="4" t="n"/>
+      <c r="Z27" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA27" s="4" t="n">
+        <v>46248</v>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD27" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE27" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF27" s="2" t="inlineStr"/>
+      <c r="AG27" s="2" t="inlineStr"/>
+      <c r="AH27" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI27" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ27" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ26"/>
-  <conditionalFormatting sqref="AD2:AD26">
+  <autoFilter ref="A1:AJ27"/>
+  <conditionalFormatting sqref="AD2:AD27">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI26">
+  <conditionalFormatting sqref="AI2:AI27">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10872,6 +11121,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE25" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE27" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -11185,7 +11435,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11311,7 +11561,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11433,7 +11683,7 @@
         <v>46241</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11559,7 +11809,7 @@
         <v>46243</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11689,7 +11939,7 @@
         <v>46243</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -11815,7 +12065,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -11941,7 +12191,7 @@
         <v>46236</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -12067,7 +12317,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -12193,7 +12443,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -12315,7 +12565,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -12433,7 +12683,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -12555,7 +12805,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -12673,7 +12923,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -12795,7 +13045,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -12921,7 +13171,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -13047,7 +13297,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -13165,7 +13415,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -13287,7 +13537,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -13409,7 +13659,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -13531,7 +13781,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -13653,7 +13903,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -13775,7 +14025,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -13897,7 +14147,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -14015,7 +14265,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -14137,7 +14387,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -14249,7 +14499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ8"/>
+  <dimension ref="A1:AJ9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14550,7 +14800,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14668,7 +14918,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14786,7 +15036,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14914,7 +15164,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -15038,7 +15288,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -15080,16 +15330,16 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CASE-7e3d4a321440d6a7</t>
+          <t>CASE-3996d04fd944424e</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>DOC-bed9330343ed06af</t>
+          <t>DOC-af179599b7f27421</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -15115,12 +15365,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>天津展达科技有限公司</t>
+          <t>信硕(天津)国际货运代理有限公司</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>91120116300738701X</t>
+          <t>91120105MA06WEYU7C</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -15131,48 +15381,38 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
+          <t>津税一稽处〔2022〕270号</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
+          <t>津税一稽处〔2022〕270号</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+          <t>我局(所)于2022年6月24日至2022年8月18日对你(单位)(地址:天津市河北区建昌道街道铁工东里增57-1号)2019年12月2日至2022年5月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位无生产经营地点,虚假注册,无社保信息,与上下游企业无银行交易记录,收取上游企业虚开的增值税发票后脱离税务机关监管,经核实,你单位不符合正常企业构成要件,认定为假企业。 你单位在2019年12月02日-2022年5月31日期间,未发生真实货物、劳务交易,对下游13户企业开具增值税普通发票990份,发票代码012001900105,发票号码04884187-04884216,04893407-04893421,04898548,06548576-06548620,06671887-06671896,06807185-06807194,06909763-06909797,07353556-07353600,07359910-07359954,07369273-07369317,07374190-07374214,07379166-07379235,09307219-09307288,09319483-09319552,09327879-09327948,11915880-11915949,11925651-11925720,11937167-11937236,11941265-11941334,11945987-11946000,11948001-11948056,发票代码012001900104,发票号码24048210-24048219,虚开增值税普通发票不含税金额73000214.83元,税额0元,价税合计73000214.83元。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="n">
-        <v>920146.9399999999</v>
-      </c>
+          <t>增值税、消费税</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="n"/>
       <c r="S7" s="3" t="n"/>
       <c r="T7" s="3" t="n"/>
       <c r="U7" s="3" t="n"/>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V7" s="2" t="inlineStr"/>
       <c r="W7" s="4" t="n"/>
       <c r="X7" s="4" t="n"/>
       <c r="Y7" s="4" t="n"/>
       <c r="Z7" s="4" t="n">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -15198,7 +15438,7 @@
       <c r="AG7" s="2" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达信硕(天津)国际货运代理有限公司《税务处理决定书》的公告</t>
         </is>
       </c>
       <c r="AI7" s="2" t="inlineStr">
@@ -15208,13 +15448,13 @@
       </c>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面未提取到可确认的官方发布日期。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -15223,7 +15463,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DOC-388bd01c01bbb789</t>
+          <t>DOC-bed9330343ed06af</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -15260,24 +15500,24 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
           <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
           <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
@@ -15288,11 +15528,11 @@
           <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
         </is>
       </c>
-      <c r="R8" s="3" t="n"/>
+      <c r="R8" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
       <c r="S8" s="3" t="n"/>
-      <c r="T8" s="3" t="n">
-        <v>131368.5</v>
-      </c>
+      <c r="T8" s="3" t="n"/>
       <c r="U8" s="3" t="n"/>
       <c r="V8" s="2" t="inlineStr">
         <is>
@@ -15306,7 +15546,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15346,20 +15586,154 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="n"/>
+      <c r="S9" s="3" t="n"/>
+      <c r="T9" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U9" s="3" t="n"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="n"/>
+      <c r="X9" s="4" t="n"/>
+      <c r="Y9" s="4" t="n"/>
+      <c r="Z9" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA9" s="4" t="n">
+        <v>46248</v>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD9" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE9" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF9" s="2" t="inlineStr"/>
+      <c r="AG9" s="2" t="inlineStr"/>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI9" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ8"/>
-  <conditionalFormatting sqref="AD2:AD8">
+  <autoFilter ref="A1:AJ9"/>
+  <conditionalFormatting sqref="AD2:AD9">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI8">
+  <conditionalFormatting sqref="AI2:AI9">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15372,6 +15746,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE6" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE7" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE9" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -15685,7 +16060,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15803,7 +16178,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15921,7 +16296,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15999,7 +16374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18424,8 +18799,61 @@
         </is>
       </c>
     </row>
+    <row r="50" ht="54" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14T13:43:30+08:00</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 至 2026-08-14</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>193</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>信硕(天津)国际货运代理有限公司</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>已完成候选发现、逐条访问核验、去重、关联和历史数据增量写入。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M49"/>
+  <autoFilter ref="A1:M50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-15
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         <v>46246</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
         <v>46241</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         <v>46241</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         <v>46240</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1705,7 +1705,7 @@
         <v>46243</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1835,7 +1835,7 @@
         <v>46243</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2093,7 +2093,7 @@
         <v>46236</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
         <v>46236</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         <v>46238</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
         <v>46233</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46234</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         <v>46238</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3103,7 +3103,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3363,7 +3363,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
         <v>46240</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         <v>46240</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3765,7 +3765,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3897,7 +3897,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4031,7 +4031,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4281,7 +4281,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4415,7 +4415,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4539,7 +4539,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4665,7 +4665,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4783,7 +4783,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4905,7 +4905,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5027,7 +5027,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5271,7 +5271,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5393,7 +5393,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5775,7 +5775,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6033,7 +6033,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6165,7 +6165,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6303,7 +6303,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6445,7 +6445,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6575,7 +6575,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6703,7 +6703,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6827,7 +6827,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v>46248</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -7085,7 +7085,7 @@
         <v>46230</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7219,7 +7219,7 @@
         <v>46230</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7674,7 +7674,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -7814,7 +7814,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -7954,7 +7954,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -8092,7 +8092,7 @@
         <v>46240</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -8354,7 +8354,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -8484,7 +8484,7 @@
         <v>46233</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -8620,7 +8620,7 @@
         <v>46234</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -8756,7 +8756,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -8896,7 +8896,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -9038,7 +9038,7 @@
         <v>46240</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -9174,7 +9174,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -9308,7 +9308,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -9440,7 +9440,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -9568,7 +9568,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -9706,7 +9706,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -9842,7 +9842,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -9974,7 +9974,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -10112,7 +10112,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -10254,7 +10254,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -10384,7 +10384,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -10512,7 +10512,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -10760,7 +10760,7 @@
         <v>46248</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -10894,7 +10894,7 @@
         <v>46230</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -11028,7 +11028,7 @@
         <v>46230</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -11435,7 +11435,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -11561,7 +11561,7 @@
         <v>46241</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -11683,7 +11683,7 @@
         <v>46241</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -11809,7 +11809,7 @@
         <v>46243</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -11939,7 +11939,7 @@
         <v>46243</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -12065,7 +12065,7 @@
         <v>46236</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -12191,7 +12191,7 @@
         <v>46236</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -12317,7 +12317,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -12443,7 +12443,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -12565,7 +12565,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -12683,7 +12683,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -12805,7 +12805,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -12923,7 +12923,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -13045,7 +13045,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -13171,7 +13171,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -13297,7 +13297,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -13415,7 +13415,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -13537,7 +13537,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -13659,7 +13659,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -13781,7 +13781,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -13903,7 +13903,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -14025,7 +14025,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -14147,7 +14147,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -14265,7 +14265,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -14387,7 +14387,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -14800,7 +14800,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14918,7 +14918,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15036,7 +15036,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15164,7 +15164,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -15288,7 +15288,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -15546,7 +15546,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15680,7 +15680,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -16060,7 +16060,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -16178,7 +16178,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -16296,7 +16296,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -16374,7 +16374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18901,8 +18901,57 @@
         </is>
       </c>
     </row>
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15T12:42:16+08:00</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08 至 2026-08-15</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M51"/>
+  <autoFilter ref="A1:M52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-16
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -895,7 +895,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
         <v>46246</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1649,7 +1649,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         <v>46249</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         <v>46242</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2169,7 +2169,7 @@
         <v>46242</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2295,7 +2295,7 @@
         <v>46241</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         <v>46241</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         <v>46240</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>46243</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2811,7 +2811,7 @@
         <v>46243</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2933,7 +2933,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3063,7 +3063,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3301,7 +3301,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
         <v>46236</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3549,7 +3549,7 @@
         <v>46236</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3675,7 +3675,7 @@
         <v>46238</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3801,7 +3801,7 @@
         <v>46238</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3931,7 +3931,7 @@
         <v>46238</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4061,7 +4061,7 @@
         <v>46233</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4197,7 +4197,7 @@
         <v>46234</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4315,7 +4315,7 @@
         <v>46238</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4433,7 +4433,7 @@
         <v>46238</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4569,7 +4569,7 @@
         <v>46238</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4693,7 +4693,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v>46240</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
         <v>46240</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5231,7 +5231,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5615,7 +5615,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5749,7 +5749,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5887,7 +5887,7 @@
         <v>46249</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6015,7 +6015,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6141,7 +6141,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6259,7 +6259,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6381,7 +6381,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6503,7 +6503,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6625,7 +6625,7 @@
         <v>46249</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6755,7 +6755,7 @@
         <v>46249</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6877,7 +6877,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6999,7 +6999,7 @@
         <v>46229</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7121,7 +7121,7 @@
         <v>46229</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7243,7 +7243,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7361,7 +7361,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7503,7 +7503,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
         <v>46229</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7761,7 +7761,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7893,7 +7893,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8173,7 +8173,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8303,7 +8303,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8431,7 +8431,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8555,7 +8555,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8679,7 +8679,7 @@
         <v>46248</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8813,7 +8813,7 @@
         <v>46230</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8947,7 +8947,7 @@
         <v>46230</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9426,7 +9426,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9566,7 +9566,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -9706,7 +9706,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -9844,7 +9844,7 @@
         <v>46240</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -9978,7 +9978,7 @@
         <v>46238</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10106,7 +10106,7 @@
         <v>46238</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10236,7 +10236,7 @@
         <v>46233</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10372,7 +10372,7 @@
         <v>46234</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10508,7 +10508,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -10648,7 +10648,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -10790,7 +10790,7 @@
         <v>46240</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -10930,7 +10930,7 @@
         <v>46229</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11064,7 +11064,7 @@
         <v>46229</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -11196,7 +11196,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -11334,7 +11334,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -11466,7 +11466,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -11592,7 +11592,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -11730,7 +11730,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -11866,7 +11866,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -11998,7 +11998,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -12136,7 +12136,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -12278,7 +12278,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -12408,7 +12408,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -12536,7 +12536,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -12660,7 +12660,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -12784,7 +12784,7 @@
         <v>46248</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -12918,7 +12918,7 @@
         <v>46230</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -13052,7 +13052,7 @@
         <v>46230</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -13462,7 +13462,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -13576,7 +13576,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -13694,7 +13694,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -13816,7 +13816,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -13942,7 +13942,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14194,7 +14194,7 @@
         <v>46249</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -14320,7 +14320,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -14438,7 +14438,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -14560,7 +14560,7 @@
         <v>46241</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -14682,7 +14682,7 @@
         <v>46241</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -14808,7 +14808,7 @@
         <v>46243</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -14938,7 +14938,7 @@
         <v>46243</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -15060,7 +15060,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -15178,7 +15178,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -15296,7 +15296,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -15418,7 +15418,7 @@
         <v>46236</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -15544,7 +15544,7 @@
         <v>46236</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -15670,7 +15670,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -15796,7 +15796,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -15918,7 +15918,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -16036,7 +16036,7 @@
         <v>46238</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -16276,7 +16276,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -16398,7 +16398,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -16524,7 +16524,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -16650,7 +16650,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -16768,7 +16768,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -16890,7 +16890,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -17012,7 +17012,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -17134,7 +17134,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -17260,7 +17260,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -17382,7 +17382,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -17504,7 +17504,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -17626,7 +17626,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -17744,7 +17744,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -17866,7 +17866,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -18296,7 +18296,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -18414,7 +18414,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -18532,7 +18532,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -18660,7 +18660,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -18784,7 +18784,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -18908,7 +18908,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -19042,7 +19042,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -19176,7 +19176,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -19556,7 +19556,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -19674,7 +19674,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -19792,7 +19792,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -19870,7 +19870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22597,8 +22597,57 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16T12:46:16+08:00</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09 至 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M55"/>
+  <autoFilter ref="A1:M56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: verify August 14-16 tax decisions
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日运行日志" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'文书汇总'!$A$1:$AJ$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'完整文书'!$A$1:$AJ$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ68"/>
+  <dimension ref="A1:AJ69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1476,11 +1476,7 @@
           <t>91450181MACQW4NT1E</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>或者股东的个人账户</t>
-        </is>
-      </c>
+      <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>税务处理决定书</t>
@@ -1970,7 +1966,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>同时,该地址也是广西槟咪科技有限公司</t>
+          <t>广西苒炙机械设备有限公司</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -2013,11 +2009,7 @@
       <c r="S12" s="3" t="n"/>
       <c r="T12" s="3" t="n"/>
       <c r="U12" s="3" t="n"/>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V12" s="2" t="inlineStr"/>
       <c r="W12" s="4" t="n">
         <v>46157</v>
       </c>
@@ -2069,7 +2061,7 @@
       </c>
       <c r="AJ12" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”存在冲突:保留原值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处理决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”,新值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处罚决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”历史冲突已由官方附件复核,保留当前值。 当事人名称经官方原文复核,由“同时,该地址也是广西槟咪科技有限公司”更正为“广西苒炙机械设备有限公司”。 字段“处理或处罚结果”历史冲突已由官方附件复核,保留当前值。 处理文书中的处罚结果串值已根据官方附件清除。</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2089,11 @@
           <t>河池市</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>金城江区</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>国家税务总局河池市税务局第二稽查局</t>
@@ -2110,7 +2106,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>同时,该地址也是广西槟咪科技有限公司</t>
+          <t>广西苒炙机械设备有限公司</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -2141,7 +2137,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处理决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。</t>
+          <t>经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处罚决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -2151,11 +2147,13 @@
       </c>
       <c r="R13" s="3" t="n"/>
       <c r="S13" s="3" t="n"/>
-      <c r="T13" s="3" t="n"/>
+      <c r="T13" s="3" t="n">
+        <v>200000</v>
+      </c>
       <c r="U13" s="3" t="n"/>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。</t>
+          <t>同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W13" s="4" t="n">
@@ -2209,7 +2207,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”存在冲突:保留原值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处理决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”,新值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处罚决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 当事人名称经官方原文复核,由“同时,该地址也是广西槟咪科技有限公司”更正为“广西苒炙机械设备有限公司”。 字段“主要违法事实”已根据官方附件重新解析。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -2258,11 +2256,7 @@
           <t>91370220MA9490X30G</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>或委托代理人持单位公章等</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>税务处理决定书</t>
@@ -2297,11 +2291,7 @@
       <c r="S14" s="3" t="n"/>
       <c r="T14" s="3" t="n"/>
       <c r="U14" s="3" t="n"/>
-      <c r="V14" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国税收征收管理法实施细则》第一百零六条第(二)款之规定,因采用其他方式无法向你单位送达税务文书,我局决定对《税务行政处罚决定书》(青税稽一罚〔2026〕65号)、《税务处理决定书》(青税稽一处〔2026〕73号)予以公告送达。 根据《中华人民共和国发票管理办法》(国函〔1993〕174号,2019年3月2日《国务院关于修改部分行政法规的决定》(中华人民共和国国务院令第709号)第二次修改)第三十七条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 构成犯罪的,依法追究刑事责任”、参照《国家税务总局关于发布&lt;税务行政处罚裁量权行使规则&gt;的公告》(国家税务总局公告2016年第78号)的规定,对你公司虚开发票行为处以罚款140000.00元。 ”、《中华人民共和国税收征收管理法实施细则》第九十六条“纳税人、扣缴义务人有下列情形之一的,依照税收征管法第七十条的规定处罚,(一)提供虚假材料,不如实反映情况,或者拒绝提供有关资料的”的规定,你单位经责令限期改正,至检查结束,拒不提供有关纳税资料,对你公司处以罚款20000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V14" s="2" t="inlineStr"/>
       <c r="W14" s="4" t="n"/>
       <c r="X14" s="4" t="n">
         <v>46240</v>
@@ -2345,7 +2335,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。 处理文书中的处罚结果串值已根据官方附件清除。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -2392,11 +2386,7 @@
           <t>91370220MA9490X30G</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>或委托代理人持单位公章等</t>
-        </is>
-      </c>
+      <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>税务行政处罚决定书</t>
@@ -2481,7 +2471,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ15" s="2" t="inlineStr"/>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -5071,7 +5065,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>查属期内违法行为均定性偷税, 需要对原处罚决定中的罚款数额 以变更,你(单位)存在违法事实及处罚决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 〔2022〕59号) 第一条、 第三条之规定, 你单位存在少缴属期2010 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 报,不缴或者少缴应纳税款的,是偷税。 务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴 内首次因偷税被税务机关处罚,并能够配合税务机关检查的,处 不缴或者少缴的税款百分之五十的罚款”之规定,对你单位城镇 土地使用税和印花税处不缴或者少缴的税款50%的罚款。 你单位印花税偷税违法行为发生于2009年11月26日,至立案 位检查属期内违法行为均定性偷税, 需要对原处理决定中的查补 情况进行了检查,违法事实及处理决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 定, 你单位存在少缴属期2010年1月至2022年6月城镇土地使 用税5,710,765.50元的违法事实。 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 该地块未缴纳契税,你单位存在少缴契税509,984.64元的违法 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。</t>
+          <t>位检查属期内违法行为均定性偷税, 需要对原处理决定中的查补 情况进行了检查,违法事实及处理决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 定, 你单位存在少缴属期2010年1月至2022年6月城镇土地使 用税5,710,765.50元的违法事实。 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 该地块未缴纳契税,你单位存在少缴契税509,984.64元的违法 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 单位未申报2010年1月1日至2022年6月30日契税。 6月申报数据,用于证明你单位未申报缴纳契税。</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
@@ -5087,7 +5081,7 @@
       <c r="U36" s="3" t="n"/>
       <c r="V36" s="2" t="inlineStr">
         <is>
-          <t>定,每日按罚款数额的百分之三加处罚款。 日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税 日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税</t>
+          <t>日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税</t>
         </is>
       </c>
       <c r="W36" s="4" t="n">
@@ -5141,7 +5135,7 @@
       </c>
       <c r="AJ36" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”已根据官方附件重新解析。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5207,7 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>查属期内违法行为均定性偷税, 需要对原处罚决定中的罚款数额 以变更,你(单位)存在违法事实及处罚决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 〔2022〕59号) 第一条、 第三条之规定, 你单位存在少缴属期2010 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 报,不缴或者少缴应纳税款的,是偷税。 务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴 内首次因偷税被税务机关处罚,并能够配合税务机关检查的,处 不缴或者少缴的税款百分之五十的罚款”之规定,对你单位城镇 土地使用税和印花税处不缴或者少缴的税款50%的罚款。 你单位印花税偷税违法行为发生于2009年11月26日,至立案 位检查属期内违法行为均定性偷税, 需要对原处理决定中的查补 情况进行了检查,违法事实及处理决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 定, 你单位存在少缴属期2010年1月至2022年6月城镇土地使 用税5,710,765.50元的违法事实。 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 该地块未缴纳契税,你单位存在少缴契税509,984.64元的违法 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。</t>
+          <t>查属期内违法行为均定性偷税, 需要对原处罚决定中的罚款数额 以变更,你(单位)存在违法事实及处罚决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 〔2022〕59号) 第一条、 第三条之规定, 你单位存在少缴属期2010 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 报,不缴或者少缴应纳税款的,是偷税。 务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴 内首次因偷税被税务机关处罚,并能够配合税务机关检查的,处 不缴或者少缴的税款百分之五十的罚款”之规定,对你单位城镇 土地使用税和印花税处不缴或者少缴的税款50%的罚款。 你单位印花税偷税违法行为发生于2009年11月26日,至立案</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
@@ -5229,7 +5223,7 @@
       <c r="U37" s="3" t="n"/>
       <c r="V37" s="2" t="inlineStr">
         <is>
-          <t>定,每日按罚款数额的百分之三加处罚款。 日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税 定,每日按罚款数额的百分之三加处罚款。</t>
+          <t>定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W37" s="4" t="n">
@@ -5283,7 +5277,7 @@
       </c>
       <c r="AJ37" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”已根据官方附件重新解析。 字段“涉及税种”存在冲突:保留原值“增值税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、契税、教育费附加、地方教育附加”,新值“房产税、城镇土地使用税、印花税”未静默覆盖。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -7555,66 +7549,66 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CASE-393a878d93a22709</t>
+          <t>CASE-eb7e9c22bd97f211</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>DOC-cda8cba853896b18</t>
+          <t>DOC-4c99e9a228472ee1</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>广东省</t>
+          <t>江苏省</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>广州市</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>番禺区</t>
-        </is>
-      </c>
+          <t>无锡市</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局广州市番禺区税务局</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr"/>
+          <t>国家税务总局无锡市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局无锡市税务局第一稽查局</t>
+        </is>
+      </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>广州赞荣服装有限公司</t>
+          <t>宜兴市华欧金属材料有限公司</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>91440113MA59AJFJ1J</t>
+          <t>91320282MA1MMJ8YXD</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="N56" s="2" t="inlineStr"/>
-      <c r="O56" s="2" t="inlineStr">
-        <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
+          <t>锡税一稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>锡税一稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr"/>
       <c r="P56" s="2" t="inlineStr"/>
       <c r="Q56" s="2" t="inlineStr"/>
       <c r="R56" s="3" t="n"/>
@@ -7624,11 +7618,11 @@
       <c r="V56" s="2" t="inlineStr"/>
       <c r="W56" s="4" t="n"/>
       <c r="X56" s="4" t="n">
-        <v>46091</v>
+        <v>46111</v>
       </c>
       <c r="Y56" s="4" t="n"/>
       <c r="Z56" s="4" t="n">
-        <v>46229</v>
+        <v>46250</v>
       </c>
       <c r="AA56" s="4" t="n">
         <v>46250</v>
@@ -7645,7 +7639,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE56" s="5" t="inlineStr">
@@ -7653,120 +7647,96 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF56" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF56" s="2" t="inlineStr"/>
       <c r="AG56" s="2" t="inlineStr"/>
       <c r="AH56" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
+          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局无锡市税务局第一稽查局关于送达《税务处理决定书》的公告(宜兴市华欧金属材料有限公司)</t>
         </is>
       </c>
       <c r="AI56" s="2" t="inlineStr">
         <is>
-          <t>内容不匹配</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ56" s="2" t="inlineStr">
         <is>
-          <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>CASE-f94bf08964abff5a</t>
+          <t>CASE-393a878d93a22709</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>DOC-4574b1aadef8f30d</t>
+          <t>DOC-cda8cba853896b18</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>江苏省</t>
+          <t>广东省</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>常州市</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
+          <t>广州市</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>番禺区</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局江苏省税务局</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局常州市税务局稽查局</t>
-        </is>
-      </c>
+          <t>国家税务总局广州市番禺区税务局</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>常州市文杰车辆配件厂</t>
+          <t>广州赞荣服装有限公司</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>91320411799075280A</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>朱某</t>
-        </is>
-      </c>
+          <t>91440113MA59AJFJ1J</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>常税稽处〔2026〕73号</t>
-        </is>
-      </c>
-      <c r="N57" s="2" t="inlineStr">
-        <is>
-          <t>常税稽处〔2026〕73号</t>
-        </is>
-      </c>
-      <c r="O57" s="2" t="inlineStr"/>
-      <c r="P57" s="2" t="inlineStr">
-        <is>
-          <t>月1日至2025年7月15日涉税情况进行了检查, 违法事实及处 述发票已被常州市税务局第一稽查局定性为虚开。 资金往来时,亦与严某个人账户存在交易,虚开团伙利用严某个 人账户提前向你单位垫付虚开资金, 你单位后通过对公账户向虚 簿上虚列进项税额及虚列支出,达到少缴税款的目的。 家税务总局关于纳税人虚开增值税专用发票征补税款问题的公 月1日至2025年7月15日涉税情况进行了检查, 违法事实及处 述发票已被常州市税务局第一稽查局定性为虚开。 资金往来时,亦与严某个人账户存在交易,虚开团伙利用严某个 人账户提前向你单位垫付虚开资金, 你单位后通过对公账户向虚 簿上虚列进项税额及虚列支出,达到少缴税款的目的。 家税务总局关于纳税人虚开增值税专用发票征补税款问题的公</t>
-        </is>
-      </c>
-      <c r="Q57" s="2" t="inlineStr">
-        <is>
-          <t>增值税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R57" s="3" t="n">
-        <v>179137.12</v>
-      </c>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr"/>
+      <c r="Q57" s="2" t="inlineStr"/>
+      <c r="R57" s="3" t="n"/>
       <c r="S57" s="3" t="n"/>
       <c r="T57" s="3" t="n"/>
       <c r="U57" s="3" t="n"/>
-      <c r="V57" s="2" t="inlineStr">
-        <is>
-          <t>份,需要补缴2017年9月增值税16211.46元,城市维护建设税 需要补缴增值税22261.06元,城市维护建设税1558.27元,教 需要补缴增值税36353.98元,城市维护建设税2544.78元,教 需要补缴增值税24057.63元,城市维护建设税1684.03元,教 需要补缴增值税19468.89元,城市维护建设税1362.82元,教 需要补缴增值税21794.95元,城市维护建设税1525.65元,教 需要补缴增值税32586.07元,城市维护建设税2281.02元,教 金额,需要补缴增值税644.16元,城市维护建设税45.09元, 金额,需要补缴增值税30.21元,城市维护建设税2.11元,教 金额,需要补缴增值税1264.25元,城市维护建设税88.5元, 金额,需要补缴增值税4464.46元,城市维护建设税312.51元, 合计需补缴增值税179137.12元, 城市维护建设税12539.58 本次检查决定追缴少申报缴纳的增值税179137.12元、 城市 份,需要补缴2017年9月增值税16211.46元,城市维护建设税 需要补缴增值税22261.06元,城市维护建设税1558.27元,教 需要补缴增值税36353.98元,城市维护建设税2544.78元,教 需要补缴增值税24057.63元,城市维护建设税1684.03元,教 需要补缴增值税19468.89元,城市维护建设税1362.82元,教 需要补缴增值税21794.95元,城市维护建设税1525.65元,教 需要补缴增值税32586.07元,城市维护建设税2281.02元,教 金额,需要补缴增值税644.16元,城市维护建设税45.09元,</t>
-        </is>
-      </c>
-      <c r="W57" s="4" t="n">
-        <v>46044</v>
-      </c>
+      <c r="V57" s="2" t="inlineStr"/>
+      <c r="W57" s="4" t="n"/>
       <c r="X57" s="4" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="Y57" s="4" t="n"/>
       <c r="Z57" s="4" t="n">
@@ -7777,7 +7747,7 @@
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
-          <t>完整文书</t>
+          <t>仅公告送达/仅文号线索</t>
         </is>
       </c>
       <c r="AC57" s="2" t="inlineStr">
@@ -7787,7 +7757,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>已核验</t>
+          <t>待核验</t>
         </is>
       </c>
       <c r="AE57" s="5" t="inlineStr">
@@ -7803,32 +7773,32 @@
       <c r="AG57" s="2" t="inlineStr"/>
       <c r="AH57" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局稽查局关于送达常州市文杰车辆配件厂《税务处理决定书》的公告</t>
+          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
         </is>
       </c>
       <c r="AI57" s="2" t="inlineStr">
         <is>
-          <t>附件正常</t>
+          <t>内容不匹配</t>
         </is>
       </c>
       <c r="AJ57" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CASE-0b4a4519ba4f5ad9</t>
+          <t>CASE-f94bf08964abff5a</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>DOC-5376b9bae81cfc82</t>
+          <t>DOC-4574b1aadef8f30d</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -7854,15 +7824,19 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>常州好佳车辆配件有限公司</t>
+          <t>常州市文杰车辆配件厂</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>91320411094264460B</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
+          <t>91320411799075280A</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>朱某</t>
+        </is>
+      </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
           <t>税务处理决定书</t>
@@ -7870,25 +7844,41 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>常税稽处〔2026〕71号</t>
+          <t>常税稽处〔2026〕73号</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>常税稽处〔2026〕71号</t>
+          <t>常税稽处〔2026〕73号</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr"/>
-      <c r="P58" s="2" t="inlineStr"/>
-      <c r="Q58" s="2" t="inlineStr"/>
-      <c r="R58" s="3" t="n"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>月1日至2025年7月15日涉税情况进行了检查, 违法事实及处 述发票已被常州市税务局第一稽查局定性为虚开。 资金往来时,亦与严某个人账户存在交易,虚开团伙利用严某个 人账户提前向你单位垫付虚开资金, 你单位后通过对公账户向虚 簿上虚列进项税额及虚列支出,达到少缴税款的目的。 家税务总局关于纳税人虚开增值税专用发票征补税款问题的公 月1日至2025年7月15日涉税情况进行了检查, 违法事实及处 述发票已被常州市税务局第一稽查局定性为虚开。 资金往来时,亦与严某个人账户存在交易,虚开团伙利用严某个 人账户提前向你单位垫付虚开资金, 你单位后通过对公账户向虚 簿上虚列进项税额及虚列支出,达到少缴税款的目的。 家税务总局关于纳税人虚开增值税专用发票征补税款问题的公</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>增值税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="n">
+        <v>179137.12</v>
+      </c>
       <c r="S58" s="3" t="n"/>
       <c r="T58" s="3" t="n"/>
       <c r="U58" s="3" t="n"/>
-      <c r="V58" s="2" t="inlineStr"/>
-      <c r="W58" s="4" t="n"/>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>份,需要补缴2017年9月增值税16211.46元,城市维护建设税 需要补缴增值税22261.06元,城市维护建设税1558.27元,教 需要补缴增值税36353.98元,城市维护建设税2544.78元,教 需要补缴增值税24057.63元,城市维护建设税1684.03元,教 需要补缴增值税19468.89元,城市维护建设税1362.82元,教 需要补缴增值税21794.95元,城市维护建设税1525.65元,教 需要补缴增值税32586.07元,城市维护建设税2281.02元,教 金额,需要补缴增值税644.16元,城市维护建设税45.09元, 金额,需要补缴增值税30.21元,城市维护建设税2.11元,教 金额,需要补缴增值税1264.25元,城市维护建设税88.5元, 金额,需要补缴增值税4464.46元,城市维护建设税312.51元, 合计需补缴增值税179137.12元, 城市维护建设税12539.58 本次检查决定追缴少申报缴纳的增值税179137.12元、 城市 份,需要补缴2017年9月增值税16211.46元,城市维护建设税 需要补缴增值税22261.06元,城市维护建设税1558.27元,教 需要补缴增值税36353.98元,城市维护建设税2544.78元,教 需要补缴增值税24057.63元,城市维护建设税1684.03元,教 需要补缴增值税19468.89元,城市维护建设税1362.82元,教 需要补缴增值税21794.95元,城市维护建设税1525.65元,教 需要补缴增值税32586.07元,城市维护建设税2281.02元,教 金额,需要补缴增值税644.16元,城市维护建设税45.09元,</t>
+        </is>
+      </c>
+      <c r="W58" s="4" t="n">
+        <v>46044</v>
+      </c>
       <c r="X58" s="4" t="n">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="Y58" s="4" t="n"/>
       <c r="Z58" s="4" t="n">
@@ -7899,7 +7889,7 @@
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
-          <t>仅公告送达/仅文号线索</t>
+          <t>完整文书</t>
         </is>
       </c>
       <c r="AC58" s="2" t="inlineStr">
@@ -7925,7 +7915,7 @@
       <c r="AG58" s="2" t="inlineStr"/>
       <c r="AH58" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局稽查局关于送达常州好佳车辆配件有限公司《税务处理决定书》的公告</t>
+          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局稽查局关于送达常州市文杰车辆配件厂《税务处理决定书》的公告</t>
         </is>
       </c>
       <c r="AI58" s="2" t="inlineStr">
@@ -7941,16 +7931,16 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>CASE-61b9b55a9d3357c7</t>
+          <t>CASE-0b4a4519ba4f5ad9</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>DOC-1228a9c92b2b0632</t>
+          <t>DOC-5376b9bae81cfc82</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -7966,22 +7956,22 @@
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局常州市税务局第一稽查局</t>
+          <t>国家税务总局江苏省税务局</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局常州市税务局第一稽查局</t>
+          <t>国家税务总局常州市税务局稽查局</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>常州市三鹏机械有限公司</t>
+          <t>常州好佳车辆配件有限公司</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>91320404732260748Q</t>
+          <t>91320411094264460B</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -7992,39 +7982,25 @@
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>常税稽一处〔2026〕35号</t>
+          <t>常税稽处〔2026〕71号</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>常税稽一处〔2026〕35号</t>
-        </is>
-      </c>
-      <c r="O59" s="2" t="inlineStr">
-        <is>
-          <t>常税稽一罚〔2026〕14号</t>
-        </is>
-      </c>
+          <t>常税稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr"/>
       <c r="P59" s="2" t="inlineStr"/>
-      <c r="Q59" s="2" t="inlineStr">
-        <is>
-          <t>增值税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="n">
-        <v>63464.09</v>
-      </c>
+      <c r="Q59" s="2" t="inlineStr"/>
+      <c r="R59" s="3" t="n"/>
       <c r="S59" s="3" t="n"/>
       <c r="T59" s="3" t="n"/>
       <c r="U59" s="3" t="n"/>
-      <c r="V59" s="2" t="inlineStr">
-        <is>
-          <t>根据《税务处理决定书》(常税稽一处〔2026〕35号)应追缴你单位增值税56664.36元、城市维护建设税3966.51元、教育费附加1699.93元、地方教育附加1133.29元; 根据《税务行政处罚决定书》(常税稽一罚〔2026〕14号)应对你单位处罚款20000元。</t>
-        </is>
-      </c>
+      <c r="V59" s="2" t="inlineStr"/>
       <c r="W59" s="4" t="n"/>
       <c r="X59" s="4" t="n">
-        <v>46066</v>
+        <v>46087</v>
       </c>
       <c r="Y59" s="4" t="n"/>
       <c r="Z59" s="4" t="n">
@@ -8035,7 +8011,7 @@
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
-          <t>完整文书</t>
+          <t>仅公告送达/仅文号线索</t>
         </is>
       </c>
       <c r="AC59" s="2" t="inlineStr">
@@ -8053,16 +8029,20 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF59" s="2" t="inlineStr"/>
+      <c r="AF59" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
       <c r="AG59" s="2" t="inlineStr"/>
       <c r="AH59" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局第一稽查局关于送达常州市三鹏机械有限公司《税务处理决定书》和《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局稽查局关于送达常州好佳车辆配件有限公司《税务处理决定书》的公告</t>
         </is>
       </c>
       <c r="AI59" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>附件正常</t>
         </is>
       </c>
       <c r="AJ59" s="2" t="inlineStr">
@@ -8073,7 +8053,7 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
@@ -8082,7 +8062,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>DOC-b97456a64b153f67</t>
+          <t>DOC-1228a9c92b2b0632</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -8119,12 +8099,12 @@
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>常税稽一罚〔2026〕14号</t>
+          <t>常税稽一处〔2026〕35号</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -8143,11 +8123,11 @@
           <t>增值税、城市维护建设税、教育费附加、地方教育附加</t>
         </is>
       </c>
-      <c r="R60" s="3" t="n"/>
+      <c r="R60" s="3" t="n">
+        <v>63464.09</v>
+      </c>
       <c r="S60" s="3" t="n"/>
-      <c r="T60" s="3" t="n">
-        <v>20000</v>
-      </c>
+      <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="n"/>
       <c r="V60" s="2" t="inlineStr">
         <is>
@@ -8205,96 +8185,90 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>CASE-f78ec1a594442165</t>
+          <t>CASE-61b9b55a9d3357c7</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>DOC-fbbe4a664b14f54b</t>
+          <t>DOC-b97456a64b153f67</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>贵州省</t>
+          <t>江苏省</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>安顺市</t>
+          <t>常州市</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局</t>
+          <t>国家税务总局常州市税务局第一稽查局</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局</t>
+          <t>国家税务总局常州市税务局第一稽查局</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
+          <t>常州市三鹏机械有限公司</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>91520423MA6DLH799Q</t>
+          <t>91320404732260748Q</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
+          <t>常税稽一罚〔2026〕14号</t>
         </is>
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>安市税稽处〔2026〕1号</t>
+          <t>常税稽一处〔2026〕35号</t>
         </is>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>安市税稽罚〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="P61" s="2" t="inlineStr">
-        <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
-        </is>
-      </c>
+          <t>常税稽一罚〔2026〕14号</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr"/>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R61" s="3" t="n">
-        <v>64884.41</v>
-      </c>
+          <t>增值税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="n"/>
       <c r="S61" s="3" t="n"/>
-      <c r="T61" s="3" t="n"/>
+      <c r="T61" s="3" t="n">
+        <v>20000</v>
+      </c>
       <c r="U61" s="3" t="n"/>
       <c r="V61" s="2" t="inlineStr">
         <is>
-          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
-        </is>
-      </c>
-      <c r="W61" s="4" t="n">
-        <v>45898</v>
-      </c>
+          <t>根据《税务处理决定书》(常税稽一处〔2026〕35号)应追缴你单位增值税56664.36元、城市维护建设税3966.51元、教育费附加1699.93元、地方教育附加1133.29元; 根据《税务行政处罚决定书》(常税稽一罚〔2026〕14号)应对你单位处罚款20000元。</t>
+        </is>
+      </c>
+      <c r="W61" s="4" t="n"/>
       <c r="X61" s="4" t="n">
-        <v>46043</v>
+        <v>46066</v>
       </c>
       <c r="Y61" s="4" t="n"/>
       <c r="Z61" s="4" t="n">
@@ -8323,31 +8297,27 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF61" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF61" s="2" t="inlineStr"/>
       <c r="AG61" s="2" t="inlineStr"/>
       <c r="AH61" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局第一稽查局关于送达常州市三鹏机械有限公司《税务处理决定书》和《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI61" s="2" t="inlineStr">
         <is>
-          <t>附件正常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ61" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。 字段“主要违法事实”存在冲突:保留原值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”,新值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
@@ -8356,7 +8326,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>DOC-9a828a6048b54b6c</t>
+          <t>DOC-fbbe4a664b14f54b</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -8393,27 +8363,27 @@
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
+          <t>安市税稽处〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>安市税稽处〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
           <t>安市税稽罚〔2026〕1号</t>
         </is>
       </c>
-      <c r="N62" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽处〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="O62" s="2" t="inlineStr">
-        <is>
-          <t>安市税稽罚〔2026〕1号</t>
-        </is>
-      </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
@@ -8421,11 +8391,11 @@
           <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
         </is>
       </c>
-      <c r="R62" s="3" t="n"/>
+      <c r="R62" s="3" t="n">
+        <v>64884.41</v>
+      </c>
       <c r="S62" s="3" t="n"/>
-      <c r="T62" s="3" t="n">
-        <v>200000</v>
-      </c>
+      <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="n"/>
       <c r="V62" s="2" t="inlineStr">
         <is>
@@ -8483,90 +8453,102 @@
       </c>
       <c r="AJ62" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“处理或处罚结果”历史冲突已由官方附件复核,保留当前值。 字段“主要违法事实”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>CASE-fe959d4c6c52d910</t>
+          <t>CASE-f78ec1a594442165</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>DOC-f2643f2a0719d8d1</t>
+          <t>DOC-9a828a6048b54b6c</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>广西壮族自治区</t>
+          <t>贵州省</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>南宁市</t>
+          <t>安顺市</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局南宁市税务局第一稽查局</t>
+          <t>国家税务总局安顺市税务局</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局南宁市税务局第一稽查局</t>
+          <t>国家税务总局安顺市税务局稽查局</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>南宁洪谦金贸易有限公司</t>
+          <t>贵州华泰宁安工程建筑设计有限责任公司</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>91450103MA5K9WHY7U</t>
+          <t>91520423MA6DLH799Q</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>南市税一稽处〔2026〕2号</t>
+          <t>安市税稽罚〔2026〕1号</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>南市税一稽处〔2026〕2号</t>
-        </is>
-      </c>
-      <c r="O63" s="2" t="inlineStr"/>
+          <t>安市税稽处〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>安市税稽罚〔2026〕1号</t>
+        </is>
+      </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>经我局2025年10月29日至2025年12月8日对你公司(地址:南宁市青秀区云景路11号春晖花园C区3栋2单元1606号)2015年12月2日至2016年12月31日期间的涉税情况进行了检查,你(单位)存在以下违法事实: 经查询你公司向税务机关报备的银行账号:广西北部湾银行南宁市财富国际支行800099398800015,经函询广西北部湾银行南宁市财富国际支行,存在以下问题: 上述行为属于开具与实际经营业务情况不符的增值税发票,违反了《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第587号修改)第二十二条第一款、第二款第(一)项的规定,属于虚开发票行为。</t>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>增值税</t>
+          <t>增值税、企业所得税、消费税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、教育费附加、地方教育附加</t>
         </is>
       </c>
       <c r="R63" s="3" t="n"/>
       <c r="S63" s="3" t="n"/>
-      <c r="T63" s="3" t="n"/>
+      <c r="T63" s="3" t="n">
+        <v>200000</v>
+      </c>
       <c r="U63" s="3" t="n"/>
-      <c r="V63" s="2" t="inlineStr"/>
-      <c r="W63" s="4" t="n"/>
+      <c r="V63" s="2" t="inlineStr">
+        <is>
+          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W63" s="4" t="n">
+        <v>45898</v>
+      </c>
       <c r="X63" s="4" t="n">
-        <v>46031</v>
+        <v>46043</v>
       </c>
       <c r="Y63" s="4" t="n"/>
       <c r="Z63" s="4" t="n">
@@ -8603,7 +8585,7 @@
       <c r="AG63" s="2" t="inlineStr"/>
       <c r="AH63" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局南宁市税务局第一稽查局税务文书送达公告_国家税务总局南宁市税务局</t>
+          <t>国家税务总局安顺市税务局稽查局关于送达《税务处理决定书》《税务行政处罚决定书》的公告</t>
         </is>
       </c>
       <c r="AI63" s="2" t="inlineStr">
@@ -8613,51 +8595,55 @@
       </c>
       <c r="AJ63" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>CASE-1983d97878508732</t>
+          <t>CASE-fe959d4c6c52d910</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>DOC-f9760895b4f08cc2</t>
+          <t>DOC-f2643f2a0719d8d1</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>内蒙古自治区</t>
+          <t>广西壮族自治区</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>二连浩特市</t>
+          <t>南宁市</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局二连浩特市税务局</t>
+          <t>国家税务总局南宁市税务局第一稽查局</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局二连浩特市税务局稽查局</t>
+          <t>国家税务总局南宁市税务局第一稽查局</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>二连市坤益腾金属有限公司</t>
-        </is>
-      </c>
-      <c r="J64" s="2" t="inlineStr"/>
+          <t>南宁洪谦金贸易有限公司</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>91450103MA5K9WHY7U</t>
+        </is>
+      </c>
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr">
         <is>
@@ -8666,18 +8652,18 @@
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>二税稽处〔2025〕1号</t>
+          <t>南市税一稽处〔2026〕2号</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>二税稽处〔2025〕1号</t>
+          <t>南市税一稽处〔2026〕2号</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr"/>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>公司院内)涉嫌虚开增值税专用发票的情况进行检查,违法事实 你公司在无真实货物交易的情况下,“让他人为自己”虚开 得有下列虚开发票行为:(一)为他人、为自己开具与实际经营 国人民代表大会常务委员会关于惩治虚开、伪造和非法出售增值 〔1996〕210号)文件:“虚开增值税专用发票的,构成虚开增 值税专用发票罪,具有下列行为之一的,属于虚开增值税专用发 定,你公司上述违法事实中,“让他人为自己”虚开增值税专用 “为他人”虚开增值税专用发票97 份,金额 87,923,181.86 元, 二条第二款的规定虚开发票的,由税务机关没收违法所得; 虚开增值税专用发票行为暂不进行行政处罚,在司法部门作出决 十二条第二款的规定虚开发票的,由税务机关没收违法所得; 依法查处违法行为过程中,发现违法事实涉及的金额、违法事实 的情节、违法事实造成的后果等,根据刑法关于破坏社会主义市 定(二)》(公通字〔2022〕12 号)第五十六条:“〔虚开增值 税专用发票、用于骗取出口退税、抵扣税款发票案(刑法第二百 零五条)〕虚开增值税专用发票或者虚开用于骗取出口退税、抵 扣税款的其他发票,虚开的税款数额在十万元以上或者致使国家 公司虚开增值税专用发票的行为移送公安机关。</t>
+          <t>经我局2025年10月29日至2025年12月8日对你公司(地址:南宁市青秀区云景路11号春晖花园C区3栋2单元1606号)2015年12月2日至2016年12月31日期间的涉税情况进行了检查,你(单位)存在以下违法事实: 经查询你公司向税务机关报备的银行账号:广西北部湾银行南宁市财富国际支行800099398800015,经函询广西北部湾银行南宁市财富国际支行,存在以下问题: 上述行为属于开具与实际经营业务情况不符的增值税发票,违反了《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第587号修改)第二十二条第一款、第二款第(一)项的规定,属于虚开发票行为。</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -8689,13 +8675,11 @@
       <c r="S64" s="3" t="n"/>
       <c r="T64" s="3" t="n"/>
       <c r="U64" s="3" t="n"/>
-      <c r="V64" s="2" t="inlineStr">
-        <is>
-          <t>二条第二款的规定虚开发票的,由税务机关没收违法所得; 十二条第二款的规定虚开发票的,由税务机关没收违法所得;</t>
-        </is>
-      </c>
+      <c r="V64" s="2" t="inlineStr"/>
       <c r="W64" s="4" t="n"/>
-      <c r="X64" s="4" t="n"/>
+      <c r="X64" s="4" t="n">
+        <v>46031</v>
+      </c>
       <c r="Y64" s="4" t="n"/>
       <c r="Z64" s="4" t="n">
         <v>46229</v>
@@ -8715,7 +8699,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE64" s="5" t="inlineStr">
@@ -8723,36 +8707,40 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF64" s="2" t="inlineStr"/>
+      <c r="AF64" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
       <c r="AG64" s="2" t="inlineStr"/>
       <c r="AH64" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>国家税务总局南宁市税务局第一稽查局税务文书送达公告_国家税务总局南宁市税务局</t>
         </is>
       </c>
       <c r="AI64" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>附件正常</t>
         </is>
       </c>
       <c r="AJ64" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“页面标题”存在冲突:保留原值“税务处理决定书”,新值“Á®éŚä°Ś§ĄÁźÜŚÜ≥ŚģöšĻ¶”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>CASE-d4b6986f3f97cd28</t>
+          <t>CASE-1983d97878508732</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>DOC-442cf3d9a5280c12</t>
+          <t>DOC-f9760895b4f08cc2</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -8762,19 +8750,23 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯市</t>
+          <t>二连浩特市</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局二连浩特市税务局</t>
+        </is>
+      </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>第二稽查局</t>
+          <t>国家税务总局二连浩特市税务局稽查局</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>廖礼平</t>
+          <t>二连市坤益腾金属有限公司</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
@@ -8786,36 +8778,32 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>鄂税二稽处〔2023〕29号</t>
+          <t>二税稽处〔2025〕1号</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>鄂税二稽处〔2023〕29号</t>
+          <t>二税稽处〔2025〕1号</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr"/>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>利煤炭有限责任公司股权涉税问题开展了检查,违法事实及处理</t>
+          <t>公司院内)涉嫌虚开增值税专用发票的情况进行检查,违法事实 你公司在无真实货物交易的情况下,“让他人为自己”虚开 得有下列虚开发票行为:(一)为他人、为自己开具与实际经营 国人民代表大会常务委员会关于惩治虚开、伪造和非法出售增值 〔1996〕210号)文件:“虚开增值税专用发票的,构成虚开增 值税专用发票罪,具有下列行为之一的,属于虚开增值税专用发 定,你公司上述违法事实中,“让他人为自己”虚开增值税专用 “为他人”虚开增值税专用发票97 份,金额 87,923,181.86 元, 二条第二款的规定虚开发票的,由税务机关没收违法所得; 虚开增值税专用发票行为暂不进行行政处罚,在司法部门作出决 十二条第二款的规定虚开发票的,由税务机关没收违法所得; 依法查处违法行为过程中,发现违法事实涉及的金额、违法事实 的情节、违法事实造成的后果等,根据刑法关于破坏社会主义市 定(二)》(公通字〔2022〕12 号)第五十六条:“〔虚开增值 税专用发票、用于骗取出口退税、抵扣税款发票案(刑法第二百 零五条)〕虚开增值税专用发票或者虚开用于骗取出口退税、抵 扣税款的其他发票,虚开的税款数额在十万元以上或者致使国家 公司虚开增值税专用发票的行为移送公安机关。</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>个人所得税、印花税</t>
-        </is>
-      </c>
-      <c r="R65" s="3" t="n">
-        <v>15072487.5</v>
-      </c>
-      <c r="S65" s="3" t="n">
-        <v>1046925</v>
-      </c>
+          <t>增值税</t>
+        </is>
+      </c>
+      <c r="R65" s="3" t="n"/>
+      <c r="S65" s="3" t="n"/>
       <c r="T65" s="3" t="n"/>
       <c r="U65" s="3" t="n"/>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>以上共计应补缴个人所得税14,997,500.00元。 以上共计应补缴印花税74,987.50元。 规定,对应补缴个人所得税14,997,500.00元加收从2011年4月1</t>
+          <t>二条第二款的规定虚开发票的,由税务机关没收违法所得; 十二条第二款的规定虚开发票的,由税务机关没收违法所得;</t>
         </is>
       </c>
       <c r="W65" s="4" t="n"/>
@@ -8861,55 +8849,47 @@
       </c>
       <c r="AJ65" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“页面标题”存在冲突:保留原值“税务处理决定书”,新值“Á®éŚä°Ś§ĄÁźÜŚÜ≥ŚģöšĻ¶”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/elht/xjtzgghhht/202501/W020250110616020148238.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/elht/tzgghhht/202501/W020250110616020148238.pdf”未静默覆盖。 字段“页面标题”存在冲突:保留原值“税务处理决定书”,新值“Á®éŚä°Ś§ĄÁźÜŚÜ≥ŚģöšĻ¶”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>CASE-3996d04fd944424e</t>
+          <t>CASE-d4b6986f3f97cd28</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>DOC-af179599b7f27421</t>
+          <t>DOC-442cf3d9a5280c12</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>天津市</t>
+          <t>内蒙古自治区</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>天津市</t>
+          <t>鄂尔多斯市</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
-        </is>
-      </c>
+      <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局天津市税务局第一稽查局</t>
+          <t>第二稽查局</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>信硕(天津)国际货运代理有限公司</t>
-        </is>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>91120105MA06WEYU7C</t>
-        </is>
-      </c>
+          <t>廖礼平</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr">
         <is>
@@ -8918,35 +8898,43 @@
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2022〕270号</t>
+          <t>鄂税二稽处〔2023〕29号</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2022〕270号</t>
+          <t>鄂税二稽处〔2023〕29号</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr"/>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>我局(所)于2022年6月24日至2022年8月18日对你(单位)(地址:天津市河北区建昌道街道铁工东里增57-1号)2019年12月2日至2022年5月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位无生产经营地点,虚假注册,无社保信息,与上下游企业无银行交易记录,收取上游企业虚开的增值税发票后脱离税务机关监管,经核实,你单位不符合正常企业构成要件,认定为假企业。 你单位在2019年12月02日-2022年5月31日期间,未发生真实货物、劳务交易,对下游13户企业开具增值税普通发票990份,发票代码012001900105,发票号码04884187-04884216,04893407-04893421,04898548,06548576-06548620,06671887-06671896,06807185-06807194,06909763-06909797,07353556-07353600,07359910-07359954,07369273-07369317,07374190-07374214,07379166-07379235,09307219-09307288,09319483-09319552,09327879-09327948,11915880-11915949,11925651-11925720,11937167-11937236,11941265-11941334,11945987-11946000,11948001-11948056,发票代码012001900104,发票号码24048210-24048219,虚开增值税普通发票不含税金额73000214.83元,税额0元,价税合计73000214.83元。</t>
+          <t>利煤炭有限责任公司股权涉税问题开展了检查,违法事实及处理</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>增值税、消费税</t>
-        </is>
-      </c>
-      <c r="R66" s="3" t="n"/>
-      <c r="S66" s="3" t="n"/>
+          <t>个人所得税、印花税</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="n">
+        <v>15072487.5</v>
+      </c>
+      <c r="S66" s="3" t="n">
+        <v>1046925</v>
+      </c>
       <c r="T66" s="3" t="n"/>
       <c r="U66" s="3" t="n"/>
-      <c r="V66" s="2" t="inlineStr"/>
+      <c r="V66" s="2" t="inlineStr">
+        <is>
+          <t>以上共计应补缴个人所得税14,997,500.00元。 以上共计应补缴印花税74,987.50元。 规定,对应补缴个人所得税14,997,500.00元加收从2011年4月1</t>
+        </is>
+      </c>
       <c r="W66" s="4" t="n"/>
       <c r="X66" s="4" t="n"/>
       <c r="Y66" s="4" t="n"/>
       <c r="Z66" s="4" t="n">
-        <v>46248</v>
+        <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
         <v>46250</v>
@@ -8975,7 +8963,7 @@
       <c r="AG66" s="2" t="inlineStr"/>
       <c r="AH66" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达信硕(天津)国际货运代理有限公司《税务处理决定书》的公告</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="AI66" s="2" t="inlineStr">
@@ -8985,22 +8973,22 @@
       </c>
       <c r="AJ66" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“涉及税种”存在冲突:保留原值“增值税、消费税”,新值“增值税”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“http://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202311/P020231101635149652485.pdf”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202311/P020231101635149652485.pdf”未静默覆盖。 字段“页面标题”存在冲突:保留原值“税务处理决定书”,新值“Á®éŚä°Ś§ĄÁźÜŚÜ≥ŚģöšĻ¶”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>CASE-7e3d4a321440d6a7</t>
+          <t>CASE-3996d04fd944424e</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>DOC-bed9330343ed06af</t>
+          <t>DOC-af179599b7f27421</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -9026,12 +9014,12 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>天津展达科技有限公司</t>
+          <t>信硕(天津)国际货运代理有限公司</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>91120116300738701X</t>
+          <t>91120105MA06WEYU7C</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
@@ -9042,45 +9030,35 @@
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
+          <t>津税一稽处〔2022〕270号</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O67" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
+          <t>津税一稽处〔2022〕270号</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr"/>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+          <t>我局(所)于2022年6月24日至2022年8月18日对你(单位)(地址:天津市河北区建昌道街道铁工东里增57-1号)2019年12月2日至2022年5月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位无生产经营地点,虚假注册,无社保信息,与上下游企业无银行交易记录,收取上游企业虚开的增值税发票后脱离税务机关监管,经核实,你单位不符合正常企业构成要件,认定为假企业。 你单位在2019年12月02日-2022年5月31日期间,未发生真实货物、劳务交易,对下游13户企业开具增值税普通发票990份,发票代码012001900105,发票号码04884187-04884216,04893407-04893421,04898548,06548576-06548620,06671887-06671896,06807185-06807194,06909763-06909797,07353556-07353600,07359910-07359954,07369273-07369317,07374190-07374214,07379166-07379235,09307219-09307288,09319483-09319552,09327879-09327948,11915880-11915949,11925651-11925720,11937167-11937236,11941265-11941334,11945987-11946000,11948001-11948056,发票代码012001900104,发票号码24048210-24048219,虚开增值税普通发票不含税金额73000214.83元,税额0元,价税合计73000214.83元。</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
-        </is>
-      </c>
-      <c r="R67" s="3" t="n">
-        <v>920146.9399999999</v>
-      </c>
+          <t>增值税、消费税</t>
+        </is>
+      </c>
+      <c r="R67" s="3" t="n"/>
       <c r="S67" s="3" t="n"/>
       <c r="T67" s="3" t="n"/>
       <c r="U67" s="3" t="n"/>
-      <c r="V67" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V67" s="2" t="inlineStr"/>
       <c r="W67" s="4" t="n"/>
       <c r="X67" s="4" t="n"/>
       <c r="Y67" s="4" t="n"/>
       <c r="Z67" s="4" t="n">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="AA67" s="4" t="n">
         <v>46250</v>
@@ -9109,7 +9087,7 @@
       <c r="AG67" s="2" t="inlineStr"/>
       <c r="AH67" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+          <t>国家税务总局天津市税务局第一稽查局关于送达信硕(天津)国际货运代理有限公司《税务处理决定书》的公告</t>
         </is>
       </c>
       <c r="AI67" s="2" t="inlineStr">
@@ -9119,13 +9097,13 @@
       </c>
       <c r="AJ67" s="2" t="inlineStr">
         <is>
-          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“涉及税种”存在冲突:保留原值“增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加”,新值“增值税、企业所得税、城市维护建设税、教育费附加、地方教育附加”未静默覆盖。</t>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“涉及税种”存在冲突:保留原值“增值税、消费税”,新值“增值税”未静默覆盖。</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
@@ -9134,7 +9112,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>DOC-388bd01c01bbb789</t>
+          <t>DOC-bed9330343ed06af</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -9171,24 +9149,24 @@
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
           <t>津税一稽罚〔2023〕21号</t>
         </is>
       </c>
-      <c r="N68" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽处〔2023〕59号</t>
-        </is>
-      </c>
-      <c r="O68" s="2" t="inlineStr">
-        <is>
-          <t>津税一稽罚〔2023〕21号</t>
-        </is>
-      </c>
       <c r="P68" s="2" t="inlineStr">
         <is>
           <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
@@ -9199,11 +9177,11 @@
           <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
         </is>
       </c>
-      <c r="R68" s="3" t="n"/>
+      <c r="R68" s="3" t="n">
+        <v>920146.9399999999</v>
+      </c>
       <c r="S68" s="3" t="n"/>
-      <c r="T68" s="3" t="n">
-        <v>131368.5</v>
-      </c>
+      <c r="T68" s="3" t="n"/>
       <c r="U68" s="3" t="n"/>
       <c r="V68" s="2" t="inlineStr">
         <is>
@@ -9257,20 +9235,154 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>CASE-7e3d4a321440d6a7</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>DOC-388bd01c01bbb789</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>天津市</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>天津展达科技有限公司</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>91120116300738701X</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>税务行政处罚决定书</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽处〔2023〕59号</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>津税一稽罚〔2023〕21号</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>我局(所)于2020年8月7日至2022年11月30日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709)2016年1月1日至2017年12月31日纳税情况进行了检查,违法事实及处理决定如下: 经查,你单位取得天津盛汇康机械制品销售有限公司已证实虚开的10份增值税专用发票,发票代码1200154130,发票号码02675003-02675012,发票金额970,696.88元,税额159,933.52元,价税合计1,130,630.4元; 取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元。 根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 经我局(所)于2022年02月14 日至2023年03月09日对你(单位)(地址:天津华苑产业区榕苑路15号1-B-1709 )2016年01月01 日至2017年12月31 日纳税情况进行检查,你(单位)存在违法事实及处罚决定如下: 你单位取得天津明珠电子器件有限公司已证实虚开的15份增值税专用发票,发票代码1200162130,发票号码15241705-15241719,发票金额1,438,034.13元,税额244,465.87元,价税合计1,682,500元,你单位利用他人虚开的专用发票,向税务机关申报抵扣税款进行偷税,少缴增值税244,465.87元、少缴城市维护建设税17,112.61元、少缴企业所得税262,737.00。</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加</t>
+        </is>
+      </c>
+      <c r="R69" s="3" t="n"/>
+      <c r="S69" s="3" t="n"/>
+      <c r="T69" s="3" t="n">
+        <v>131368.5</v>
+      </c>
+      <c r="U69" s="3" t="n"/>
+      <c r="V69" s="2" t="inlineStr">
+        <is>
+          <t>根据《中华人民共和国增值税暂行条例》第九条、《中华人民共和国增值税暂行条例实施细则》第十九条、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(2012年第33号)中“纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额”之规定,决定追缴2016年8月增值税159,933.52元,2017年1月增值税244,465.87元。 到期不缴纳罚款,我局(所)可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+        </is>
+      </c>
+      <c r="W69" s="4" t="n"/>
+      <c r="X69" s="4" t="n"/>
+      <c r="Y69" s="4" t="n"/>
+      <c r="Z69" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="AA69" s="4" t="n">
+        <v>46250</v>
+      </c>
+      <c r="AB69" s="2" t="inlineStr">
+        <is>
+          <t>完整文书</t>
+        </is>
+      </c>
+      <c r="AC69" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD69" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="AE69" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF69" s="2" t="inlineStr"/>
+      <c r="AG69" s="2" t="inlineStr"/>
+      <c r="AH69" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局天津市税务局第一稽查局关于送达天津展达科技有限公司《税务处理决定书》《税务行政处罚决定书》的公告</t>
+        </is>
+      </c>
+      <c r="AI69" s="2" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="AJ69" s="2" t="inlineStr">
+        <is>
+          <t>页面未提取到可确认的官方发布日期。 Excel 与 CSV 历史数据已合并核对。 字段“涉及税种”存在冲突:保留原值“增值税、企业所得税、消费税、城市维护建设税、教育费附加、地方教育附加”,新值“增值税、企业所得税、城市维护建设税、教育费附加、地方教育附加”未静默覆盖。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ68"/>
-  <conditionalFormatting sqref="AD2:AD68">
+  <autoFilter ref="A1:AJ69"/>
+  <conditionalFormatting sqref="AD2:AD69">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI68">
+  <conditionalFormatting sqref="AI2:AI69">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9353,24 +9465,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE56" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF56" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE57" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF57" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE58" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF58" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE59" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE57" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF57" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE58" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF58" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE59" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF59" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE60" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE61" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF61" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE62" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF62" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF63" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE64" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE62" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF62" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF63" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE64" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF64" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE66" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE67" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId97"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -9651,11 +9764,7 @@
           <t>91450181MACQW4NT1E</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>或者股东的个人账户</t>
-        </is>
-      </c>
+      <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>税务处理决定书</t>
@@ -9779,7 +9888,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>同时,该地址也是广西槟咪科技有限公司</t>
+          <t>广西苒炙机械设备有限公司</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -9822,11 +9931,7 @@
       <c r="S3" s="3" t="n"/>
       <c r="T3" s="3" t="n"/>
       <c r="U3" s="3" t="n"/>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="4" t="n">
         <v>46157</v>
       </c>
@@ -9878,7 +9983,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”存在冲突:保留原值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处理决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”,新值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处罚决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”历史冲突已由官方附件复核,保留当前值。 当事人名称经官方原文复核,由“同时,该地址也是广西槟咪科技有限公司”更正为“广西苒炙机械设备有限公司”。 字段“处理或处罚结果”历史冲突已由官方附件复核,保留当前值。 处理文书中的处罚结果串值已根据官方附件清除。</t>
         </is>
       </c>
     </row>
@@ -9906,7 +10011,11 @@
           <t>河池市</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>金城江区</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>国家税务总局河池市税务局第二稽查局</t>
@@ -9919,7 +10028,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>同时,该地址也是广西槟咪科技有限公司</t>
+          <t>广西苒炙机械设备有限公司</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -9950,7 +10059,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处理决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。</t>
+          <t>经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处罚决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -9960,11 +10069,13 @@
       </c>
       <c r="R4" s="3" t="n"/>
       <c r="S4" s="3" t="n"/>
-      <c r="T4" s="3" t="n"/>
+      <c r="T4" s="3" t="n">
+        <v>200000</v>
+      </c>
       <c r="U4" s="3" t="n"/>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 2026〕12 号)、《国家税务总局河池市税务局第二稽查局税务行政处罚决定书》(河市税二稽罚〔2026〕6号)予以公告送达。 同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。</t>
+          <t>同时根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第三十五条第一款、参照《国家税务总局广东省税务局 国家税务总局河南省税务局 国家税务总局湖北省税务局 国家税务总局湖南省税务局 国家税务总局广西壮族自治区税务局 国家税务总局海南省税务局 国家税务总局深圳市税务局关于发布〈中南区域税务行政处罚裁量基准〉的公告》(国家税务总局广东省税务局 国家税务总局河南省税务局等税务局公告2023年第5号)附件《中南区域税务行政处罚裁量基准》第45项违法行为第3档裁量基准“虚开金额在100万元以上(不含本数)500万元以下的,没收违法所得,并处20万元以上50万元以下的罚款”之规定,你公司虚开发票行为属于第3档“严重”情形,对你公司虚开增值税电子普通发票的行为处以200,000.00元的罚款。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W4" s="4" t="n">
@@ -10018,7 +10129,7 @@
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”存在冲突:保留原值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处理决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”,新值“经我局于2026年3月24日至2026年5月15日对你公司(地址:河池市金城江区明月路21号幸福嘉园6栋2-108号)2026年01月26日至2026年02月28日期间涉税情况进行检查,你公司存在违法事实及处罚决定如下: 你公司存续时间短,开具发票后,直接走逃失踪不进行纳税申报:通过金税三期税收管理系统、增值税发票电子底账系统、广西税务局大数据分析应用集成平台查询,你公司的“申报明细”信息数为“0”,“未申报信息”信息数为“17”,“税款入库信息”信息数为“0”,即:你公司未进行任何纳税申报,无任何税款入库信息。 综合以上调查情况,你公司无实际办公经营场所、无真实货物购进,未向税务机关报备银行存款账号,未进行纳税申报,相关工作人员均无法联系,经公告送达文书后亦无人向税务机关反馈,参照《国家税务总局关于走逃(失联)企业开具增值税专用发票认定处理有关问题的公告》(国家税务总局公告2016年第76号)、《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司为走逃失联企业,且无真实办公场所,无真实经营业务。 经核查,你公司已走逃失联,经公告送达文书后亦无公司相关人员联系配合调查,注册地址无实际经营场所,无货物购进发票,开票后已连续多月未进行纳税申报,根据《中华人民共和国发票管理办法》(财政部令第6号发布,国务院令第764号修订)第二十一条第二款第(一)项、《中华人民共和国发票管理办法实施细则》(国家税务总局令第56号)第二十九条第(一)项、参照《国家税务总局关于走逃(失联)企业涉嫌虚开增值税专用发票检查问题的通知》(税总发〔2016〕172号)规定,认定你公司开具的上述53份增值税电子普通发票为虚开。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 当事人名称经官方原文复核,由“同时,该地址也是广西槟咪科技有限公司”更正为“广西苒炙机械设备有限公司”。 字段“主要违法事实”已根据官方附件重新解析。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -10067,11 +10178,7 @@
           <t>91370220MA9490X30G</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>或委托代理人持单位公章等</t>
-        </is>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>税务处理决定书</t>
@@ -10106,11 +10213,7 @@
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="3" t="n"/>
-      <c r="V5" s="2" t="inlineStr">
-        <is>
-          <t>根据《中华人民共和国税收征收管理法实施细则》第一百零六条第(二)款之规定,因采用其他方式无法向你单位送达税务文书,我局决定对《税务行政处罚决定书》(青税稽一罚〔2026〕65号)、《税务处理决定书》(青税稽一处〔2026〕73号)予以公告送达。 根据《中华人民共和国发票管理办法》(国函〔1993〕174号,2019年3月2日《国务院关于修改部分行政法规的决定》(中华人民共和国国务院令第709号)第二次修改)第三十七条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 构成犯罪的,依法追究刑事责任”、参照《国家税务总局关于发布&lt;税务行政处罚裁量权行使规则&gt;的公告》(国家税务总局公告2016年第78号)的规定,对你公司虚开发票行为处以罚款140000.00元。 ”、《中华人民共和国税收征收管理法实施细则》第九十六条“纳税人、扣缴义务人有下列情形之一的,依照税收征管法第七十条的规定处罚,(一)提供虚假材料,不如实反映情况,或者拒绝提供有关资料的”的规定,你单位经责令限期改正,至检查结束,拒不提供有关纳税资料,对你公司处以罚款20000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
-        </is>
-      </c>
+      <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="4" t="n"/>
       <c r="X5" s="4" t="n">
         <v>46240</v>
@@ -10154,7 +10257,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。 处理文书中的处罚结果串值已根据官方附件清除。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -10201,11 +10308,7 @@
           <t>91370220MA9490X30G</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>或委托代理人持单位公章等</t>
-        </is>
-      </c>
+      <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>税务行政处罚决定书</t>
@@ -10290,7 +10393,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -11160,7 +11267,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>查属期内违法行为均定性偷税, 需要对原处罚决定中的罚款数额 以变更,你(单位)存在违法事实及处罚决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 〔2022〕59号) 第一条、 第三条之规定, 你单位存在少缴属期2010 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 报,不缴或者少缴应纳税款的,是偷税。 务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴 内首次因偷税被税务机关处罚,并能够配合税务机关检查的,处 不缴或者少缴的税款百分之五十的罚款”之规定,对你单位城镇 土地使用税和印花税处不缴或者少缴的税款50%的罚款。 你单位印花税偷税违法行为发生于2009年11月26日,至立案 位检查属期内违法行为均定性偷税, 需要对原处理决定中的查补 情况进行了检查,违法事实及处理决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 定, 你单位存在少缴属期2010年1月至2022年6月城镇土地使 用税5,710,765.50元的违法事实。 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 该地块未缴纳契税,你单位存在少缴契税509,984.64元的违法 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。</t>
+          <t>位检查属期内违法行为均定性偷税, 需要对原处理决定中的查补 情况进行了检查,违法事实及处理决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 定, 你单位存在少缴属期2010年1月至2022年6月城镇土地使 用税5,710,765.50元的违法事实。 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 该地块未缴纳契税,你单位存在少缴契税509,984.64元的违法 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 单位未申报2010年1月1日至2022年6月30日契税。 6月申报数据,用于证明你单位未申报缴纳契税。</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -11176,7 +11283,7 @@
       <c r="U13" s="3" t="n"/>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>定,每日按罚款数额的百分之三加处罚款。 日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税 日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税</t>
+          <t>日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税</t>
         </is>
       </c>
       <c r="W13" s="4" t="n">
@@ -11230,7 +11337,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”已根据官方附件重新解析。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -11302,7 +11409,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>查属期内违法行为均定性偷税, 需要对原处罚决定中的罚款数额 以变更,你(单位)存在违法事实及处罚决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 〔2022〕59号) 第一条、 第三条之规定, 你单位存在少缴属期2010 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 报,不缴或者少缴应纳税款的,是偷税。 务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴 内首次因偷税被税务机关处罚,并能够配合税务机关检查的,处 不缴或者少缴的税款百分之五十的罚款”之规定,对你单位城镇 土地使用税和印花税处不缴或者少缴的税款50%的罚款。 你单位印花税偷税违法行为发生于2009年11月26日,至立案 位检查属期内违法行为均定性偷税, 需要对原处理决定中的查补 情况进行了检查,违法事实及处理决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 定, 你单位存在少缴属期2010年1月至2022年6月城镇土地使 用税5,710,765.50元的违法事实。 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 该地块未缴纳契税,你单位存在少缴契税509,984.64元的违法 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。</t>
+          <t>查属期内违法行为均定性偷税, 需要对原处罚决定中的罚款数额 以变更,你(单位)存在违法事实及处罚决定如下: 月至2011年8月和2016年6月未申报城镇土地使用税,2011 〔2022〕59号) 第一条、 第三条之规定, 你单位存在少缴属期2010 签订了 TLTN200907《国有建设用地使用权出让合同》 , 未申报缴 之规定, 你单位存在少缴2009年11月26日印花税6,374.80元 用于证明你单位采用虚假纳税申报或未申报方式申报2010年1 你单位未申报2010年1月1日至2022年6月30日印花税。 月属期申报数据,用于证明你单位未申报缴纳印花税。 报,不缴或者少缴应纳税款的,是偷税。 务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴 内首次因偷税被税务机关处罚,并能够配合税务机关检查的,处 不缴或者少缴的税款百分之五十的罚款”之规定,对你单位城镇 土地使用税和印花税处不缴或者少缴的税款50%的罚款。 你单位印花税偷税违法行为发生于2009年11月26日,至立案</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -11318,7 +11425,7 @@
       <c r="U14" s="3" t="n"/>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>定,每日按罚款数额的百分之三加处罚款。 日”之规定,你单位每月应补缴城镇土地使用税44,269.50元 征收城镇土地使用税, 自2010年1月至2022年6月应补缴城镇 所载金额的万分之五,你单位应补缴2009年11月26日印花税 定,每日按罚款数额的百分之三加处罚款。</t>
+          <t>定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W14" s="4" t="n">
@@ -11372,7 +11479,7 @@
       </c>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 字段“关联处理决定书文号”存在冲突:保留原值“铁税一稽处〔2026〕35号”,新值“铁税一稽处〔2024〕9号”未静默覆盖。 字段“关联处罚决定书文号”存在冲突:保留原值“铁税一稽罚〔2026〕17号”,新值“铁税一稽罚〔2024〕8号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。 字段“主要违法事实”已根据官方附件重新解析。 字段“涉及税种”存在冲突:保留原值“增值税、城市维护建设税、房产税、城镇土地使用税、印花税、资源税、契税、教育费附加、地方教育附加”,新值“房产税、城镇土地使用税、印花税”未静默覆盖。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -12648,7 +12755,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
+          <t>我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -12718,7 +12825,7 @@
       </c>
       <c r="AJ24" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636255688.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。 字段“主要违法事实”存在冲突:保留原值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,你单位存在违法事实及处罚决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”,新值“我局于2022年5月9日至2025年8月29日对你单位(地址:贵州省安顺市镇宁布依族苗族自治县城关镇城西村五组)2019年1月1日至2022年3月31日涉税情况进行了检查,违法事实及处理决定如下: 2022年6月,安顺市税务局稽查局将你单位上述虚开发票的线索移送给镇宁布依族苗族自治县公安局经济犯罪侦查大队,经公安机关对王*立案及检察院起诉后,2024年12月30日镇宁布依族苗族自治县人民法院作出王*犯虚开增值税发票罪的刑事判决,《刑事判决书》((2024)黔0423刑初198号)确认上述贵州宏翼翔汽车销售服务有限公司开具给你单位的6份增值税专用发票(金额460,177.02元,税额59,822.98元)、安顺润亨化工贸易有限公司开具给你单位的91份增值税专用发票(金额8,325,968.72元,税额1,047,999.48元)为虚开发票,判决王*犯虚开增值税专用发票罪,并处罚金人民币5万元。 经查,上述业务款项是贵州安顺家喻物业管理有限公司直接付款给罗*,罗*为了向贵州安顺家喻物业管理有限公司提供发票,通过支付手续费的方式找王*为其提供发票,王*指使贵州理得清财务有限公司员工彭*毕通过微信收取罗*手续费2,129.00元,后彭*毕又将该笔资金转到了贵州理得清财务有限公司微信账号。 根据《中华人民共和国发票管理办法》第二十一条第二款“任何单位和个人不得有下列虚开发票行为:(一)为他人、为自己开具与实际经营业务情况不符的发票; ”、《国家税务总局关于纳税人虚开增值税专用发票征补税款问题的公告》(国家税务总局公告2012年第33号)“......纳税人取得虚开的增值税专用发票,不得作为增值税合法有效的扣税凭证抵扣其进项税额。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“追缴税款金额”存在冲突:保留原值“64884.41”,新值“1521925.53”未静默覆盖。 字段“处理或处罚结果”历史冲突已由官方附件复核,保留当前值。 字段“主要违法事实”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -12806,7 +12913,7 @@
       <c r="U25" s="3" t="n"/>
       <c r="V25" s="2" t="inlineStr">
         <is>
-          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。</t>
+          <t>你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W25" s="4" t="n">
@@ -12860,7 +12967,7 @@
       </c>
       <c r="AJ25" s="2" t="inlineStr">
         <is>
-          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。”未静默覆盖。 字段“官方原文链接”存在冲突:保留原值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/t20260121_89320381.html”,新值“https://guizhou.chinatax.gov.cn/sjpd/ass/tzgg_59745/202601/P020260121598636222410.docx”未静默覆盖。 字段“处理或处罚结果”存在冲突:保留原值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共计应补缴企业所得税64,884.41元。 ”、第五十二条“因税务机关的责任,致使纳税人、扣缴义务人未缴或者少缴税款的,税务机关在三年内可以要求纳税人、扣缴义务人补缴税款,但是不得加收滞纳金。 ”、《中华人民共和国税收征收管理法实施细则》(国务院令第362号)第七十五条“税收征管法第三十二条规定的加收滞纳金的起止时间,为法律、行政法规规定或者税务机关依照法律、行政法规的规定确定的税款缴纳期限届满次日起至纳税人、扣缴义务人实际缴纳或者解缴税款之日止”之规定,我局决定追缴你单位少缴的增值税696,485.49元、城市维护建设税50,019.66元、印花税312.70元、企业所得税64,884.41元。 逾期仍不补缴的,对单位处以1000元以上3万元以下罚款,对个人处以100元以上1000元以下的罚款”之规定,现责令你单位缴纳少缴的教育费附加30,011.79元、地方教育附加20,007.86元,并对少缴的教育费附加、地方教育附加从滞纳之日起至实际缴纳之日止,按日加收万分之五的滞纳金。”,新值“你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; 综上,应追缴你单位2020年至2022年少缴的城市维护建设税50,019.66元。 ”之规定,本次稽查你单位2020年应补缴的城市维护建设税20,172.19元、教育费附加12,103.32元、地方教育附加8,068.88元、印花税95.20元准予在企业所得税前扣除,应调减2020年企业所得税应纳税所得额40,439.59元; 2021年应补缴的城市维护建设税24,475.99元、教育费附加14,685.58元、地方教育附加9,790.39元、印花税217.50元准予在企业所得税前扣除,应调减2021年企业所得税应纳税所得额49,169.46元。 你单位2020年至2021年共应补缴企业所得税64,884.41元。 ”、《中华人民共和国发票管理办法》第三十五条第一款“违反本办法的规定虚开发票的,由税务机关没收违法所得; 对你单位取得安顺润亨化工贸易有限公司2021年12月虚开28份增值税专用发票以及2019年6月向贵州安顺家喻物业管理有限公司虚开1份增值税专用发票的行为,决定处以罚款200,000.00元。 综上,对你单位决定处以罚款200,000.00元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。 你单位应就少缴的增值税696,485.49元补缴城市维护建设税34,824.28元; ”之规定,你单位应就少缴的增值税696,485.49元补缴教育费附加20,894.56元,应补缴地方教育附加13,929.71元。 ”之规定,你单位应补缴印花税312.70元。”未静默覆盖。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。 字段“处理或处罚结果”已根据官方附件重新解析。</t>
         </is>
       </c>
     </row>
@@ -13705,7 +13812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AJ38"/>
+  <dimension ref="A1:AJ39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18212,66 +18319,66 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>CASE-393a878d93a22709</t>
+          <t>CASE-eb7e9c22bd97f211</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>DOC-cda8cba853896b18</t>
+          <t>DOC-4c99e9a228472ee1</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>广东省</t>
+          <t>江苏省</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>广州市</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>番禺区</t>
-        </is>
-      </c>
+          <t>无锡市</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局广州市番禺区税务局</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr"/>
+          <t>国家税务总局无锡市税务局第一稽查局</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局无锡市税务局第一稽查局</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>广州赞荣服装有限公司</t>
+          <t>宜兴市华欧金属材料有限公司</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>91440113MA59AJFJ1J</t>
+          <t>91320282MA1MMJ8YXD</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>税务行政处罚决定书</t>
+          <t>税务处理决定书</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr">
-        <is>
-          <t>穗番税退罚字〔2026〕1号</t>
-        </is>
-      </c>
+          <t>锡税一稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>锡税一稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr"/>
       <c r="P37" s="2" t="inlineStr"/>
       <c r="Q37" s="2" t="inlineStr"/>
       <c r="R37" s="3" t="n"/>
@@ -18281,11 +18388,11 @@
       <c r="V37" s="2" t="inlineStr"/>
       <c r="W37" s="4" t="n"/>
       <c r="X37" s="4" t="n">
-        <v>46091</v>
+        <v>46111</v>
       </c>
       <c r="Y37" s="4" t="n"/>
       <c r="Z37" s="4" t="n">
-        <v>46229</v>
+        <v>46250</v>
       </c>
       <c r="AA37" s="4" t="n">
         <v>46250</v>
@@ -18302,7 +18409,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>待核验</t>
+          <t>已核验</t>
         </is>
       </c>
       <c r="AE37" s="5" t="inlineStr">
@@ -18310,90 +18417,86 @@
           <t>打开原文</t>
         </is>
       </c>
-      <c r="AF37" s="5" t="inlineStr">
-        <is>
-          <t>打开附件</t>
-        </is>
-      </c>
+      <c r="AF37" s="2" t="inlineStr"/>
       <c r="AG37" s="2" t="inlineStr"/>
       <c r="AH37" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
+          <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局无锡市税务局第一稽查局关于送达《税务处理决定书》的公告(宜兴市华欧金属材料有限公司)</t>
         </is>
       </c>
       <c r="AI37" s="2" t="inlineStr">
         <is>
-          <t>内容不匹配</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="AJ37" s="2" t="inlineStr">
         <is>
-          <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>CASE-0b4a4519ba4f5ad9</t>
+          <t>CASE-393a878d93a22709</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>DOC-5376b9bae81cfc82</t>
+          <t>DOC-cda8cba853896b18</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>江苏省</t>
+          <t>广东省</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>常州市</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
+          <t>广州市</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>番禺区</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>国家税务总局江苏省税务局</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>国家税务总局常州市税务局稽查局</t>
-        </is>
-      </c>
+          <t>国家税务总局广州市番禺区税务局</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>常州好佳车辆配件有限公司</t>
+          <t>广州赞荣服装有限公司</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>91320411094264460B</t>
+          <t>91440113MA59AJFJ1J</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>税务处理决定书</t>
+          <t>税务行政处罚决定书</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>常税稽处〔2026〕71号</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>常税稽处〔2026〕71号</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr"/>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>穗番税退罚字〔2026〕1号</t>
+        </is>
+      </c>
       <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="3" t="n"/>
@@ -18403,7 +18506,7 @@
       <c r="V38" s="2" t="inlineStr"/>
       <c r="W38" s="4" t="n"/>
       <c r="X38" s="4" t="n">
-        <v>46087</v>
+        <v>46091</v>
       </c>
       <c r="Y38" s="4" t="n"/>
       <c r="Z38" s="4" t="n">
@@ -18424,7 +18527,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>已核验</t>
+          <t>待核验</t>
         </is>
       </c>
       <c r="AE38" s="5" t="inlineStr">
@@ -18440,34 +18543,156 @@
       <c r="AG38" s="2" t="inlineStr"/>
       <c r="AH38" s="2" t="inlineStr">
         <is>
+          <t>国家税务总局广州市番禺区税务局关于送达税务行政处罚告知书的公告</t>
+        </is>
+      </c>
+      <c r="AI38" s="2" t="inlineStr">
+        <is>
+          <t>内容不匹配</t>
+        </is>
+      </c>
+      <c r="AJ38" s="2" t="inlineStr">
+        <is>
+          <t>页面标题与正文/附件文书类型不一致,需人工复核。 Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>CASE-0b4a4519ba4f5ad9</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>DOC-5376b9bae81cfc82</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>江苏省</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>常州市</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局江苏省税务局</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>国家税务总局常州市税务局稽查局</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>常州好佳车辆配件有限公司</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>91320411094264460B</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>税务处理决定书</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>常税稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>常税稽处〔2026〕71号</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="3" t="n"/>
+      <c r="S39" s="3" t="n"/>
+      <c r="T39" s="3" t="n"/>
+      <c r="U39" s="3" t="n"/>
+      <c r="V39" s="2" t="inlineStr"/>
+      <c r="W39" s="4" t="n"/>
+      <c r="X39" s="4" t="n">
+        <v>46087</v>
+      </c>
+      <c r="Y39" s="4" t="n"/>
+      <c r="Z39" s="4" t="n">
+        <v>46229</v>
+      </c>
+      <c r="AA39" s="4" t="n">
+        <v>46250</v>
+      </c>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>仅公告送达/仅文号线索</t>
+        </is>
+      </c>
+      <c r="AC39" s="2" t="inlineStr">
+        <is>
+          <t>税务机关官网</t>
+        </is>
+      </c>
+      <c r="AD39" s="2" t="inlineStr">
+        <is>
+          <t>已核验</t>
+        </is>
+      </c>
+      <c r="AE39" s="5" t="inlineStr">
+        <is>
+          <t>打开原文</t>
+        </is>
+      </c>
+      <c r="AF39" s="5" t="inlineStr">
+        <is>
+          <t>打开附件</t>
+        </is>
+      </c>
+      <c r="AG39" s="2" t="inlineStr"/>
+      <c r="AH39" s="2" t="inlineStr">
+        <is>
           <t>国家税务总局江苏省税务局网站 通知公告 国家税务总局常州市税务局稽查局关于送达常州好佳车辆配件有限公司《税务处理决定书》的公告</t>
         </is>
       </c>
-      <c r="AI38" s="2" t="inlineStr">
+      <c r="AI39" s="2" t="inlineStr">
         <is>
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ38" s="2" t="inlineStr">
+      <c r="AJ39" s="2" t="inlineStr">
         <is>
           <t>Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ38"/>
-  <conditionalFormatting sqref="AD2:AD38">
+  <autoFilter ref="A1:AJ39"/>
+  <conditionalFormatting sqref="AD2:AD39">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$AD2="待核验"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI2:AI38">
+  <conditionalFormatting sqref="AI2:AI39">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND($AI2&lt;&gt;"正常",$AI2&lt;&gt;"附件正常")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="AD2:AD38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AD2:AD39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"已核验,待核验,人工复核完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -18524,9 +18749,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE35" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE36" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF37" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE38" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF38" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE38" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF38" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE39" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF39" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -20414,7 +20640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23243,8 +23469,261 @@
         </is>
       </c>
     </row>
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16T15:44:56+08:00</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 至 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>208</v>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>宜兴市华欧金属材料有限公司</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://qingdao.chinatax.gov.cn/bsfw2019/ssgg/sdgg/dyjcj/: HTT...</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>已完成候选发现、逐条访问核验、去重、关联和历史数据增量写入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16T15:49:43+08:00</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 至 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://qingdao.chinatax.gov.cn/bsfw2019/ssgg/sdgg/dyjcj/: HTT...</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16T15:59:45+08:00</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 至 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>常州硕策商贸有限公司</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://qingdao.chinatax.gov.cn/bsfw2019/ssgg/sdgg/dyjcj/: HTT...</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>已完成候选发现、逐条访问核验、去重、关联和历史数据增量写入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16T16:07:18+08:00</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 至 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://qingdao.chinatax.gov.cn/bsfw2019/ssgg/sdgg/dyjcj/: HTT...</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="54" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16T16:13:21+08:00</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 至 2026-08-16</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: HTTPError: 412 Client Error: Precondition Failed for url: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/ | discover_official_index: https://qingdao.chinatax.gov.cn/bsfw2019/ssgg/sdgg/dyjcj/: HTT...</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M57"/>
+  <autoFilter ref="A1:M62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-17
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -895,7 +895,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         <v>46246</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1645,7 +1645,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         <v>46249</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46242</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         <v>46242</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>46250</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         <v>46250</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>46241</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>46241</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2815,7 +2815,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
         <v>46243</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>46243</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>46236</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3813,7 +3813,7 @@
         <v>46236</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3939,7 +3939,7 @@
         <v>46238</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4065,7 +4065,7 @@
         <v>46238</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v>46238</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
         <v>46233</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         <v>46234</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4579,7 +4579,7 @@
         <v>46238</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4697,7 +4697,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         <v>46240</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5237,7 +5237,7 @@
         <v>46240</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5495,7 +5495,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5753,7 +5753,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5879,7 +5879,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6013,7 +6013,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6151,7 +6151,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6279,7 +6279,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6405,7 +6405,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6889,7 +6889,7 @@
         <v>46249</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         <v>46249</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7141,7 +7141,7 @@
         <v>46229</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7263,7 +7263,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7385,7 +7385,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
         <v>46250</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7743,7 +7743,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -8007,7 +8007,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8275,7 +8275,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8413,7 +8413,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8555,7 +8555,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8685,7 +8685,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8813,7 +8813,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
         <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9061,7 +9061,7 @@
         <v>46248</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9195,7 +9195,7 @@
         <v>46230</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9329,7 +9329,7 @@
         <v>46230</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9807,7 +9807,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9943,7 +9943,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10089,7 +10089,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         <v>46250</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10359,7 +10359,7 @@
         <v>46250</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10493,7 +10493,7 @@
         <v>46240</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10627,7 +10627,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10755,7 +10755,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
         <v>46233</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11021,7 +11021,7 @@
         <v>46234</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11157,7 +11157,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11297,7 +11297,7 @@
         <v>46240</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         <v>46240</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -11579,7 +11579,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -11713,7 +11713,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -11845,7 +11845,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -11983,7 +11983,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12115,7 +12115,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -12379,7 +12379,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -12515,7 +12515,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -12647,7 +12647,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -12785,7 +12785,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -12927,7 +12927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -13057,7 +13057,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -13185,7 +13185,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -13309,7 +13309,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         <v>46248</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -13567,7 +13567,7 @@
         <v>46230</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -13701,7 +13701,7 @@
         <v>46230</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -14113,7 +14113,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14227,7 +14227,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14467,7 +14467,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14719,7 +14719,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14845,7 +14845,7 @@
         <v>46249</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -14971,7 +14971,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15089,7 +15089,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15211,7 +15211,7 @@
         <v>46241</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
         <v>46241</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -15459,7 +15459,7 @@
         <v>46243</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -15589,7 +15589,7 @@
         <v>46243</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -15829,7 +15829,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16069,7 +16069,7 @@
         <v>46236</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16195,7 +16195,7 @@
         <v>46236</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -16447,7 +16447,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -16569,7 +16569,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>46238</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -16927,7 +16927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17049,7 +17049,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -17175,7 +17175,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -17301,7 +17301,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -17419,7 +17419,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -17541,7 +17541,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -17663,7 +17663,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -17785,7 +17785,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -17911,7 +17911,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18033,7 +18033,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -18155,7 +18155,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -18277,7 +18277,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -18395,7 +18395,7 @@
         <v>46250</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -18635,7 +18635,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19066,7 +19066,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -19184,7 +19184,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -19302,7 +19302,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -19430,7 +19430,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -19554,7 +19554,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -19678,7 +19678,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -19812,7 +19812,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -19946,7 +19946,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -20326,7 +20326,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20444,7 +20444,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -20562,7 +20562,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -20640,7 +20640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23722,8 +23722,57 @@
         </is>
       </c>
     </row>
+    <row r="63" ht="54" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17T12:54:09+08:00</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10 至 2026-08-17</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/laibin/tzgg_15610/tzgg_15611/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /laibin/tzgg_15610/tzgg_15611/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M62"/>
+  <autoFilter ref="A1:M63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-18
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -895,7 +895,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         <v>46246</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1645,7 +1645,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         <v>46249</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46242</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         <v>46242</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>46250</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         <v>46250</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>46241</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>46241</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2815,7 +2815,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
         <v>46243</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>46243</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>46236</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3813,7 +3813,7 @@
         <v>46236</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3939,7 +3939,7 @@
         <v>46238</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4065,7 +4065,7 @@
         <v>46238</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v>46238</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
         <v>46233</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         <v>46234</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4579,7 +4579,7 @@
         <v>46238</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4697,7 +4697,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         <v>46240</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5237,7 +5237,7 @@
         <v>46240</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5495,7 +5495,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5753,7 +5753,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5879,7 +5879,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6013,7 +6013,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6151,7 +6151,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6279,7 +6279,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6405,7 +6405,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6889,7 +6889,7 @@
         <v>46249</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         <v>46249</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7141,7 +7141,7 @@
         <v>46229</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7263,7 +7263,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7385,7 +7385,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
         <v>46250</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7743,7 +7743,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -8007,7 +8007,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8275,7 +8275,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8413,7 +8413,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8555,7 +8555,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8685,7 +8685,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8813,7 +8813,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
         <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9061,7 +9061,7 @@
         <v>46248</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9195,7 +9195,7 @@
         <v>46230</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9329,7 +9329,7 @@
         <v>46230</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9807,7 +9807,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9943,7 +9943,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10089,7 +10089,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         <v>46250</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10359,7 +10359,7 @@
         <v>46250</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10493,7 +10493,7 @@
         <v>46240</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10627,7 +10627,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10755,7 +10755,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
         <v>46233</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11021,7 +11021,7 @@
         <v>46234</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11157,7 +11157,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11297,7 +11297,7 @@
         <v>46240</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         <v>46240</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -11579,7 +11579,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -11713,7 +11713,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -11845,7 +11845,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -11983,7 +11983,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12115,7 +12115,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -12379,7 +12379,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -12515,7 +12515,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -12647,7 +12647,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -12785,7 +12785,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -12927,7 +12927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -13057,7 +13057,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -13185,7 +13185,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -13309,7 +13309,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         <v>46248</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -13567,7 +13567,7 @@
         <v>46230</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -13701,7 +13701,7 @@
         <v>46230</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -14113,7 +14113,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14227,7 +14227,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14467,7 +14467,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14719,7 +14719,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14845,7 +14845,7 @@
         <v>46249</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -14971,7 +14971,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15089,7 +15089,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15211,7 +15211,7 @@
         <v>46241</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
         <v>46241</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -15459,7 +15459,7 @@
         <v>46243</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -15589,7 +15589,7 @@
         <v>46243</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -15829,7 +15829,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16069,7 +16069,7 @@
         <v>46236</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16195,7 +16195,7 @@
         <v>46236</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -16447,7 +16447,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -16569,7 +16569,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>46238</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -16927,7 +16927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17049,7 +17049,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -17175,7 +17175,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -17301,7 +17301,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -17419,7 +17419,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -17541,7 +17541,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -17663,7 +17663,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -17785,7 +17785,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -17911,7 +17911,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18033,7 +18033,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -18155,7 +18155,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -18277,7 +18277,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -18395,7 +18395,7 @@
         <v>46250</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -18635,7 +18635,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19066,7 +19066,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -19184,7 +19184,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -19302,7 +19302,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -19430,7 +19430,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -19554,7 +19554,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -19678,7 +19678,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -19812,7 +19812,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -19946,7 +19946,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -20326,7 +20326,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20444,7 +20444,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -20562,7 +20562,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -20640,7 +20640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23820,8 +23820,57 @@
         </is>
       </c>
     </row>
+    <row r="65" ht="54" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18T12:47:09+08:00</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11 至 2026-08-18</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/smsswj/xxgk/sjxxgk/qtgg/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /smsswj/xxgk/sjxxgk/qtgg/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', p...</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M64"/>
+  <autoFilter ref="A1:M65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-19
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -895,7 +895,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         <v>46246</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1645,7 +1645,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         <v>46249</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46242</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         <v>46242</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>46250</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         <v>46250</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>46241</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>46241</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2815,7 +2815,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
         <v>46243</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>46243</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>46236</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3813,7 +3813,7 @@
         <v>46236</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3939,7 +3939,7 @@
         <v>46238</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4065,7 +4065,7 @@
         <v>46238</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v>46238</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
         <v>46233</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         <v>46234</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4579,7 +4579,7 @@
         <v>46238</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4697,7 +4697,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         <v>46240</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5237,7 +5237,7 @@
         <v>46240</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5495,7 +5495,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5753,7 +5753,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5879,7 +5879,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6013,7 +6013,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6151,7 +6151,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6279,7 +6279,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6405,7 +6405,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6889,7 +6889,7 @@
         <v>46249</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         <v>46249</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7141,7 +7141,7 @@
         <v>46229</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7263,7 +7263,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7385,7 +7385,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
         <v>46250</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7743,7 +7743,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -8007,7 +8007,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8275,7 +8275,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8413,7 +8413,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8555,7 +8555,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8685,7 +8685,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8813,7 +8813,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
         <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9061,7 +9061,7 @@
         <v>46248</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9195,7 +9195,7 @@
         <v>46230</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9329,7 +9329,7 @@
         <v>46230</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9807,7 +9807,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9943,7 +9943,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10089,7 +10089,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         <v>46250</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10359,7 +10359,7 @@
         <v>46250</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10493,7 +10493,7 @@
         <v>46240</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10627,7 +10627,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10755,7 +10755,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
         <v>46233</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11021,7 +11021,7 @@
         <v>46234</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11157,7 +11157,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11297,7 +11297,7 @@
         <v>46240</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         <v>46240</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -11579,7 +11579,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -11713,7 +11713,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -11845,7 +11845,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -11983,7 +11983,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12115,7 +12115,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -12379,7 +12379,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -12515,7 +12515,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -12647,7 +12647,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -12785,7 +12785,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -12927,7 +12927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -13057,7 +13057,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -13185,7 +13185,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -13309,7 +13309,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         <v>46248</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -13567,7 +13567,7 @@
         <v>46230</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -13701,7 +13701,7 @@
         <v>46230</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -14113,7 +14113,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14227,7 +14227,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14467,7 +14467,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14719,7 +14719,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14845,7 +14845,7 @@
         <v>46249</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -14971,7 +14971,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15089,7 +15089,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15211,7 +15211,7 @@
         <v>46241</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
         <v>46241</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -15459,7 +15459,7 @@
         <v>46243</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -15589,7 +15589,7 @@
         <v>46243</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -15829,7 +15829,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16069,7 +16069,7 @@
         <v>46236</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16195,7 +16195,7 @@
         <v>46236</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -16447,7 +16447,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -16569,7 +16569,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>46238</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -16927,7 +16927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17049,7 +17049,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -17175,7 +17175,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -17301,7 +17301,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -17419,7 +17419,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -17541,7 +17541,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -17663,7 +17663,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -17785,7 +17785,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -17911,7 +17911,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18033,7 +18033,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -18155,7 +18155,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -18277,7 +18277,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -18395,7 +18395,7 @@
         <v>46250</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -18635,7 +18635,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19066,7 +19066,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -19184,7 +19184,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -19302,7 +19302,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -19430,7 +19430,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -19554,7 +19554,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -19678,7 +19678,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -19812,7 +19812,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -19946,7 +19946,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -20326,7 +20326,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20444,7 +20444,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -20562,7 +20562,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -20640,7 +20640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23918,8 +23918,57 @@
         </is>
       </c>
     </row>
+    <row r="67" ht="54" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19T12:47:57+08:00</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12 至 2026-08-19</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M66"/>
+  <autoFilter ref="A1:M67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-20
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -895,7 +895,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         <v>46246</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1645,7 +1645,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         <v>46249</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46242</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         <v>46242</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>46250</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         <v>46250</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>46241</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>46241</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2815,7 +2815,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
         <v>46243</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>46243</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
         <v>46236</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3813,7 +3813,7 @@
         <v>46236</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3939,7 +3939,7 @@
         <v>46238</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4065,7 +4065,7 @@
         <v>46238</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v>46238</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
         <v>46233</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         <v>46234</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4579,7 +4579,7 @@
         <v>46238</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4697,7 +4697,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         <v>46240</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5237,7 +5237,7 @@
         <v>46240</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5495,7 +5495,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5753,7 +5753,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5879,7 +5879,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -6013,7 +6013,7 @@
         <v>46229</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6151,7 +6151,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6279,7 +6279,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6405,7 +6405,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6889,7 +6889,7 @@
         <v>46249</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         <v>46249</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7141,7 +7141,7 @@
         <v>46229</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7263,7 +7263,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7385,7 +7385,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7507,7 +7507,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
         <v>46250</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7743,7 +7743,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -8007,7 +8007,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8275,7 +8275,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8413,7 +8413,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8555,7 +8555,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8685,7 +8685,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8813,7 +8813,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
         <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9061,7 +9061,7 @@
         <v>46248</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9195,7 +9195,7 @@
         <v>46230</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9329,7 +9329,7 @@
         <v>46230</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9807,7 +9807,7 @@
         <v>46246</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -9943,7 +9943,7 @@
         <v>46242</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -10089,7 +10089,7 @@
         <v>46242</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         <v>46250</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -10359,7 +10359,7 @@
         <v>46250</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -10493,7 +10493,7 @@
         <v>46240</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -10627,7 +10627,7 @@
         <v>46238</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -10755,7 +10755,7 @@
         <v>46238</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
         <v>46233</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -11021,7 +11021,7 @@
         <v>46234</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -11157,7 +11157,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -11297,7 +11297,7 @@
         <v>46240</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         <v>46240</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -11579,7 +11579,7 @@
         <v>46229</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -11713,7 +11713,7 @@
         <v>46229</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -11845,7 +11845,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -11983,7 +11983,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -12115,7 +12115,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -12379,7 +12379,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -12515,7 +12515,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -12647,7 +12647,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -12785,7 +12785,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -12927,7 +12927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -13057,7 +13057,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -13185,7 +13185,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -13309,7 +13309,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -13433,7 +13433,7 @@
         <v>46248</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -13567,7 +13567,7 @@
         <v>46230</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -13701,7 +13701,7 @@
         <v>46230</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -14113,7 +14113,7 @@
         <v>46249</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14227,7 +14227,7 @@
         <v>46249</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         <v>46249</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14467,7 +14467,7 @@
         <v>46249</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         <v>46249</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -14719,7 +14719,7 @@
         <v>46246</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -14845,7 +14845,7 @@
         <v>46249</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -14971,7 +14971,7 @@
         <v>46249</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15089,7 +15089,7 @@
         <v>46249</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15211,7 +15211,7 @@
         <v>46241</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
         <v>46241</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -15459,7 +15459,7 @@
         <v>46243</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -15589,7 +15589,7 @@
         <v>46243</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -15829,7 +15829,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16069,7 +16069,7 @@
         <v>46236</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16195,7 +16195,7 @@
         <v>46236</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
         <v>46238</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -16447,7 +16447,7 @@
         <v>46238</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -16569,7 +16569,7 @@
         <v>46238</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -16687,7 +16687,7 @@
         <v>46238</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -16927,7 +16927,7 @@
         <v>46229</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17049,7 +17049,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -17175,7 +17175,7 @@
         <v>46229</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -17301,7 +17301,7 @@
         <v>46229</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -17419,7 +17419,7 @@
         <v>46229</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -17541,7 +17541,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -17663,7 +17663,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -17785,7 +17785,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -17911,7 +17911,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18033,7 +18033,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -18155,7 +18155,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -18277,7 +18277,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -18395,7 +18395,7 @@
         <v>46250</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -18635,7 +18635,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19066,7 +19066,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -19184,7 +19184,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -19302,7 +19302,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -19430,7 +19430,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -19554,7 +19554,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -19678,7 +19678,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -19812,7 +19812,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -19946,7 +19946,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -20326,7 +20326,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20444,7 +20444,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -20562,7 +20562,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -20640,7 +20640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24016,8 +24016,57 @@
         </is>
       </c>
     </row>
+    <row r="69" ht="54" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20T12:48:46+08:00</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 至 2026-08-20</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M68"/>
+  <autoFilter ref="A1:M69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: preserve latest scheduled run status
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -29852,7 +29852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -33530,6 +33530,54 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-20T12:48:46+08:00</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-08-13 至 2026-08-20</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>188</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
+        <v>4</v>
+      </c>
+      <c r="H75" t="n">
+        <v>3</v>
+      </c>
+      <c r="I75" t="n">
+        <v>8</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-21
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1653,7 +1653,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2141,7 +2141,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
         <v>46254</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v>46246</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3625,7 +3625,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3743,7 +3743,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3875,7 +3875,7 @@
         <v>46242</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4021,7 +4021,7 @@
         <v>46242</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         <v>46250</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
         <v>46250</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4413,7 +4413,7 @@
         <v>46241</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4535,7 +4535,7 @@
         <v>46241</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
         <v>46240</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4799,7 +4799,7 @@
         <v>46243</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4929,7 +4929,7 @@
         <v>46243</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5051,7 +5051,7 @@
         <v>46249</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5181,7 +5181,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5301,7 +5301,7 @@
         <v>46249</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         <v>46249</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5541,7 +5541,7 @@
         <v>46236</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5667,7 +5667,7 @@
         <v>46236</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5793,7 +5793,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
         <v>46238</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6049,7 +6049,7 @@
         <v>46238</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6179,7 +6179,7 @@
         <v>46233</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v>46234</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6437,7 +6437,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6563,7 +6563,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6699,7 +6699,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6961,7 +6961,7 @@
         <v>46240</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7103,7 +7103,7 @@
         <v>46240</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7225,7 +7225,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7345,7 +7345,7 @@
         <v>46254</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7485,7 +7485,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7605,7 +7605,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7737,7 +7737,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7861,7 +7861,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7987,7 +7987,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8109,7 +8109,7 @@
         <v>46254</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8231,7 +8231,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8365,7 +8365,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8503,7 +8503,7 @@
         <v>46249</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8643,7 +8643,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8769,7 +8769,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8895,7 +8895,7 @@
         <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9013,7 +9013,7 @@
         <v>46229</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9135,7 +9135,7 @@
         <v>46229</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9257,7 +9257,7 @@
         <v>46254</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9371,7 +9371,7 @@
         <v>46254</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9493,7 +9493,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9631,7 +9631,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9875,7 +9875,7 @@
         <v>46249</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10001,7 +10001,7 @@
         <v>46254</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10123,7 +10123,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10249,7 +10249,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10383,7 +10383,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10513,7 +10513,7 @@
         <v>46249</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10641,7 +10641,7 @@
         <v>46254</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10897,7 +10897,7 @@
         <v>46229</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11019,7 +11019,7 @@
         <v>46229</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11153,7 +11153,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11277,7 +11277,7 @@
         <v>46229</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11399,7 +11399,7 @@
         <v>46229</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46250</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11635,7 +11635,7 @@
         <v>46229</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11777,7 +11777,7 @@
         <v>46229</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11899,7 +11899,7 @@
         <v>46254</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12021,7 +12021,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46229</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12289,7 +12289,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46254</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
         <v>46254</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12665,7 +12665,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12807,7 +12807,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12949,7 +12949,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13091,7 +13091,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13221,7 +13221,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13349,7 +13349,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13473,7 +13473,7 @@
         <v>46229</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13597,7 +13597,7 @@
         <v>46248</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13731,7 +13731,7 @@
         <v>46230</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13865,7 +13865,7 @@
         <v>46230</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -14396,7 +14396,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14528,7 +14528,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14658,7 +14658,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14794,7 +14794,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14940,7 +14940,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -15074,7 +15074,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -15210,7 +15210,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15344,7 +15344,7 @@
         <v>46240</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15478,7 +15478,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -15736,7 +15736,7 @@
         <v>46233</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -15872,7 +15872,7 @@
         <v>46234</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -16008,7 +16008,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -16148,7 +16148,7 @@
         <v>46240</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -16290,7 +16290,7 @@
         <v>46240</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -16430,7 +16430,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16564,7 +16564,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16696,7 +16696,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -16834,7 +16834,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -16974,7 +16974,7 @@
         <v>46254</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -17104,7 +17104,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -17238,7 +17238,7 @@
         <v>46254</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -17368,7 +17368,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -17502,7 +17502,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17632,7 +17632,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -17760,7 +17760,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -17890,7 +17890,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -18028,7 +18028,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -18168,7 +18168,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -18304,7 +18304,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -18436,7 +18436,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -18574,7 +18574,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18716,7 +18716,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -18858,7 +18858,7 @@
         <v>46254</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -19000,7 +19000,7 @@
         <v>46254</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -19130,7 +19130,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -19258,7 +19258,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -19382,7 +19382,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19506,7 +19506,7 @@
         <v>46248</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -19640,7 +19640,7 @@
         <v>46230</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -19774,7 +19774,7 @@
         <v>46230</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -20209,7 +20209,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20335,7 +20335,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -20465,7 +20465,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -20595,7 +20595,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -20717,7 +20717,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -20835,7 +20835,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -20953,7 +20953,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -21077,7 +21077,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -21201,7 +21201,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -21321,7 +21321,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -21441,7 +21441,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -21561,7 +21561,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -21679,7 +21679,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -21801,7 +21801,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -21915,7 +21915,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -22033,7 +22033,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -22155,7 +22155,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -22281,7 +22281,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -22407,7 +22407,7 @@
         <v>46246</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -22533,7 +22533,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -22659,7 +22659,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -22777,7 +22777,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -22899,7 +22899,7 @@
         <v>46241</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -23021,7 +23021,7 @@
         <v>46241</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -23147,7 +23147,7 @@
         <v>46243</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -23277,7 +23277,7 @@
         <v>46243</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -23399,7 +23399,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -23517,7 +23517,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -23635,7 +23635,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -23757,7 +23757,7 @@
         <v>46236</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -23883,7 +23883,7 @@
         <v>46236</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -24009,7 +24009,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -24135,7 +24135,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -24261,7 +24261,7 @@
         <v>46238</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -24387,7 +24387,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -24509,7 +24509,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -24627,7 +24627,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -24747,7 +24747,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -24869,7 +24869,7 @@
         <v>46254</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -24991,7 +24991,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -25117,7 +25117,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -25239,7 +25239,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25361,7 +25361,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -25487,7 +25487,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -25605,7 +25605,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -25727,7 +25727,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -25849,7 +25849,7 @@
         <v>46254</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -25963,7 +25963,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -26085,7 +26085,7 @@
         <v>46254</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -26207,7 +26207,7 @@
         <v>46229</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -26329,7 +26329,7 @@
         <v>46249</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -26455,7 +26455,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -26577,7 +26577,7 @@
         <v>46254</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -26699,7 +26699,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -26821,7 +26821,7 @@
         <v>46229</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -26943,7 +26943,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -27065,7 +27065,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -27183,7 +27183,7 @@
         <v>46250</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -27301,7 +27301,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -27423,7 +27423,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -27545,7 +27545,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -27663,7 +27663,7 @@
         <v>46254</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -27783,7 +27783,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -28256,7 +28256,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28382,7 +28382,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -28500,7 +28500,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -28628,7 +28628,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -28752,7 +28752,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -28876,7 +28876,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -29010,7 +29010,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -29144,7 +29144,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -29529,7 +29529,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -29655,7 +29655,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -29773,7 +29773,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29852,7 +29852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -33530,56 +33530,106 @@
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="75" ht="54" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>2026-08-20T12:48:46+08:00</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>2026-08-13 至 2026-08-20</t>
         </is>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" s="2" t="n">
         <v>188</v>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G75" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H75" t="n">
+      <c r="H75" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I75" t="n">
+      <c r="I75" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>成功</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="54" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T12:50:23+08:00</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 至 2026-08-21</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/fangchenggang/tzgg_15261/tzgg_15262/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /fangchenggang/tzgg_15261/tzgg_15262/ (Caused by ProtocolError('Connection aborted.', Remot...</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
         <is>
           <t>本次检索未发现符合收录标准的新文书。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M74"/>
+  <autoFilter ref="A1:M76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-22
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1653,7 +1653,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2141,7 +2141,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
         <v>46254</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v>46246</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3625,7 +3625,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3743,7 +3743,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3875,7 +3875,7 @@
         <v>46242</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4021,7 +4021,7 @@
         <v>46242</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         <v>46250</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
         <v>46250</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4413,7 +4413,7 @@
         <v>46241</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4535,7 +4535,7 @@
         <v>46241</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
         <v>46240</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4799,7 +4799,7 @@
         <v>46243</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4929,7 +4929,7 @@
         <v>46243</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5051,7 +5051,7 @@
         <v>46249</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5181,7 +5181,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5301,7 +5301,7 @@
         <v>46249</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         <v>46249</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5541,7 +5541,7 @@
         <v>46236</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5667,7 +5667,7 @@
         <v>46236</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5793,7 +5793,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
         <v>46238</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6049,7 +6049,7 @@
         <v>46238</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6179,7 +6179,7 @@
         <v>46233</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v>46234</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6437,7 +6437,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6563,7 +6563,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6699,7 +6699,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6961,7 +6961,7 @@
         <v>46240</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7103,7 +7103,7 @@
         <v>46240</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7225,7 +7225,7 @@
         <v>46229</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7345,7 +7345,7 @@
         <v>46254</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7485,7 +7485,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7605,7 +7605,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7737,7 +7737,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7861,7 +7861,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7987,7 +7987,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8109,7 +8109,7 @@
         <v>46254</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8231,7 +8231,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8365,7 +8365,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8503,7 +8503,7 @@
         <v>46249</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8643,7 +8643,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8769,7 +8769,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8895,7 +8895,7 @@
         <v>46229</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9013,7 +9013,7 @@
         <v>46229</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9135,7 +9135,7 @@
         <v>46229</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9257,7 +9257,7 @@
         <v>46254</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9371,7 +9371,7 @@
         <v>46254</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9493,7 +9493,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9631,7 +9631,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9875,7 +9875,7 @@
         <v>46249</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10001,7 +10001,7 @@
         <v>46254</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10123,7 +10123,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10249,7 +10249,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10383,7 +10383,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10513,7 +10513,7 @@
         <v>46249</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10641,7 +10641,7 @@
         <v>46254</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10897,7 +10897,7 @@
         <v>46229</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11019,7 +11019,7 @@
         <v>46229</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11153,7 +11153,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11277,7 +11277,7 @@
         <v>46229</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11399,7 +11399,7 @@
         <v>46229</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46250</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11635,7 +11635,7 @@
         <v>46229</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11777,7 +11777,7 @@
         <v>46229</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11899,7 +11899,7 @@
         <v>46254</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12021,7 +12021,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46229</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12289,7 +12289,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46254</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
         <v>46254</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12665,7 +12665,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12807,7 +12807,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12949,7 +12949,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13091,7 +13091,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13221,7 +13221,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13349,7 +13349,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13473,7 +13473,7 @@
         <v>46229</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13597,7 +13597,7 @@
         <v>46248</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13731,7 +13731,7 @@
         <v>46230</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13865,7 +13865,7 @@
         <v>46230</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -14396,7 +14396,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14528,7 +14528,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14658,7 +14658,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -14794,7 +14794,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -14940,7 +14940,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -15074,7 +15074,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -15210,7 +15210,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15344,7 +15344,7 @@
         <v>46240</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15478,7 +15478,7 @@
         <v>46238</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
         <v>46238</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -15736,7 +15736,7 @@
         <v>46233</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -15872,7 +15872,7 @@
         <v>46234</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -16008,7 +16008,7 @@
         <v>46238</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -16148,7 +16148,7 @@
         <v>46240</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -16290,7 +16290,7 @@
         <v>46240</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -16430,7 +16430,7 @@
         <v>46229</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16564,7 +16564,7 @@
         <v>46229</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16696,7 +16696,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -16834,7 +16834,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -16974,7 +16974,7 @@
         <v>46254</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -17104,7 +17104,7 @@
         <v>46229</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -17238,7 +17238,7 @@
         <v>46254</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -17368,7 +17368,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -17502,7 +17502,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17632,7 +17632,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -17760,7 +17760,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -17890,7 +17890,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -18028,7 +18028,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -18168,7 +18168,7 @@
         <v>46229</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -18304,7 +18304,7 @@
         <v>46229</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -18436,7 +18436,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -18574,7 +18574,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18716,7 +18716,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -18858,7 +18858,7 @@
         <v>46254</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -19000,7 +19000,7 @@
         <v>46254</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -19130,7 +19130,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -19258,7 +19258,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -19382,7 +19382,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19506,7 +19506,7 @@
         <v>46248</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -19640,7 +19640,7 @@
         <v>46230</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -19774,7 +19774,7 @@
         <v>46230</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -20209,7 +20209,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20335,7 +20335,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -20465,7 +20465,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -20595,7 +20595,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -20717,7 +20717,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -20835,7 +20835,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -20953,7 +20953,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -21077,7 +21077,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -21201,7 +21201,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -21321,7 +21321,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -21441,7 +21441,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -21561,7 +21561,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -21679,7 +21679,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -21801,7 +21801,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -21915,7 +21915,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -22033,7 +22033,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -22155,7 +22155,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -22281,7 +22281,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -22407,7 +22407,7 @@
         <v>46246</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -22533,7 +22533,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -22659,7 +22659,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -22777,7 +22777,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -22899,7 +22899,7 @@
         <v>46241</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -23021,7 +23021,7 @@
         <v>46241</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -23147,7 +23147,7 @@
         <v>46243</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -23277,7 +23277,7 @@
         <v>46243</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -23399,7 +23399,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -23517,7 +23517,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -23635,7 +23635,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -23757,7 +23757,7 @@
         <v>46236</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -23883,7 +23883,7 @@
         <v>46236</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -24009,7 +24009,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -24135,7 +24135,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -24261,7 +24261,7 @@
         <v>46238</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -24387,7 +24387,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -24509,7 +24509,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -24627,7 +24627,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -24747,7 +24747,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -24869,7 +24869,7 @@
         <v>46254</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -24991,7 +24991,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -25117,7 +25117,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -25239,7 +25239,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25361,7 +25361,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -25487,7 +25487,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -25605,7 +25605,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -25727,7 +25727,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -25849,7 +25849,7 @@
         <v>46254</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -25963,7 +25963,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -26085,7 +26085,7 @@
         <v>46254</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -26207,7 +26207,7 @@
         <v>46229</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -26329,7 +26329,7 @@
         <v>46249</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -26455,7 +26455,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -26577,7 +26577,7 @@
         <v>46254</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -26699,7 +26699,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -26821,7 +26821,7 @@
         <v>46229</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -26943,7 +26943,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -27065,7 +27065,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -27183,7 +27183,7 @@
         <v>46250</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -27301,7 +27301,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -27423,7 +27423,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -27545,7 +27545,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -27663,7 +27663,7 @@
         <v>46254</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -27783,7 +27783,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -28256,7 +28256,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28382,7 +28382,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -28500,7 +28500,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -28628,7 +28628,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -28752,7 +28752,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -28876,7 +28876,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -29010,7 +29010,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -29144,7 +29144,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -29529,7 +29529,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -29655,7 +29655,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -29773,7 +29773,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29852,7 +29852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M77"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -33677,8 +33677,57 @@
         </is>
       </c>
     </row>
+    <row r="78" ht="54" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22T12:44:10+08:00</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15 至 2026-08-22</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>189</v>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M77"/>
+  <autoFilter ref="A1:M78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-23
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -4461,7 +4461,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ31" s="2" t="inlineStr"/>
+      <c r="AJ31" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -4593,7 +4597,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ32" s="2" t="inlineStr"/>
+      <c r="AJ32" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -15646,7 +15654,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -15778,7 +15790,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -30384,7 +30400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34360,8 +34376,57 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="54" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23T13:09:49+08:00</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16 至 2026-08-23</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M80"/>
+  <autoFilter ref="A1:M81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-24
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1653,7 +1653,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2141,7 +2141,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2855,7 +2855,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
         <v>46254</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v>46246</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3625,7 +3625,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3743,7 +3743,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3875,7 +3875,7 @@
         <v>46242</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -4021,7 +4021,7 @@
         <v>46242</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         <v>46250</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
         <v>46250</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4427,7 +4427,7 @@
         <v>46257</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4563,7 +4563,7 @@
         <v>46257</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4685,7 +4685,7 @@
         <v>46241</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4807,7 +4807,7 @@
         <v>46241</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4941,7 +4941,7 @@
         <v>46240</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5071,7 +5071,7 @@
         <v>46243</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5201,7 +5201,7 @@
         <v>46243</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
         <v>46249</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5453,7 +5453,7 @@
         <v>46238</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v>46249</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5691,7 +5691,7 @@
         <v>46249</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5813,7 +5813,7 @@
         <v>46236</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5939,7 +5939,7 @@
         <v>46236</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6065,7 +6065,7 @@
         <v>46238</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         <v>46238</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6321,7 +6321,7 @@
         <v>46238</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6451,7 +6451,7 @@
         <v>46233</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6587,7 +6587,7 @@
         <v>46234</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6709,7 +6709,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6835,7 +6835,7 @@
         <v>46238</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6971,7 +6971,7 @@
         <v>46238</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7095,7 +7095,7 @@
         <v>46229</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7233,7 +7233,7 @@
         <v>46240</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
         <v>46240</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7497,7 +7497,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7617,7 +7617,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7757,7 +7757,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7877,7 +7877,7 @@
         <v>46254</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -8009,7 +8009,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8133,7 +8133,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8259,7 +8259,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8381,7 +8381,7 @@
         <v>46254</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8503,7 +8503,7 @@
         <v>46254</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8637,7 +8637,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8775,7 +8775,7 @@
         <v>46249</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8915,7 +8915,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9041,7 +9041,7 @@
         <v>46229</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9167,7 +9167,7 @@
         <v>46229</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9285,7 +9285,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9407,7 +9407,7 @@
         <v>46229</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9529,7 +9529,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9643,7 +9643,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9765,7 +9765,7 @@
         <v>46254</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9903,7 +9903,7 @@
         <v>46254</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10025,7 +10025,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10147,7 +10147,7 @@
         <v>46249</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10395,7 +10395,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10521,7 +10521,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
         <v>46254</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10785,7 +10785,7 @@
         <v>46249</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10913,7 +10913,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11043,7 +11043,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11169,7 +11169,7 @@
         <v>46229</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11291,7 +11291,7 @@
         <v>46229</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11425,7 +11425,7 @@
         <v>46254</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11549,7 +11549,7 @@
         <v>46229</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11671,7 +11671,7 @@
         <v>46229</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11789,7 +11789,7 @@
         <v>46250</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11907,7 +11907,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12049,7 +12049,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12171,7 +12171,7 @@
         <v>46254</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12293,7 +12293,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12429,7 +12429,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12561,7 +12561,7 @@
         <v>46229</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12675,7 +12675,7 @@
         <v>46254</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12795,7 +12795,7 @@
         <v>46254</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12937,7 +12937,7 @@
         <v>46229</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13079,7 +13079,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13221,7 +13221,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13363,7 +13363,7 @@
         <v>46254</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13493,7 +13493,7 @@
         <v>46229</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13621,7 +13621,7 @@
         <v>46229</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13745,7 +13745,7 @@
         <v>46229</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13869,7 +13869,7 @@
         <v>46248</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -14003,7 +14003,7 @@
         <v>46230</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -14137,7 +14137,7 @@
         <v>46230</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14670,7 +14670,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -14802,7 +14802,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -14932,7 +14932,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -15068,7 +15068,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -15214,7 +15214,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -15348,7 +15348,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -15484,7 +15484,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -15620,7 +15620,7 @@
         <v>46257</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -15756,7 +15756,7 @@
         <v>46257</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -15890,7 +15890,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -16024,7 +16024,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -16152,7 +16152,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -16282,7 +16282,7 @@
         <v>46233</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -16418,7 +16418,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -16554,7 +16554,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -16694,7 +16694,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -16836,7 +16836,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -16976,7 +16976,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -17110,7 +17110,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -17242,7 +17242,7 @@
         <v>46229</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -17380,7 +17380,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -17520,7 +17520,7 @@
         <v>46254</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -17650,7 +17650,7 @@
         <v>46229</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -17784,7 +17784,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -17914,7 +17914,7 @@
         <v>46254</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -18048,7 +18048,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -18178,7 +18178,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -18306,7 +18306,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -18436,7 +18436,7 @@
         <v>46254</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -18574,7 +18574,7 @@
         <v>46254</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -18714,7 +18714,7 @@
         <v>46229</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -18850,7 +18850,7 @@
         <v>46229</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -18982,7 +18982,7 @@
         <v>46229</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -19120,7 +19120,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -19262,7 +19262,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -19404,7 +19404,7 @@
         <v>46254</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -19546,7 +19546,7 @@
         <v>46254</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -19676,7 +19676,7 @@
         <v>46229</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -19804,7 +19804,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -19928,7 +19928,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -20052,7 +20052,7 @@
         <v>46248</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -20186,7 +20186,7 @@
         <v>46230</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -20320,7 +20320,7 @@
         <v>46230</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -20757,7 +20757,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -20883,7 +20883,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -21013,7 +21013,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -21143,7 +21143,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -21265,7 +21265,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -21383,7 +21383,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -21501,7 +21501,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -21625,7 +21625,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -21749,7 +21749,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -21869,7 +21869,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -21989,7 +21989,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -22109,7 +22109,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -22227,7 +22227,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -22349,7 +22349,7 @@
         <v>46249</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -22463,7 +22463,7 @@
         <v>46249</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -22581,7 +22581,7 @@
         <v>46249</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -22703,7 +22703,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -22829,7 +22829,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -22955,7 +22955,7 @@
         <v>46246</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -23081,7 +23081,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -23207,7 +23207,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -23325,7 +23325,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>46241</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -23569,7 +23569,7 @@
         <v>46241</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -23695,7 +23695,7 @@
         <v>46243</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -23825,7 +23825,7 @@
         <v>46243</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -23947,7 +23947,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -24065,7 +24065,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -24183,7 +24183,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -24305,7 +24305,7 @@
         <v>46236</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -24431,7 +24431,7 @@
         <v>46236</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -24557,7 +24557,7 @@
         <v>46238</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -24683,7 +24683,7 @@
         <v>46238</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -24809,7 +24809,7 @@
         <v>46238</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -24935,7 +24935,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -25057,7 +25057,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -25175,7 +25175,7 @@
         <v>46229</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -25295,7 +25295,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -25417,7 +25417,7 @@
         <v>46254</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -25539,7 +25539,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -25665,7 +25665,7 @@
         <v>46229</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -25787,7 +25787,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25909,7 +25909,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -26035,7 +26035,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -26153,7 +26153,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -26275,7 +26275,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -26397,7 +26397,7 @@
         <v>46254</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -26511,7 +26511,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -26633,7 +26633,7 @@
         <v>46254</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -26755,7 +26755,7 @@
         <v>46229</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -26877,7 +26877,7 @@
         <v>46249</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -27003,7 +27003,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -27125,7 +27125,7 @@
         <v>46254</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -27247,7 +27247,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -27369,7 +27369,7 @@
         <v>46229</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -27491,7 +27491,7 @@
         <v>46229</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -27613,7 +27613,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -27731,7 +27731,7 @@
         <v>46250</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -27849,7 +27849,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -27971,7 +27971,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -28093,7 +28093,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -28211,7 +28211,7 @@
         <v>46254</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -28331,7 +28331,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -28804,7 +28804,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28930,7 +28930,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -29048,7 +29048,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29176,7 +29176,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -29300,7 +29300,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -29424,7 +29424,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -29558,7 +29558,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -29692,7 +29692,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -30077,7 +30077,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -30203,7 +30203,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -30321,7 +30321,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -30400,7 +30400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34425,8 +34425,57 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="54" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24T12:56:56+08:00</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17 至 2026-08-24</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/fangchenggang/tzgg_15261/tzgg_15262/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /fangchenggang/tzgg_15261/tzgg_15262/ (Caused by ProtocolError('Connection aborted.', Remot...</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M81"/>
+  <autoFilter ref="A1:M82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-25
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>46258</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46258</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>46254</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3221,7 +3221,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         <v>46246</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>46246</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>46249</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -3987,7 +3987,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>46242</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
         <v>46242</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>46250</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         <v>46250</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4789,7 +4789,7 @@
         <v>46257</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4925,7 +4925,7 @@
         <v>46257</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>46241</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         <v>46241</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         <v>46240</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         <v>46243</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         <v>46243</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5677,7 +5677,7 @@
         <v>46249</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         <v>46249</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
         <v>46236</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>46236</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6675,7 +6675,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>46233</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         <v>46234</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         <v>46238</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7325,7 +7325,7 @@
         <v>46238</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>46240</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
         <v>46240</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7847,7 +7847,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
         <v>46254</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8743,7 +8743,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
         <v>46258</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -8999,7 +8999,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9121,7 +9121,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9393,7 +9393,7 @@
         <v>46249</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9533,7 +9533,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         <v>46229</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9899,7 +9899,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10143,7 +10143,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10257,7 +10257,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10379,7 +10379,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
         <v>46229</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10757,7 +10757,7 @@
         <v>46249</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10883,7 +10883,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11005,7 +11005,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11131,7 +11131,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11265,7 +11265,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11395,7 +11395,7 @@
         <v>46249</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46258</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11645,7 +11645,7 @@
         <v>46254</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11775,7 +11775,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46254</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12521,7 +12521,7 @@
         <v>46250</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12639,7 +12639,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12903,7 +12903,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13025,7 +13025,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13407,7 +13407,7 @@
         <v>46254</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13541,7 +13541,7 @@
         <v>46258</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13683,7 +13683,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13825,7 +13825,7 @@
         <v>46229</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13967,7 +13967,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -14109,7 +14109,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         <v>46254</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -14507,7 +14507,7 @@
         <v>46258</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14631,7 +14631,7 @@
         <v>46229</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14755,7 +14755,7 @@
         <v>46229</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14879,7 @@
         <v>46248</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         <v>46230</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -15147,7 +15147,7 @@
         <v>46230</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15690,7 +15690,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15822,7 +15822,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15952,7 +15952,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -16088,7 +16088,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -16234,7 +16234,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -16368,7 +16368,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -16640,7 +16640,7 @@
         <v>46257</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -16776,7 +16776,7 @@
         <v>46257</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -16910,7 +16910,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -17044,7 +17044,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -17302,7 +17302,7 @@
         <v>46233</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -17438,7 +17438,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -17714,7 +17714,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -17856,7 +17856,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -17996,7 +17996,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -18130,7 +18130,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>46258</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>46258</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -18530,7 +18530,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -18668,7 +18668,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -18938,7 +18938,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -19072,7 +19072,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -19336,7 +19336,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -19466,7 +19466,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -19588,7 +19588,7 @@
         <v>46258</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -19716,7 +19716,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -19846,7 +19846,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -19984,7 +19984,7 @@
         <v>46254</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -20124,7 +20124,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -20260,7 +20260,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20668,7 +20668,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -20952,7 +20952,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -21094,7 +21094,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -21236,7 +21236,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -21366,7 +21366,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -21492,7 +21492,7 @@
         <v>46258</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -21616,7 +21616,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -21740,7 +21740,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -21864,7 +21864,7 @@
         <v>46248</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -21998,7 +21998,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -22132,7 +22132,7 @@
         <v>46230</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -22573,7 +22573,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -22825,7 +22825,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -22951,7 +22951,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -23077,7 +23077,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -23203,7 +23203,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -23325,7 +23325,7 @@
         <v>46258</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -23569,7 +23569,7 @@
         <v>46258</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -23687,7 +23687,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -23811,7 +23811,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -23935,7 +23935,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -24055,7 +24055,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -24175,7 +24175,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -24295,7 +24295,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -24413,7 +24413,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -24535,7 +24535,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -24649,7 +24649,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24889,7 +24889,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -25015,7 +25015,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -25137,7 +25137,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -25263,7 +25263,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -25389,7 +25389,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -25507,7 +25507,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -25629,7 +25629,7 @@
         <v>46241</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -25751,7 +25751,7 @@
         <v>46241</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -25873,7 +25873,7 @@
         <v>46243</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -25999,7 +25999,7 @@
         <v>46243</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -26121,7 +26121,7 @@
         <v>46249</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -26239,7 +26239,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -26357,7 +26357,7 @@
         <v>46249</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -26479,7 +26479,7 @@
         <v>46236</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -26605,7 +26605,7 @@
         <v>46236</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -26731,7 +26731,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -26857,7 +26857,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         <v>46238</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -27109,7 +27109,7 @@
         <v>46238</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -27227,7 +27227,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -27345,7 +27345,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -27465,7 +27465,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -27587,7 +27587,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -27709,7 +27709,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -28079,7 +28079,7 @@
         <v>46254</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -28201,7 +28201,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -28441,7 +28441,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28563,7 +28563,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -28677,7 +28677,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -28799,7 +28799,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -28921,7 +28921,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46249</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -29165,7 +29165,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -29287,7 +29287,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -29409,7 +29409,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -29653,7 +29653,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -29775,7 +29775,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -29893,7 +29893,7 @@
         <v>46250</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -30011,7 +30011,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -30133,7 +30133,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -30255,7 +30255,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30373,7 +30373,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -30844,7 +30844,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -30970,7 +30970,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31088,7 +31088,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31216,7 +31216,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31340,7 +31340,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -31464,7 +31464,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -31732,7 +31732,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -32117,7 +32117,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32243,7 +32243,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32361,7 +32361,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32440,7 +32440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M85"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36665,8 +36665,57 @@
         </is>
       </c>
     </row>
+    <row r="86" ht="54" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25T12:50:03+08:00</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18 至 2026-08-25</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>203</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/hechi/tzgg_15562/tzgg_15563/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /hechi/tzgg_15562/tzgg_15563/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('R...</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M85"/>
+  <autoFilter ref="A1:M86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-26
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>46258</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46258</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>46254</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3221,7 +3221,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         <v>46246</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>46246</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>46249</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -3987,7 +3987,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>46242</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
         <v>46242</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>46250</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         <v>46250</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4789,7 +4789,7 @@
         <v>46257</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4925,7 +4925,7 @@
         <v>46257</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>46241</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         <v>46241</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         <v>46240</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         <v>46243</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         <v>46243</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5677,7 +5677,7 @@
         <v>46249</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         <v>46249</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
         <v>46236</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>46236</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6675,7 +6675,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>46233</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         <v>46234</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         <v>46238</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7325,7 +7325,7 @@
         <v>46238</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>46240</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
         <v>46240</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7847,7 +7847,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
         <v>46254</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8743,7 +8743,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
         <v>46258</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -8999,7 +8999,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9121,7 +9121,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9393,7 +9393,7 @@
         <v>46249</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9533,7 +9533,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         <v>46229</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9899,7 +9899,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10143,7 +10143,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10257,7 +10257,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10379,7 +10379,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
         <v>46229</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10757,7 +10757,7 @@
         <v>46249</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10883,7 +10883,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11005,7 +11005,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11131,7 +11131,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11265,7 +11265,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11395,7 +11395,7 @@
         <v>46249</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46258</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11645,7 +11645,7 @@
         <v>46254</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11775,7 +11775,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46254</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12521,7 +12521,7 @@
         <v>46250</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12639,7 +12639,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12903,7 +12903,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13025,7 +13025,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13407,7 +13407,7 @@
         <v>46254</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13541,7 +13541,7 @@
         <v>46258</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13683,7 +13683,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13825,7 +13825,7 @@
         <v>46229</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13967,7 +13967,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -14109,7 +14109,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         <v>46254</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -14507,7 +14507,7 @@
         <v>46258</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14631,7 +14631,7 @@
         <v>46229</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14755,7 +14755,7 @@
         <v>46229</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14879,7 @@
         <v>46248</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         <v>46230</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -15147,7 +15147,7 @@
         <v>46230</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15690,7 +15690,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15822,7 +15822,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15952,7 +15952,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -16088,7 +16088,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -16234,7 +16234,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -16368,7 +16368,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -16640,7 +16640,7 @@
         <v>46257</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -16776,7 +16776,7 @@
         <v>46257</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -16910,7 +16910,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -17044,7 +17044,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -17302,7 +17302,7 @@
         <v>46233</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -17438,7 +17438,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -17714,7 +17714,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -17856,7 +17856,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -17996,7 +17996,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -18130,7 +18130,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>46258</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>46258</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -18530,7 +18530,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -18668,7 +18668,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -18938,7 +18938,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -19072,7 +19072,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -19336,7 +19336,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -19466,7 +19466,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -19588,7 +19588,7 @@
         <v>46258</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -19716,7 +19716,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -19846,7 +19846,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -19984,7 +19984,7 @@
         <v>46254</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -20124,7 +20124,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -20260,7 +20260,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20668,7 +20668,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -20952,7 +20952,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -21094,7 +21094,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -21236,7 +21236,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -21366,7 +21366,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -21492,7 +21492,7 @@
         <v>46258</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -21616,7 +21616,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -21740,7 +21740,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -21864,7 +21864,7 @@
         <v>46248</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -21998,7 +21998,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -22132,7 +22132,7 @@
         <v>46230</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -22573,7 +22573,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -22825,7 +22825,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -22951,7 +22951,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -23077,7 +23077,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -23203,7 +23203,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -23325,7 +23325,7 @@
         <v>46258</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -23569,7 +23569,7 @@
         <v>46258</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -23687,7 +23687,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -23811,7 +23811,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -23935,7 +23935,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -24055,7 +24055,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -24175,7 +24175,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -24295,7 +24295,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -24413,7 +24413,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -24535,7 +24535,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -24649,7 +24649,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24889,7 +24889,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -25015,7 +25015,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -25137,7 +25137,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -25263,7 +25263,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -25389,7 +25389,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -25507,7 +25507,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -25629,7 +25629,7 @@
         <v>46241</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -25751,7 +25751,7 @@
         <v>46241</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -25873,7 +25873,7 @@
         <v>46243</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -25999,7 +25999,7 @@
         <v>46243</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -26121,7 +26121,7 @@
         <v>46249</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -26239,7 +26239,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -26357,7 +26357,7 @@
         <v>46249</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -26479,7 +26479,7 @@
         <v>46236</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -26605,7 +26605,7 @@
         <v>46236</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -26731,7 +26731,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -26857,7 +26857,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         <v>46238</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -27109,7 +27109,7 @@
         <v>46238</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -27227,7 +27227,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -27345,7 +27345,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -27465,7 +27465,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -27587,7 +27587,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -27709,7 +27709,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -28079,7 +28079,7 @@
         <v>46254</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -28201,7 +28201,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -28441,7 +28441,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28563,7 +28563,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -28677,7 +28677,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -28799,7 +28799,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -28921,7 +28921,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46249</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -29165,7 +29165,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -29287,7 +29287,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -29409,7 +29409,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -29653,7 +29653,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -29775,7 +29775,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -29893,7 +29893,7 @@
         <v>46250</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -30011,7 +30011,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -30133,7 +30133,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -30255,7 +30255,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30373,7 +30373,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -30844,7 +30844,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -30970,7 +30970,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31088,7 +31088,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31216,7 +31216,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31340,7 +31340,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -31464,7 +31464,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -31732,7 +31732,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -32117,7 +32117,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32243,7 +32243,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32361,7 +32361,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32440,7 +32440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36763,8 +36763,57 @@
         </is>
       </c>
     </row>
+    <row r="88" ht="54" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26T12:51:38+08:00</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19 至 2026-08-26</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>225</v>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/hechi/tzgg_15562/tzgg_15563/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /hechi/tzgg_15562/tzgg_15563/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('R...</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M87"/>
+  <autoFilter ref="A1:M88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-27
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>46258</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46258</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>46254</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3221,7 +3221,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         <v>46246</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>46246</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>46249</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -3987,7 +3987,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>46242</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
         <v>46242</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>46250</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         <v>46250</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4789,7 +4789,7 @@
         <v>46257</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4925,7 +4925,7 @@
         <v>46257</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>46241</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         <v>46241</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         <v>46240</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         <v>46243</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         <v>46243</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5677,7 +5677,7 @@
         <v>46249</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         <v>46249</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
         <v>46236</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>46236</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6675,7 +6675,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>46233</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         <v>46234</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         <v>46238</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7325,7 +7325,7 @@
         <v>46238</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>46240</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
         <v>46240</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7847,7 +7847,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
         <v>46254</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8743,7 +8743,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
         <v>46258</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -8999,7 +8999,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9121,7 +9121,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9393,7 +9393,7 @@
         <v>46249</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9533,7 +9533,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         <v>46229</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9899,7 +9899,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10143,7 +10143,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10257,7 +10257,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10379,7 +10379,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
         <v>46229</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10757,7 +10757,7 @@
         <v>46249</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10883,7 +10883,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11005,7 +11005,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11131,7 +11131,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11265,7 +11265,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11395,7 +11395,7 @@
         <v>46249</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46258</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11645,7 +11645,7 @@
         <v>46254</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11775,7 +11775,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46254</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12521,7 +12521,7 @@
         <v>46250</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12639,7 +12639,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12903,7 +12903,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13025,7 +13025,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13407,7 +13407,7 @@
         <v>46254</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13541,7 +13541,7 @@
         <v>46258</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13683,7 +13683,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13825,7 +13825,7 @@
         <v>46229</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13967,7 +13967,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -14109,7 +14109,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         <v>46254</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -14507,7 +14507,7 @@
         <v>46258</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14631,7 +14631,7 @@
         <v>46229</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14755,7 +14755,7 @@
         <v>46229</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14879,7 @@
         <v>46248</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         <v>46230</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -15147,7 +15147,7 @@
         <v>46230</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15690,7 +15690,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15822,7 +15822,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15952,7 +15952,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -16088,7 +16088,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -16234,7 +16234,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -16368,7 +16368,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -16640,7 +16640,7 @@
         <v>46257</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -16776,7 +16776,7 @@
         <v>46257</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -16910,7 +16910,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -17044,7 +17044,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -17302,7 +17302,7 @@
         <v>46233</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -17438,7 +17438,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -17714,7 +17714,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -17856,7 +17856,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -17996,7 +17996,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -18130,7 +18130,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>46258</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>46258</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -18530,7 +18530,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -18668,7 +18668,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -18938,7 +18938,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -19072,7 +19072,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -19336,7 +19336,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -19466,7 +19466,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -19588,7 +19588,7 @@
         <v>46258</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -19716,7 +19716,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -19846,7 +19846,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -19984,7 +19984,7 @@
         <v>46254</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -20124,7 +20124,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -20260,7 +20260,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20668,7 +20668,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -20952,7 +20952,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -21094,7 +21094,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -21236,7 +21236,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -21366,7 +21366,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -21492,7 +21492,7 @@
         <v>46258</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -21616,7 +21616,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -21740,7 +21740,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -21864,7 +21864,7 @@
         <v>46248</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -21998,7 +21998,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -22132,7 +22132,7 @@
         <v>46230</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -22573,7 +22573,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -22825,7 +22825,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -22951,7 +22951,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -23077,7 +23077,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -23203,7 +23203,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -23325,7 +23325,7 @@
         <v>46258</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -23569,7 +23569,7 @@
         <v>46258</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -23687,7 +23687,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -23811,7 +23811,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -23935,7 +23935,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -24055,7 +24055,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -24175,7 +24175,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -24295,7 +24295,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -24413,7 +24413,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -24535,7 +24535,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -24649,7 +24649,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24889,7 +24889,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -25015,7 +25015,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -25137,7 +25137,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -25263,7 +25263,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -25389,7 +25389,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -25507,7 +25507,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -25629,7 +25629,7 @@
         <v>46241</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -25751,7 +25751,7 @@
         <v>46241</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -25873,7 +25873,7 @@
         <v>46243</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -25999,7 +25999,7 @@
         <v>46243</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -26121,7 +26121,7 @@
         <v>46249</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -26239,7 +26239,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -26357,7 +26357,7 @@
         <v>46249</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -26479,7 +26479,7 @@
         <v>46236</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -26605,7 +26605,7 @@
         <v>46236</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -26731,7 +26731,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -26857,7 +26857,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         <v>46238</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -27109,7 +27109,7 @@
         <v>46238</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -27227,7 +27227,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -27345,7 +27345,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -27465,7 +27465,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -27587,7 +27587,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -27709,7 +27709,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -28079,7 +28079,7 @@
         <v>46254</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -28201,7 +28201,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -28441,7 +28441,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28563,7 +28563,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -28677,7 +28677,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -28799,7 +28799,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -28921,7 +28921,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46249</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -29165,7 +29165,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -29287,7 +29287,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -29409,7 +29409,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -29653,7 +29653,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -29775,7 +29775,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -29893,7 +29893,7 @@
         <v>46250</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -30011,7 +30011,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -30133,7 +30133,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -30255,7 +30255,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30373,7 +30373,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -30844,7 +30844,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -30970,7 +30970,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31088,7 +31088,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31216,7 +31216,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31340,7 +31340,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -31464,7 +31464,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -31732,7 +31732,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -32117,7 +32117,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32243,7 +32243,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32361,7 +32361,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32440,7 +32440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:M90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36861,8 +36861,57 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="54" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27T23:09:07+08:00</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20 至 2026-08-27</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>254</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M89"/>
+  <autoFilter ref="A1:M90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-28
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -32440,7 +32440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M90"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36910,8 +36910,57 @@
         </is>
       </c>
     </row>
+    <row r="91" ht="54" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27T23:36:34+08:00</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20 至 2026-08-27</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>244</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/fangchenggang/tzgg_15261/tzgg_15262/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /fangchenggang/tzgg_15261/tzgg_15262/ (Caused by ProtocolError('Connection aborted.', Remot...</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M90"/>
+  <autoFilter ref="A1:M91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: pin updater timestamps to Shanghai timezone
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>46258</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46258</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>46254</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3221,7 +3221,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         <v>46246</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>46246</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>46249</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -3987,7 +3987,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>46242</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
         <v>46242</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>46250</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         <v>46250</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4789,7 +4789,7 @@
         <v>46257</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4925,7 +4925,7 @@
         <v>46257</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>46241</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         <v>46241</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         <v>46240</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         <v>46243</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         <v>46243</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5677,7 +5677,7 @@
         <v>46249</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         <v>46249</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
         <v>46236</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>46236</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6675,7 +6675,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>46233</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         <v>46234</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         <v>46238</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7325,7 +7325,7 @@
         <v>46238</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>46240</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
         <v>46240</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7847,7 +7847,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
         <v>46254</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8743,7 +8743,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
         <v>46258</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -8999,7 +8999,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9121,7 +9121,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9393,7 +9393,7 @@
         <v>46249</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9533,7 +9533,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         <v>46229</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9899,7 +9899,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10143,7 +10143,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10257,7 +10257,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10379,7 +10379,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
         <v>46229</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10757,7 +10757,7 @@
         <v>46249</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10883,7 +10883,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11005,7 +11005,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11131,7 +11131,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11265,7 +11265,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11395,7 +11395,7 @@
         <v>46249</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46258</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11645,7 +11645,7 @@
         <v>46254</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11775,7 +11775,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46254</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12521,7 +12521,7 @@
         <v>46250</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12639,7 +12639,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12903,7 +12903,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13025,7 +13025,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13407,7 +13407,7 @@
         <v>46254</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13541,7 +13541,7 @@
         <v>46258</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13683,7 +13683,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13825,7 +13825,7 @@
         <v>46229</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13967,7 +13967,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -14109,7 +14109,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         <v>46254</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -14507,7 +14507,7 @@
         <v>46258</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14631,7 +14631,7 @@
         <v>46229</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14755,7 +14755,7 @@
         <v>46229</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14879,7 @@
         <v>46248</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         <v>46230</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -15147,7 +15147,7 @@
         <v>46230</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15690,7 +15690,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15822,7 +15822,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15952,7 +15952,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -16088,7 +16088,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -16234,7 +16234,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -16368,7 +16368,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -16640,7 +16640,7 @@
         <v>46257</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -16776,7 +16776,7 @@
         <v>46257</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -16910,7 +16910,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -17044,7 +17044,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -17302,7 +17302,7 @@
         <v>46233</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -17438,7 +17438,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -17714,7 +17714,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -17856,7 +17856,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -17996,7 +17996,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -18130,7 +18130,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>46258</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>46258</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -18530,7 +18530,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -18668,7 +18668,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -18938,7 +18938,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -19072,7 +19072,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -19336,7 +19336,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -19466,7 +19466,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -19588,7 +19588,7 @@
         <v>46258</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -19716,7 +19716,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -19846,7 +19846,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -19984,7 +19984,7 @@
         <v>46254</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -20124,7 +20124,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -20260,7 +20260,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20668,7 +20668,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -20952,7 +20952,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -21094,7 +21094,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -21236,7 +21236,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -21366,7 +21366,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -21492,7 +21492,7 @@
         <v>46258</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -21616,7 +21616,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -21740,7 +21740,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -21864,7 +21864,7 @@
         <v>46248</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -21998,7 +21998,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -22132,7 +22132,7 @@
         <v>46230</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -22573,7 +22573,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -22825,7 +22825,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -22951,7 +22951,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -23077,7 +23077,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -23203,7 +23203,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -23325,7 +23325,7 @@
         <v>46258</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -23569,7 +23569,7 @@
         <v>46258</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -23687,7 +23687,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -23811,7 +23811,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -23935,7 +23935,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -24055,7 +24055,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -24175,7 +24175,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -24295,7 +24295,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -24413,7 +24413,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -24535,7 +24535,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -24649,7 +24649,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24889,7 +24889,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -25015,7 +25015,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -25137,7 +25137,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -25263,7 +25263,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -25389,7 +25389,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -25507,7 +25507,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -25629,7 +25629,7 @@
         <v>46241</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -25751,7 +25751,7 @@
         <v>46241</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -25873,7 +25873,7 @@
         <v>46243</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -25999,7 +25999,7 @@
         <v>46243</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -26121,7 +26121,7 @@
         <v>46249</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -26239,7 +26239,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -26357,7 +26357,7 @@
         <v>46249</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -26479,7 +26479,7 @@
         <v>46236</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -26605,7 +26605,7 @@
         <v>46236</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -26731,7 +26731,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -26857,7 +26857,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         <v>46238</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -27109,7 +27109,7 @@
         <v>46238</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -27227,7 +27227,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -27345,7 +27345,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -27465,7 +27465,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -27587,7 +27587,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -27709,7 +27709,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -28079,7 +28079,7 @@
         <v>46254</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -28201,7 +28201,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -28441,7 +28441,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28563,7 +28563,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -28677,7 +28677,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -28799,7 +28799,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -28921,7 +28921,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46249</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -29165,7 +29165,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -29287,7 +29287,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -29409,7 +29409,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -29653,7 +29653,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -29775,7 +29775,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -29893,7 +29893,7 @@
         <v>46250</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -30011,7 +30011,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -30133,7 +30133,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -30255,7 +30255,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30373,7 +30373,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -30844,7 +30844,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -30970,7 +30970,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31088,7 +31088,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31216,7 +31216,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31340,7 +31340,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -31464,7 +31464,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -31732,7 +31732,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -32117,7 +32117,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32243,7 +32243,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32361,7 +32361,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32440,7 +32440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36959,8 +36959,57 @@
         </is>
       </c>
     </row>
+    <row r="92" ht="54" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28T00:16:08+08:00</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21 至 2026-08-28</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>245</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H92" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I92" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/chongzuo/xxgk_15621/swjcgg/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /chongzuo/xxgk_15621/swjcgg/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('Rem...</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M91"/>
+  <autoFilter ref="A1:M92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-29
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         <v>46254</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>46258</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
         <v>46254</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
         <v>46258</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>46254</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2981,7 +2981,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3221,7 +3221,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v>46249</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>46254</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         <v>46246</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>46246</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>46249</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -3987,7 +3987,7 @@
         <v>46249</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4105,7 +4105,7 @@
         <v>46249</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>46242</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
         <v>46242</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>46250</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         <v>46250</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4789,7 +4789,7 @@
         <v>46257</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4925,7 +4925,7 @@
         <v>46257</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         <v>46241</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         <v>46241</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         <v>46240</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         <v>46243</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5555,7 +5555,7 @@
         <v>46243</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5677,7 +5677,7 @@
         <v>46249</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
         <v>46238</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         <v>46249</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
         <v>46249</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6167,7 +6167,7 @@
         <v>46236</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>46236</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>46238</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
         <v>46238</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6675,7 +6675,7 @@
         <v>46238</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>46233</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         <v>46234</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -7189,7 +7189,7 @@
         <v>46238</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7325,7 +7325,7 @@
         <v>46238</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>46229</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>46240</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
         <v>46240</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7847,7 +7847,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
         <v>46254</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
         <v>46229</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         <v>46229</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8743,7 +8743,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
         <v>46258</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -8999,7 +8999,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -9121,7 +9121,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9393,7 +9393,7 @@
         <v>46249</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9533,7 +9533,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         <v>46229</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9781,7 +9781,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9899,7 +9899,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -10143,7 +10143,7 @@
         <v>46254</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10257,7 +10257,7 @@
         <v>46254</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10379,7 +10379,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
         <v>46229</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10757,7 +10757,7 @@
         <v>46249</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10883,7 +10883,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -11005,7 +11005,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11131,7 +11131,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11265,7 +11265,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11395,7 +11395,7 @@
         <v>46249</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         <v>46258</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11645,7 +11645,7 @@
         <v>46254</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -11775,7 +11775,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         <v>46254</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12281,7 +12281,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12403,7 +12403,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12521,7 +12521,7 @@
         <v>46250</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12639,7 +12639,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         <v>46229</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12903,7 +12903,7 @@
         <v>46254</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13025,7 +13025,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         <v>46229</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>46229</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13407,7 +13407,7 @@
         <v>46254</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13541,7 +13541,7 @@
         <v>46258</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -13683,7 +13683,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13825,7 +13825,7 @@
         <v>46229</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13967,7 +13967,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -14109,7 +14109,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14251,7 +14251,7 @@
         <v>46254</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -14507,7 +14507,7 @@
         <v>46258</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14631,7 +14631,7 @@
         <v>46229</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14755,7 +14755,7 @@
         <v>46229</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14879,7 @@
         <v>46248</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         <v>46230</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -15147,7 +15147,7 @@
         <v>46230</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15690,7 +15690,7 @@
         <v>46254</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -15822,7 +15822,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -15952,7 +15952,7 @@
         <v>46246</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -16088,7 +16088,7 @@
         <v>46242</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -16234,7 +16234,7 @@
         <v>46242</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -16368,7 +16368,7 @@
         <v>46250</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>46250</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -16640,7 +16640,7 @@
         <v>46257</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -16776,7 +16776,7 @@
         <v>46257</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -16910,7 +16910,7 @@
         <v>46240</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -17044,7 +17044,7 @@
         <v>46238</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -17172,7 +17172,7 @@
         <v>46238</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -17302,7 +17302,7 @@
         <v>46233</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -17438,7 +17438,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>46238</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -17714,7 +17714,7 @@
         <v>46240</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -17856,7 +17856,7 @@
         <v>46240</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -17996,7 +17996,7 @@
         <v>46229</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -18130,7 +18130,7 @@
         <v>46229</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>46258</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         <v>46258</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -18530,7 +18530,7 @@
         <v>46229</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -18668,7 +18668,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -18808,7 +18808,7 @@
         <v>46254</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -18938,7 +18938,7 @@
         <v>46229</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -19072,7 +19072,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -19336,7 +19336,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -19466,7 +19466,7 @@
         <v>46249</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -19588,7 +19588,7 @@
         <v>46258</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -19716,7 +19716,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -19846,7 +19846,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -19984,7 +19984,7 @@
         <v>46254</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -20124,7 +20124,7 @@
         <v>46229</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -20260,7 +20260,7 @@
         <v>46229</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
         <v>46229</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20668,7 +20668,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -20952,7 +20952,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -21094,7 +21094,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -21236,7 +21236,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -21366,7 +21366,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -21492,7 +21492,7 @@
         <v>46258</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -21616,7 +21616,7 @@
         <v>46229</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -21740,7 +21740,7 @@
         <v>46229</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -21864,7 +21864,7 @@
         <v>46248</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -21998,7 +21998,7 @@
         <v>46230</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -22132,7 +22132,7 @@
         <v>46230</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -22573,7 +22573,7 @@
         <v>46258</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22699,7 +22699,7 @@
         <v>46254</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -22825,7 +22825,7 @@
         <v>46254</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -22951,7 +22951,7 @@
         <v>46254</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -23077,7 +23077,7 @@
         <v>46254</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -23203,7 +23203,7 @@
         <v>46254</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -23325,7 +23325,7 @@
         <v>46258</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -23447,7 +23447,7 @@
         <v>46254</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -23569,7 +23569,7 @@
         <v>46258</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -23687,7 +23687,7 @@
         <v>46254</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -23811,7 +23811,7 @@
         <v>46254</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -23935,7 +23935,7 @@
         <v>46254</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -24055,7 +24055,7 @@
         <v>46254</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -24175,7 +24175,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -24295,7 +24295,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -24413,7 +24413,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -24535,7 +24535,7 @@
         <v>46249</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -24649,7 +24649,7 @@
         <v>46249</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         <v>46249</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24889,7 +24889,7 @@
         <v>46249</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -25015,7 +25015,7 @@
         <v>46249</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -25137,7 +25137,7 @@
         <v>46246</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -25263,7 +25263,7 @@
         <v>46249</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -25389,7 +25389,7 @@
         <v>46249</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -25507,7 +25507,7 @@
         <v>46249</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -25629,7 +25629,7 @@
         <v>46241</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -25751,7 +25751,7 @@
         <v>46241</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -25873,7 +25873,7 @@
         <v>46243</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -25999,7 +25999,7 @@
         <v>46243</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -26121,7 +26121,7 @@
         <v>46249</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -26239,7 +26239,7 @@
         <v>46249</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -26357,7 +26357,7 @@
         <v>46249</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -26479,7 +26479,7 @@
         <v>46236</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -26605,7 +26605,7 @@
         <v>46236</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -26731,7 +26731,7 @@
         <v>46238</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -26857,7 +26857,7 @@
         <v>46238</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         <v>46238</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -27109,7 +27109,7 @@
         <v>46238</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -27227,7 +27227,7 @@
         <v>46229</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -27345,7 +27345,7 @@
         <v>46229</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -27465,7 +27465,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -27587,7 +27587,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -27709,7 +27709,7 @@
         <v>46229</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         <v>46229</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -28079,7 +28079,7 @@
         <v>46254</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -28201,7 +28201,7 @@
         <v>46229</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -28319,7 +28319,7 @@
         <v>46229</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -28441,7 +28441,7 @@
         <v>46229</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28563,7 +28563,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -28677,7 +28677,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -28799,7 +28799,7 @@
         <v>46254</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -28921,7 +28921,7 @@
         <v>46229</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46249</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -29165,7 +29165,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -29287,7 +29287,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -29409,7 +29409,7 @@
         <v>46229</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -29531,7 +29531,7 @@
         <v>46229</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -29653,7 +29653,7 @@
         <v>46229</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -29775,7 +29775,7 @@
         <v>46229</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -29893,7 +29893,7 @@
         <v>46250</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -30011,7 +30011,7 @@
         <v>46229</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -30133,7 +30133,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -30255,7 +30255,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30373,7 +30373,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -30844,7 +30844,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -30970,7 +30970,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31088,7 +31088,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31216,7 +31216,7 @@
         <v>46229</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31340,7 +31340,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -31464,7 +31464,7 @@
         <v>46248</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>46230</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -31732,7 +31732,7 @@
         <v>46230</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -32117,7 +32117,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32243,7 +32243,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32361,7 +32361,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32440,7 +32440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -37008,8 +37008,57 @@
         </is>
       </c>
     </row>
+    <row r="93" ht="54" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:34:06+08:00</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22 至 2026-08-29</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>262</v>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I93" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/chongzuo/xxgk_15621/swjcgg/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /chongzuo/xxgk_15621/swjcgg/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('Rem...</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>本次检索未发现符合收录标准的新文书。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M92"/>
+  <autoFilter ref="A1:M93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-30
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -8211,7 +8211,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -12883,7 +12883,7 @@
         <v>46229</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13651,7 +13651,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13785,7 +13785,7 @@
         <v>46258</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
         <v>46254</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -20774,7 +20774,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20916,7 +20916,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -30503,7 +30503,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30865,7 +30865,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -31584,7 +31584,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32857,7 +32857,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32936,7 +32936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M98"/>
+  <dimension ref="A1:M99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -37794,8 +37794,57 @@
         </is>
       </c>
     </row>
+    <row r="99" ht="54" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-30T17:54:23+08:00</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 至 2026-08-30</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>262</v>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G99" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H99" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I99" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J99" s="2" t="inlineStr"/>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/hechi/tzgg_15562/tzgg_15563/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /hechi/tzgg_15562/tzgg_15563/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected('R...</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问20页，访问失败254页，持久化待复核239个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M98"/>
+  <autoFilter ref="A1:M99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-08-31
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46264</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46264</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -8211,7 +8211,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -12883,7 +12883,7 @@
         <v>46229</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13651,7 +13651,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13785,7 +13785,7 @@
         <v>46258</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
         <v>46254</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -20774,7 +20774,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20916,7 +20916,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -22821,7 +22821,7 @@
         <v>46264</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22943,7 +22943,7 @@
         <v>46264</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -30503,7 +30503,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30865,7 +30865,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -31584,7 +31584,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32857,7 +32857,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32936,7 +32936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M100"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -37892,8 +37892,57 @@
         </is>
       </c>
     </row>
+    <row r="101" ht="54" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31T18:47:34+08:00</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 至 2026-08-31</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="n">
+        <v>279</v>
+      </c>
+      <c r="D101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H101" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I101" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J101" s="2" t="inlineStr"/>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问19页，访问失败260页，持久化待复核245个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M100"/>
+  <autoFilter ref="A1:M101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-01
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46264</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46264</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -8211,7 +8211,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -12883,7 +12883,7 @@
         <v>46229</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13651,7 +13651,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13785,7 +13785,7 @@
         <v>46258</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
         <v>46254</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -20774,7 +20774,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20916,7 +20916,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -22821,7 +22821,7 @@
         <v>46264</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22943,7 +22943,7 @@
         <v>46264</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -30503,7 +30503,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30865,7 +30865,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -31584,7 +31584,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32857,7 +32857,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32936,7 +32936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M102"/>
+  <dimension ref="A1:M103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -37990,8 +37990,57 @@
         </is>
       </c>
     </row>
+    <row r="103" ht="54" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01T17:21:50+08:00</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 至 2026-09-01</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="n">
+        <v>277</v>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G103" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H103" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I103" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J103" s="2" t="inlineStr"/>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问25页，访问失败263页，持久化待复核248个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M102"/>
+  <autoFilter ref="A1:M103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-02
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46264</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46264</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -8211,7 +8211,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -12883,7 +12883,7 @@
         <v>46229</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -13651,7 +13651,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13785,7 +13785,7 @@
         <v>46258</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
         <v>46254</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -20774,7 +20774,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -20916,7 +20916,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -22821,7 +22821,7 @@
         <v>46264</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -22943,7 +22943,7 @@
         <v>46264</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27957,7 +27957,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -30503,7 +30503,7 @@
         <v>46229</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -30865,7 +30865,7 @@
         <v>46254</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -31584,7 +31584,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32857,7 +32857,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32936,7 +32936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M104"/>
+  <dimension ref="A1:M105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -38088,8 +38088,57 @@
         </is>
       </c>
     </row>
+    <row r="105" ht="54" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02T16:44:17+08:00</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 至 2026-09-02</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="n">
+        <v>279</v>
+      </c>
+      <c r="D105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G105" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H105" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I105" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J105" s="2" t="inlineStr"/>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://guangxi.chinatax.gov.cn/beihai/tzgg_15227/tzgg_15228/: ConnectionError: HTTPSConnectionPool(host='guangxi.chinatax.gov.cn', port=443): Max retries exceeded with url: /beihai/tzgg_15227/tzgg_15228/ (Caused by ProtocolError('Connection aborted.', RemoteDisconnected(...</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问16页，访问失败268页，持久化待复核253个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M104"/>
+  <autoFilter ref="A1:M105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-03
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -821,7 +821,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1489,12 +1489,12 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr"/>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="AJ8" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1611,12 +1611,12 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr"/>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="AJ10" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="AJ11" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -2107,12 +2107,12 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -2229,12 +2229,12 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr"/>
@@ -2293,7 +2293,7 @@
       </c>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -24109,7 +24109,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -24231,7 +24231,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -24533,12 +24533,12 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr"/>
@@ -24597,7 +24597,7 @@
       </c>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -24655,12 +24655,12 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr"/>
@@ -24719,7 +24719,7 @@
       </c>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -24777,12 +24777,12 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr"/>
@@ -24841,7 +24841,7 @@
       </c>
       <c r="AJ8" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -24899,12 +24899,12 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr"/>
@@ -24963,7 +24963,7 @@
       </c>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -25089,7 +25089,7 @@
       </c>
       <c r="AJ10" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -25215,7 +25215,7 @@
       </c>
       <c r="AJ11" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -25395,12 +25395,12 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr"/>
@@ -25459,7 +25459,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -25517,12 +25517,12 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽处〔2026〕14号</t>
+          <t>河市税二稽处〔2026〕17号</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>河市税二稽罚〔2026〕7号</t>
+          <t>河市税二稽罚〔2026〕10号</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr"/>
@@ -25581,7 +25581,7 @@
       </c>
       <c r="AJ14" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -35432,7 +35432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M107"/>
+  <dimension ref="A1:M108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40735,8 +40735,57 @@
         </is>
       </c>
     </row>
+    <row r="108" ht="54" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03T17:26:09+08:00</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 至 2026-09-03</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="n">
+        <v>293</v>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问50页，访问失败242页，持久化待复核233个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M107"/>
+  <autoFilter ref="A1:M108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-04
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46268</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46268</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2505,7 +2505,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -5075,7 +5075,7 @@
         <v>46246</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -8413,7 +8413,7 @@
         <v>46234</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8535,7 +8535,7 @@
         <v>46238</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8661,7 +8661,7 @@
         <v>46238</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -9439,7 +9439,7 @@
         <v>46254</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -14111,7 +14111,7 @@
         <v>46229</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14879,7 @@
         <v>46254</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         <v>46258</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15155,7 +15155,7 @@
         <v>46254</v>
       </c>
       <c r="AA116" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB116" s="2" t="inlineStr">
         <is>
@@ -18934,7 +18934,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -22022,7 +22022,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -22164,7 +22164,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -24069,7 +24069,7 @@
         <v>46268</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -24191,7 +24191,7 @@
         <v>46268</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -25667,7 +25667,7 @@
         <v>46254</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -25793,7 +25793,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -28105,7 +28105,7 @@
         <v>46246</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -29951,7 +29951,7 @@
         <v>46238</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -30077,7 +30077,7 @@
         <v>46238</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -30433,7 +30433,7 @@
         <v>46254</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -32979,7 +32979,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -33341,7 +33341,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -33836,7 +33836,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -33962,7 +33962,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -34080,7 +34080,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35109,7 +35109,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -35235,7 +35235,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35353,7 +35353,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35432,7 +35432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M108"/>
+  <dimension ref="A1:M109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40784,8 +40784,57 @@
         </is>
       </c>
     </row>
+    <row r="109" ht="54" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04T16:48:28+08:00</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28 至 2026-09-04</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G109" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H109" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I109" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J109" s="2" t="inlineStr"/>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问52页，访问失败242页，持久化待复核233个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M108"/>
+  <autoFilter ref="A1:M109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-05
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46269</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -5197,7 +5197,7 @@
         <v>46246</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -8535,7 +8535,7 @@
         <v>46234</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
         <v>46238</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8783,7 +8783,7 @@
         <v>46238</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9561,7 +9561,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -15135,7 +15135,7 @@
         <v>46258</v>
       </c>
       <c r="AA116" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB116" s="2" t="inlineStr">
         <is>
@@ -15277,7 +15277,7 @@
         <v>46254</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -19058,7 +19058,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -22146,7 +22146,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -22288,7 +22288,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -24193,7 +24193,7 @@
         <v>46269</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -24233,7 +24233,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -25913,7 +25913,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -26039,7 +26039,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -28351,7 +28351,7 @@
         <v>46246</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -30197,7 +30197,7 @@
         <v>46238</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -30323,7 +30323,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -30679,7 +30679,7 @@
         <v>46254</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -34084,7 +34084,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -34210,7 +34210,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35357,7 +35357,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -35483,7 +35483,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35680,7 +35680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M110"/>
+  <dimension ref="A1:M111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41134,8 +41134,57 @@
         </is>
       </c>
     </row>
+    <row r="111" ht="54" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05T16:18:59+08:00</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-29 至 2026-09-05</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="n">
+        <v>301</v>
+      </c>
+      <c r="D111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G111" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I111" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J111" s="2" t="inlineStr"/>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/smsswj/xxgk/sjxxgk/qtgg/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /smsswj/xxgk/sjxxgk/qtgg/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', p...</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问48页，访问失败249页，持久化待复核240个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M110"/>
+  <autoFilter ref="A1:M111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-06
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46269</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -5197,7 +5197,7 @@
         <v>46246</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -8535,7 +8535,7 @@
         <v>46234</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
         <v>46238</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8783,7 +8783,7 @@
         <v>46238</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9561,7 +9561,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -13875,7 +13875,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -13997,7 +13997,7 @@
         <v>46229</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -14233,7 +14233,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -15001,7 +15001,7 @@
         <v>46254</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15135,7 +15135,7 @@
         <v>46258</v>
       </c>
       <c r="AA116" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB116" s="2" t="inlineStr">
         <is>
@@ -15277,7 +15277,7 @@
         <v>46254</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -19058,7 +19058,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -22146,7 +22146,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -22288,7 +22288,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -24193,7 +24193,7 @@
         <v>46269</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -25913,7 +25913,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -26039,7 +26039,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -28351,7 +28351,7 @@
         <v>46246</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -30197,7 +30197,7 @@
         <v>46238</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -30323,7 +30323,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -30679,7 +30679,7 @@
         <v>46254</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -32867,7 +32867,7 @@
         <v>46229</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -32989,7 +32989,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -33225,7 +33225,7 @@
         <v>46229</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -33587,7 +33587,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -34084,7 +34084,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -34210,7 +34210,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -34328,7 +34328,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35357,7 +35357,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -35483,7 +35483,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35601,7 +35601,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35680,7 +35680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M112"/>
+  <dimension ref="A1:M113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41232,8 +41232,57 @@
         </is>
       </c>
     </row>
+    <row r="113" ht="54" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06T16:37:32+08:00</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-30 至 2026-09-06</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="n">
+        <v>311</v>
+      </c>
+      <c r="D113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="G113" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I113" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J113" s="2" t="inlineStr"/>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问55页，访问失败253页，持久化待复核244个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M112"/>
+  <autoFilter ref="A1:M113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-07
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46269</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -5197,7 +5197,7 @@
         <v>46246</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -8535,7 +8535,7 @@
         <v>46234</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
         <v>46238</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8783,7 +8783,7 @@
         <v>46238</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -9561,7 +9561,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -14233,7 +14233,7 @@
         <v>46229</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -15001,7 +15001,7 @@
         <v>46254</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -15135,7 +15135,7 @@
         <v>46258</v>
       </c>
       <c r="AA116" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB116" s="2" t="inlineStr">
         <is>
@@ -15277,7 +15277,7 @@
         <v>46254</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -19058,7 +19058,7 @@
         <v>46234</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -22146,7 +22146,7 @@
         <v>46258</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -22288,7 +22288,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -24193,7 +24193,7 @@
         <v>46269</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -25913,7 +25913,7 @@
         <v>46254</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -26039,7 +26039,7 @@
         <v>46254</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -28351,7 +28351,7 @@
         <v>46246</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -30197,7 +30197,7 @@
         <v>46238</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -30323,7 +30323,7 @@
         <v>46238</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -30679,7 +30679,7 @@
         <v>46254</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -33225,7 +33225,7 @@
         <v>46229</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -33587,7 +33587,7 @@
         <v>46254</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -34084,7 +34084,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -34210,7 +34210,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -34328,7 +34328,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35357,7 +35357,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -35483,7 +35483,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35601,7 +35601,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35680,7 +35680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M114"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41330,8 +41330,57 @@
         </is>
       </c>
     </row>
+    <row r="115" ht="54" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T17:16:37+08:00</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31 至 2026-09-07</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v>313</v>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G115" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I115" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J115" s="2" t="inlineStr"/>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问52页，访问失败254页，持久化待复核248个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M114"/>
+  <autoFilter ref="A1:M115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-10
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46273</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46273</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46269</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
         <v>46273</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         <v>46274</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1673,7 +1673,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4083,7 +4087,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4209,7 +4213,7 @@
         <v>46254</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -6905,7 +6909,7 @@
         <v>46246</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -10243,7 +10247,7 @@
         <v>46234</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -10365,7 +10369,7 @@
         <v>46238</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10495,7 @@
         <v>46238</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -11269,7 +11273,7 @@
         <v>46254</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11785,7 +11789,7 @@
         <v>46229</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -11911,7 +11915,7 @@
         <v>46229</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -15941,7 +15945,7 @@
         <v>46229</v>
       </c>
       <c r="AA123" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB123" s="2" t="inlineStr">
         <is>
@@ -16709,7 +16713,7 @@
         <v>46254</v>
       </c>
       <c r="AA129" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB129" s="2" t="inlineStr">
         <is>
@@ -16843,7 +16847,7 @@
         <v>46258</v>
       </c>
       <c r="AA130" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB130" s="2" t="inlineStr">
         <is>
@@ -16985,7 +16989,7 @@
         <v>46254</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -17927,7 +17931,7 @@
         <v>46258</v>
       </c>
       <c r="AA138" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB138" s="2" t="inlineStr">
         <is>
@@ -21281,7 +21285,7 @@
         <v>46234</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -24369,7 +24373,7 @@
         <v>46258</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -24511,7 +24515,7 @@
         <v>46254</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -25335,7 +25339,7 @@
         <v>46258</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -26423,7 +26427,7 @@
         <v>46273</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -26549,7 +26553,7 @@
         <v>46273</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -26671,7 +26675,7 @@
         <v>46269</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -26793,7 +26797,7 @@
         <v>46273</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -27151,7 +27155,7 @@
         <v>46274</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -27185,7 +27189,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -29343,7 +29351,7 @@
         <v>46254</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -29469,7 +29477,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -31907,7 +31915,7 @@
         <v>46246</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -33753,7 +33761,7 @@
         <v>46238</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -33879,7 +33887,7 @@
         <v>46238</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -34235,7 +34243,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -34479,7 +34487,7 @@
         <v>46229</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -34605,7 +34613,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -36781,7 +36789,7 @@
         <v>46229</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -37143,7 +37151,7 @@
         <v>46254</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -37774,7 +37782,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -37900,7 +37908,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -38018,7 +38026,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -39047,7 +39055,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -39173,7 +39181,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -39291,7 +39299,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -39370,7 +39378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M120"/>
+  <dimension ref="A1:M121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -45330,8 +45338,57 @@
         </is>
       </c>
     </row>
+    <row r="121" ht="54" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T16:54:54+08:00</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03 至 2026-09-10</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G121" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H121" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I121" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J121" s="2" t="inlineStr"/>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问72页，访问失败204页，持久化待复核198个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M120"/>
+  <autoFilter ref="A1:M121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-11
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -819,7 +819,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -903,7 +907,7 @@
         <v>46273</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1033,7 @@
         <v>46273</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1155,7 @@
         <v>46269</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1425,7 +1429,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1541,7 +1549,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4435,7 +4447,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4561,7 +4573,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -7257,7 +7269,7 @@
         <v>46246</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -10595,7 +10607,7 @@
         <v>46234</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10717,7 +10729,7 @@
         <v>46238</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -10843,7 +10855,7 @@
         <v>46238</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11621,7 +11633,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -12137,7 +12149,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12263,7 +12275,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -17195,7 +17207,7 @@
         <v>46258</v>
       </c>
       <c r="AA133" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB133" s="2" t="inlineStr">
         <is>
@@ -17337,7 +17349,7 @@
         <v>46254</v>
       </c>
       <c r="AA134" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB134" s="2" t="inlineStr">
         <is>
@@ -18279,7 +18291,7 @@
         <v>46258</v>
       </c>
       <c r="AA141" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB141" s="2" t="inlineStr">
         <is>
@@ -19542,7 +19554,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -19658,7 +19674,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -21870,7 +21890,7 @@
         <v>46234</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24958,7 +24978,7 @@
         <v>46258</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25100,7 +25120,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -25924,7 +25944,7 @@
         <v>46258</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -27014,7 +27034,7 @@
         <v>46273</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -27140,7 +27160,7 @@
         <v>46273</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27262,7 +27282,7 @@
         <v>46269</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -27536,7 +27556,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -30052,7 +30076,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -30178,7 +30202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -32616,7 +32640,7 @@
         <v>46246</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -34462,7 +34486,7 @@
         <v>46238</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -34588,7 +34612,7 @@
         <v>46238</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -34944,7 +34968,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -35188,7 +35212,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -35314,7 +35338,7 @@
         <v>46229</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -38484,7 +38508,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -38610,7 +38634,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -39757,7 +39781,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -39883,7 +39907,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -40080,7 +40104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M122"/>
+  <dimension ref="A1:M123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -46142,8 +46166,57 @@
         </is>
       </c>
     </row>
+    <row r="123" ht="54" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T16:52:45+08:00</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04 至 2026-09-11</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="n">
+        <v>295</v>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G123" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H123" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I123" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问73页，访问失败213页，持久化待复核207个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M122"/>
+  <autoFilter ref="A1:M123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-12
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -907,7 +907,7 @@
         <v>46273</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46273</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -7269,7 +7269,7 @@
         <v>46246</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -10607,7 +10607,7 @@
         <v>46234</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -10729,7 +10729,7 @@
         <v>46238</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -10855,7 +10855,7 @@
         <v>46238</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -11633,7 +11633,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -12149,7 +12149,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12275,7 +12275,7 @@
         <v>46229</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -16305,7 +16305,7 @@
         <v>46229</v>
       </c>
       <c r="AA126" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB126" s="2" t="inlineStr">
         <is>
@@ -17073,7 +17073,7 @@
         <v>46254</v>
       </c>
       <c r="AA132" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB132" s="2" t="inlineStr">
         <is>
@@ -17207,7 +17207,7 @@
         <v>46258</v>
       </c>
       <c r="AA133" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB133" s="2" t="inlineStr">
         <is>
@@ -17349,7 +17349,7 @@
         <v>46254</v>
       </c>
       <c r="AA134" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB134" s="2" t="inlineStr">
         <is>
@@ -18291,7 +18291,7 @@
         <v>46258</v>
       </c>
       <c r="AA141" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB141" s="2" t="inlineStr">
         <is>
@@ -21890,7 +21890,7 @@
         <v>46234</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -24978,7 +24978,7 @@
         <v>46258</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25120,7 +25120,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -25944,7 +25944,7 @@
         <v>46258</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -27034,7 +27034,7 @@
         <v>46273</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -27160,7 +27160,7 @@
         <v>46273</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -30076,7 +30076,7 @@
         <v>46254</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -30202,7 +30202,7 @@
         <v>46254</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -32640,7 +32640,7 @@
         <v>46246</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -34486,7 +34486,7 @@
         <v>46238</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -34612,7 +34612,7 @@
         <v>46238</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -34968,7 +34968,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -35212,7 +35212,7 @@
         <v>46229</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -35338,7 +35338,7 @@
         <v>46229</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -37514,7 +37514,7 @@
         <v>46229</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -37876,7 +37876,7 @@
         <v>46254</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -38508,7 +38508,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -38634,7 +38634,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -38752,7 +38752,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -39781,7 +39781,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -39907,7 +39907,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -40025,7 +40025,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -40104,7 +40104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M124"/>
+  <dimension ref="A1:M125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -46264,8 +46264,57 @@
         </is>
       </c>
     </row>
+    <row r="125" ht="54" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:36:22+08:00</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05 至 2026-09-12</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="n">
+        <v>297</v>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="G125" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H125" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I125" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J125" s="2" t="inlineStr"/>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='...</t>
+        </is>
+      </c>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问78页，访问失败210页，持久化待复核203个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M124"/>
+  <autoFilter ref="A1:M125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>